<commit_message>
🤖 自動盤後數據、Direct Buy、Swing BuyNow與績效稽核: 2026-08-19 06:24:18
</commit_message>
<xml_diff>
--- a/data/swing_performance_analysis.xlsx
+++ b/data/swing_performance_analysis.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'T20_Tracking'!$A$1:$AJ$145</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'T20_Tracking'!$A$1:$AJ$152</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ145"/>
+  <dimension ref="A1:AJ152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -731,7 +731,7 @@
         </is>
       </c>
       <c r="Z2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA2" t="n">
         <v>-1.45</v>
@@ -800,7 +800,7 @@
         </is>
       </c>
       <c r="Z3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA3" t="n">
         <v>-5.5</v>
@@ -809,7 +809,7 @@
         <v>0</v>
       </c>
       <c r="AH3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI3" t="inlineStr">
         <is>
@@ -869,7 +869,7 @@
         </is>
       </c>
       <c r="Z4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA4" t="n">
         <v>21.91</v>
@@ -938,7 +938,7 @@
         </is>
       </c>
       <c r="Z5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA5" t="n">
         <v>3.92</v>
@@ -1007,7 +1007,7 @@
         </is>
       </c>
       <c r="Z6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA6" t="n">
         <v>7.73</v>
@@ -1076,7 +1076,7 @@
         </is>
       </c>
       <c r="Z7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA7" t="n">
         <v>5.54</v>
@@ -1145,7 +1145,7 @@
         </is>
       </c>
       <c r="Z8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA8" t="n">
         <v>-11.56</v>
@@ -1214,7 +1214,7 @@
         </is>
       </c>
       <c r="Z9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA9" t="n">
         <v>-10.14</v>
@@ -1283,7 +1283,7 @@
         </is>
       </c>
       <c r="Z10" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA10" t="n">
         <v>-12.27</v>
@@ -1352,7 +1352,7 @@
         </is>
       </c>
       <c r="Z11" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA11" t="n">
         <v>-6.97</v>
@@ -1421,7 +1421,7 @@
         </is>
       </c>
       <c r="Z12" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA12" t="n">
         <v>5.13</v>
@@ -1490,7 +1490,7 @@
         </is>
       </c>
       <c r="Z13" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA13" t="n">
         <v>-5.54</v>
@@ -1621,7 +1621,7 @@
         </is>
       </c>
       <c r="Z15" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA15" t="n">
         <v>3.09</v>
@@ -1690,7 +1690,7 @@
         </is>
       </c>
       <c r="Z16" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA16" t="n">
         <v>9.31</v>
@@ -1759,7 +1759,7 @@
         </is>
       </c>
       <c r="Z17" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA17" t="n">
         <v>-1.43</v>
@@ -1828,7 +1828,7 @@
         </is>
       </c>
       <c r="Z18" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA18" t="n">
         <v>-6.69</v>
@@ -1897,7 +1897,7 @@
         </is>
       </c>
       <c r="Z19" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA19" t="n">
         <v>-4.07</v>
@@ -1966,7 +1966,7 @@
         </is>
       </c>
       <c r="Z20" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA20" t="n">
         <v>-1.42</v>
@@ -1975,7 +1975,7 @@
         <v>0</v>
       </c>
       <c r="AH20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI20" t="inlineStr">
         <is>
@@ -2035,7 +2035,7 @@
         </is>
       </c>
       <c r="Z21" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA21" t="n">
         <v>-3.59</v>
@@ -2044,7 +2044,7 @@
         <v>0</v>
       </c>
       <c r="AH21" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI21" t="inlineStr">
         <is>
@@ -2104,7 +2104,7 @@
         </is>
       </c>
       <c r="Z22" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA22" t="n">
         <v>14.67</v>
@@ -2173,7 +2173,7 @@
         </is>
       </c>
       <c r="Z23" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA23" t="n">
         <v>2.43</v>
@@ -2242,7 +2242,7 @@
         </is>
       </c>
       <c r="Z24" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA24" t="n">
         <v>1.05</v>
@@ -2311,7 +2311,7 @@
         </is>
       </c>
       <c r="Z25" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA25" t="n">
         <v>8.18</v>
@@ -2380,13 +2380,13 @@
         </is>
       </c>
       <c r="Z26" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA26" t="n">
         <v>6.01</v>
       </c>
       <c r="AG26" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH26" t="b">
         <v>0</v>
@@ -2449,7 +2449,7 @@
         </is>
       </c>
       <c r="Z27" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA27" t="n">
         <v>13.83</v>
@@ -2518,7 +2518,7 @@
         </is>
       </c>
       <c r="Z28" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA28" t="n">
         <v>-10.91</v>
@@ -2587,7 +2587,7 @@
         </is>
       </c>
       <c r="Z29" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA29" t="n">
         <v>-2.87</v>
@@ -2656,7 +2656,7 @@
         </is>
       </c>
       <c r="Z30" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA30" t="n">
         <v>-8.630000000000001</v>
@@ -2725,7 +2725,7 @@
         </is>
       </c>
       <c r="Z31" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA31" t="n">
         <v>-0.91</v>
@@ -2794,7 +2794,7 @@
         </is>
       </c>
       <c r="Z32" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA32" t="n">
         <v>-6.43</v>
@@ -2863,7 +2863,7 @@
         </is>
       </c>
       <c r="Z33" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA33" t="n">
         <v>-3.11</v>
@@ -3056,7 +3056,7 @@
         </is>
       </c>
       <c r="Z36" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA36" t="n">
         <v>-3.48</v>
@@ -3065,7 +3065,7 @@
         <v>0</v>
       </c>
       <c r="AH36" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI36" t="inlineStr">
         <is>
@@ -3125,7 +3125,7 @@
         </is>
       </c>
       <c r="Z37" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA37" t="n">
         <v>10.15</v>
@@ -3194,7 +3194,7 @@
         </is>
       </c>
       <c r="Z38" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA38" t="n">
         <v>-5.23</v>
@@ -3263,7 +3263,7 @@
         </is>
       </c>
       <c r="Z39" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA39" t="n">
         <v>-5.13</v>
@@ -3332,7 +3332,7 @@
         </is>
       </c>
       <c r="Z40" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA40" t="n">
         <v>-3.13</v>
@@ -3401,7 +3401,7 @@
         </is>
       </c>
       <c r="Z41" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA41" t="n">
         <v>-4.05</v>
@@ -3470,7 +3470,7 @@
         </is>
       </c>
       <c r="Z42" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA42" t="n">
         <v>1.86</v>
@@ -3539,7 +3539,7 @@
         </is>
       </c>
       <c r="Z43" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA43" t="n">
         <v>8.460000000000001</v>
@@ -3608,7 +3608,7 @@
         </is>
       </c>
       <c r="Z44" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA44" t="n">
         <v>10.82</v>
@@ -3677,7 +3677,7 @@
         </is>
       </c>
       <c r="Z45" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA45" t="n">
         <v>-0.71</v>
@@ -3746,7 +3746,7 @@
         </is>
       </c>
       <c r="Z46" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA46" t="n">
         <v>12.1</v>
@@ -3815,7 +3815,7 @@
         </is>
       </c>
       <c r="Z47" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA47" t="n">
         <v>2.72</v>
@@ -3884,7 +3884,7 @@
         </is>
       </c>
       <c r="Z48" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA48" t="n">
         <v>5.32</v>
@@ -3953,7 +3953,7 @@
         </is>
       </c>
       <c r="Z49" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA49" t="n">
         <v>-3.36</v>
@@ -4022,7 +4022,7 @@
         </is>
       </c>
       <c r="Z50" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA50" t="n">
         <v>9.17</v>
@@ -4091,13 +4091,13 @@
         </is>
       </c>
       <c r="Z51" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA51" t="n">
         <v>8.08</v>
       </c>
       <c r="AG51" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH51" t="b">
         <v>0</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="Z52" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA52" t="n">
         <v>20.55</v>
@@ -4229,7 +4229,7 @@
         </is>
       </c>
       <c r="Z53" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA53" t="n">
         <v>-0.32</v>
@@ -4298,7 +4298,7 @@
         </is>
       </c>
       <c r="Z54" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA54" t="n">
         <v>-5.24</v>
@@ -4307,7 +4307,7 @@
         <v>0</v>
       </c>
       <c r="AH54" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI54" t="inlineStr">
         <is>
@@ -4429,7 +4429,7 @@
         </is>
       </c>
       <c r="Z56" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA56" t="n">
         <v>-4.49</v>
@@ -4498,7 +4498,10 @@
         </is>
       </c>
       <c r="Z57" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA57" t="n">
+        <v>-0.28</v>
       </c>
       <c r="AG57" t="b">
         <v>0</v>
@@ -4564,7 +4567,10 @@
         </is>
       </c>
       <c r="Z58" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA58" t="n">
+        <v>-8.779999999999999</v>
       </c>
       <c r="AG58" t="b">
         <v>0</v>
@@ -4630,7 +4636,10 @@
         </is>
       </c>
       <c r="Z59" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA59" t="n">
+        <v>-4.05</v>
       </c>
       <c r="AG59" t="b">
         <v>0</v>
@@ -4696,7 +4705,10 @@
         </is>
       </c>
       <c r="Z60" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA60" t="n">
+        <v>-9.26</v>
       </c>
       <c r="AG60" t="b">
         <v>0</v>
@@ -4762,7 +4774,10 @@
         </is>
       </c>
       <c r="Z61" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA61" t="n">
+        <v>8.57</v>
       </c>
       <c r="AG61" t="b">
         <v>1</v>
@@ -4828,7 +4843,10 @@
         </is>
       </c>
       <c r="Z62" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA62" t="n">
+        <v>-3.42</v>
       </c>
       <c r="AG62" t="b">
         <v>0</v>
@@ -4894,7 +4912,10 @@
         </is>
       </c>
       <c r="Z63" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA63" t="n">
+        <v>2.62</v>
       </c>
       <c r="AG63" t="b">
         <v>0</v>
@@ -4960,7 +4981,10 @@
         </is>
       </c>
       <c r="Z64" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA64" t="n">
+        <v>1.17</v>
       </c>
       <c r="AG64" t="b">
         <v>0</v>
@@ -5026,7 +5050,10 @@
         </is>
       </c>
       <c r="Z65" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA65" t="n">
+        <v>12.12</v>
       </c>
       <c r="AG65" t="b">
         <v>0</v>
@@ -5092,7 +5119,10 @@
         </is>
       </c>
       <c r="Z66" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA66" t="n">
+        <v>-1.13</v>
       </c>
       <c r="AG66" t="b">
         <v>0</v>
@@ -5158,10 +5188,13 @@
         </is>
       </c>
       <c r="Z67" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA67" t="n">
+        <v>21.05</v>
       </c>
       <c r="AG67" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH67" t="b">
         <v>0</v>
@@ -5224,7 +5257,10 @@
         </is>
       </c>
       <c r="Z68" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA68" t="n">
+        <v>6.36</v>
       </c>
       <c r="AG68" t="b">
         <v>0</v>
@@ -5290,7 +5326,10 @@
         </is>
       </c>
       <c r="Z69" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA69" t="n">
+        <v>-5.94</v>
       </c>
       <c r="AG69" t="b">
         <v>0</v>
@@ -5418,7 +5457,10 @@
         </is>
       </c>
       <c r="Z71" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA71" t="n">
+        <v>3.22</v>
       </c>
       <c r="AG71" t="b">
         <v>0</v>
@@ -5484,7 +5526,10 @@
         </is>
       </c>
       <c r="Z72" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA72" t="n">
+        <v>-2.78</v>
       </c>
       <c r="AG72" t="b">
         <v>0</v>
@@ -5550,7 +5595,10 @@
         </is>
       </c>
       <c r="Z73" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA73" t="n">
+        <v>5.81</v>
       </c>
       <c r="AG73" t="b">
         <v>0</v>
@@ -5616,7 +5664,10 @@
         </is>
       </c>
       <c r="Z74" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA74" t="n">
+        <v>-5.04</v>
       </c>
       <c r="AG74" t="b">
         <v>0</v>
@@ -5682,7 +5733,7 @@
         </is>
       </c>
       <c r="Z75" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG75" t="b">
         <v>0</v>
@@ -5748,7 +5799,7 @@
         </is>
       </c>
       <c r="Z76" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG76" t="b">
         <v>0</v>
@@ -5814,7 +5865,7 @@
         </is>
       </c>
       <c r="Z77" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG77" t="b">
         <v>0</v>
@@ -5880,7 +5931,7 @@
         </is>
       </c>
       <c r="Z78" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG78" t="b">
         <v>0</v>
@@ -5946,7 +5997,7 @@
         </is>
       </c>
       <c r="Z79" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG79" t="b">
         <v>0</v>
@@ -6012,7 +6063,7 @@
         </is>
       </c>
       <c r="Z80" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG80" t="b">
         <v>0</v>
@@ -6078,7 +6129,7 @@
         </is>
       </c>
       <c r="Z81" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG81" t="b">
         <v>0</v>
@@ -6144,7 +6195,7 @@
         </is>
       </c>
       <c r="Z82" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG82" t="b">
         <v>1</v>
@@ -6210,7 +6261,7 @@
         </is>
       </c>
       <c r="Z83" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG83" t="b">
         <v>0</v>
@@ -6276,10 +6327,10 @@
         </is>
       </c>
       <c r="Z84" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG84" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH84" t="b">
         <v>0</v>
@@ -6342,7 +6393,7 @@
         </is>
       </c>
       <c r="Z85" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG85" t="b">
         <v>0</v>
@@ -6408,7 +6459,7 @@
         </is>
       </c>
       <c r="Z86" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG86" t="b">
         <v>0</v>
@@ -6474,7 +6525,7 @@
         </is>
       </c>
       <c r="Z87" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG87" t="b">
         <v>0</v>
@@ -6540,7 +6591,7 @@
         </is>
       </c>
       <c r="Z88" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG88" t="b">
         <v>0</v>
@@ -6606,7 +6657,7 @@
         </is>
       </c>
       <c r="Z89" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG89" t="b">
         <v>0</v>
@@ -6734,7 +6785,7 @@
         </is>
       </c>
       <c r="Z91" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG91" t="b">
         <v>0</v>
@@ -6800,7 +6851,7 @@
         </is>
       </c>
       <c r="Z92" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG92" t="b">
         <v>0</v>
@@ -6866,7 +6917,7 @@
         </is>
       </c>
       <c r="Z93" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG93" t="b">
         <v>0</v>
@@ -6932,7 +6983,7 @@
         </is>
       </c>
       <c r="Z94" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG94" t="b">
         <v>0</v>
@@ -6998,7 +7049,7 @@
         </is>
       </c>
       <c r="Z95" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG95" t="b">
         <v>0</v>
@@ -7064,7 +7115,7 @@
         </is>
       </c>
       <c r="Z96" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG96" t="b">
         <v>0</v>
@@ -7130,7 +7181,7 @@
         </is>
       </c>
       <c r="Z97" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG97" t="b">
         <v>0</v>
@@ -7196,7 +7247,7 @@
         </is>
       </c>
       <c r="Z98" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG98" t="b">
         <v>0</v>
@@ -7262,7 +7313,7 @@
         </is>
       </c>
       <c r="Z99" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG99" t="b">
         <v>0</v>
@@ -7328,7 +7379,7 @@
         </is>
       </c>
       <c r="Z100" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG100" t="b">
         <v>0</v>
@@ -7394,7 +7445,7 @@
         </is>
       </c>
       <c r="Z101" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG101" t="b">
         <v>1</v>
@@ -7460,7 +7511,7 @@
         </is>
       </c>
       <c r="Z102" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG102" t="b">
         <v>1</v>
@@ -7526,7 +7577,7 @@
         </is>
       </c>
       <c r="Z103" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG103" t="b">
         <v>0</v>
@@ -7592,7 +7643,7 @@
         </is>
       </c>
       <c r="Z104" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG104" t="b">
         <v>0</v>
@@ -7658,10 +7709,10 @@
         </is>
       </c>
       <c r="Z105" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG105" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH105" t="b">
         <v>0</v>
@@ -7724,7 +7775,7 @@
         </is>
       </c>
       <c r="Z106" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG106" t="b">
         <v>0</v>
@@ -7790,7 +7841,7 @@
         </is>
       </c>
       <c r="Z107" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG107" t="b">
         <v>0</v>
@@ -7856,7 +7907,7 @@
         </is>
       </c>
       <c r="Z108" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG108" t="b">
         <v>0</v>
@@ -7922,7 +7973,7 @@
         </is>
       </c>
       <c r="Z109" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG109" t="b">
         <v>0</v>
@@ -7988,7 +8039,7 @@
         </is>
       </c>
       <c r="Z110" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG110" t="b">
         <v>0</v>
@@ -8054,7 +8105,7 @@
         </is>
       </c>
       <c r="Z111" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG111" t="b">
         <v>0</v>
@@ -8120,7 +8171,7 @@
         </is>
       </c>
       <c r="Z112" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG112" t="b">
         <v>0</v>
@@ -8186,7 +8237,7 @@
         </is>
       </c>
       <c r="Z113" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG113" t="b">
         <v>0</v>
@@ -8252,7 +8303,7 @@
         </is>
       </c>
       <c r="Z114" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG114" t="b">
         <v>0</v>
@@ -8318,13 +8369,13 @@
         </is>
       </c>
       <c r="Z115" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG115" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH115" t="b">
         <v>1</v>
-      </c>
-      <c r="AG115" t="b">
-        <v>0</v>
-      </c>
-      <c r="AH115" t="b">
-        <v>0</v>
       </c>
       <c r="AI115" t="inlineStr">
         <is>
@@ -8384,7 +8435,7 @@
         </is>
       </c>
       <c r="Z116" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG116" t="b">
         <v>0</v>
@@ -8450,7 +8501,7 @@
         </is>
       </c>
       <c r="Z117" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG117" t="b">
         <v>0</v>
@@ -8516,13 +8567,13 @@
         </is>
       </c>
       <c r="Z118" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG118" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH118" t="b">
         <v>1</v>
-      </c>
-      <c r="AG118" t="b">
-        <v>0</v>
-      </c>
-      <c r="AH118" t="b">
-        <v>0</v>
       </c>
       <c r="AI118" t="inlineStr">
         <is>
@@ -8582,13 +8633,13 @@
         </is>
       </c>
       <c r="Z119" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG119" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH119" t="b">
         <v>1</v>
-      </c>
-      <c r="AG119" t="b">
-        <v>0</v>
-      </c>
-      <c r="AH119" t="b">
-        <v>0</v>
       </c>
       <c r="AI119" t="inlineStr">
         <is>
@@ -8648,13 +8699,13 @@
         </is>
       </c>
       <c r="Z120" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG120" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH120" t="b">
         <v>1</v>
-      </c>
-      <c r="AG120" t="b">
-        <v>0</v>
-      </c>
-      <c r="AH120" t="b">
-        <v>0</v>
       </c>
       <c r="AI120" t="inlineStr">
         <is>
@@ -8714,7 +8765,7 @@
         </is>
       </c>
       <c r="Z121" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG121" t="b">
         <v>0</v>
@@ -8780,7 +8831,7 @@
         </is>
       </c>
       <c r="Z122" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG122" t="b">
         <v>0</v>
@@ -8846,7 +8897,7 @@
         </is>
       </c>
       <c r="Z123" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG123" t="b">
         <v>0</v>
@@ -8912,7 +8963,7 @@
         </is>
       </c>
       <c r="Z124" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG124" t="b">
         <v>0</v>
@@ -8978,7 +9029,7 @@
         </is>
       </c>
       <c r="Z125" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG125" t="b">
         <v>0</v>
@@ -9044,13 +9095,13 @@
         </is>
       </c>
       <c r="Z126" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG126" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH126" t="b">
         <v>1</v>
-      </c>
-      <c r="AG126" t="b">
-        <v>0</v>
-      </c>
-      <c r="AH126" t="b">
-        <v>0</v>
       </c>
       <c r="AI126" t="inlineStr">
         <is>
@@ -9110,7 +9161,7 @@
         </is>
       </c>
       <c r="Z127" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG127" t="b">
         <v>0</v>
@@ -9176,13 +9227,13 @@
         </is>
       </c>
       <c r="Z128" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG128" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH128" t="b">
         <v>1</v>
-      </c>
-      <c r="AG128" t="b">
-        <v>0</v>
-      </c>
-      <c r="AH128" t="b">
-        <v>0</v>
       </c>
       <c r="AI128" t="inlineStr">
         <is>
@@ -9242,7 +9293,7 @@
         </is>
       </c>
       <c r="Z129" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG129" t="b">
         <v>0</v>
@@ -9357,7 +9408,7 @@
         </is>
       </c>
       <c r="Z130" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG130" t="b">
         <v>0</v>
@@ -9472,7 +9523,7 @@
         </is>
       </c>
       <c r="Z131" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG131" t="b">
         <v>0</v>
@@ -9587,7 +9638,7 @@
         </is>
       </c>
       <c r="Z132" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG132" t="b">
         <v>0</v>
@@ -9702,7 +9753,7 @@
         </is>
       </c>
       <c r="Z133" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG133" t="b">
         <v>0</v>
@@ -9817,7 +9868,7 @@
         </is>
       </c>
       <c r="Z134" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG134" t="b">
         <v>0</v>
@@ -9932,7 +9983,7 @@
         </is>
       </c>
       <c r="Z135" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG135" t="b">
         <v>0</v>
@@ -10047,7 +10098,7 @@
         </is>
       </c>
       <c r="Z136" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG136" t="b">
         <v>0</v>
@@ -10159,7 +10210,7 @@
         </is>
       </c>
       <c r="Z137" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG137" t="b">
         <v>0</v>
@@ -10274,7 +10325,7 @@
         </is>
       </c>
       <c r="Z138" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG138" t="b">
         <v>0</v>
@@ -10389,7 +10440,7 @@
         </is>
       </c>
       <c r="Z139" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG139" t="b">
         <v>0</v>
@@ -10504,7 +10555,7 @@
         </is>
       </c>
       <c r="Z140" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG140" t="b">
         <v>0</v>
@@ -10619,7 +10670,7 @@
         </is>
       </c>
       <c r="Z141" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG141" t="b">
         <v>0</v>
@@ -10734,7 +10785,7 @@
         </is>
       </c>
       <c r="Z142" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG142" t="b">
         <v>0</v>
@@ -10849,7 +10900,7 @@
         </is>
       </c>
       <c r="Z143" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG143" t="b">
         <v>0</v>
@@ -10964,7 +11015,7 @@
         </is>
       </c>
       <c r="Z144" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG144" t="b">
         <v>0</v>
@@ -11079,7 +11130,7 @@
         </is>
       </c>
       <c r="Z145" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG145" t="b">
         <v>0</v>
@@ -11093,8 +11144,813 @@
         </is>
       </c>
     </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>1102</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>亞泥</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E146" t="n">
+        <v>72.81999999999999</v>
+      </c>
+      <c r="F146" t="n">
+        <v>43.53</v>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>Reject</t>
+        </is>
+      </c>
+      <c r="I146" t="b">
+        <v>0</v>
+      </c>
+      <c r="J146" t="n">
+        <v>5.33</v>
+      </c>
+      <c r="K146" t="n">
+        <v>35.6</v>
+      </c>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M146" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="N146" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="O146" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="P146" t="n">
+        <v>32.72</v>
+      </c>
+      <c r="Q146" t="n">
+        <v>60.17</v>
+      </c>
+      <c r="R146" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="S146" t="n">
+        <v>5.5283</v>
+      </c>
+      <c r="T146" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U146" t="inlineStr">
+        <is>
+          <t>materials</t>
+        </is>
+      </c>
+      <c r="V146" t="n">
+        <v>33.8</v>
+      </c>
+      <c r="W146" t="n">
+        <v>37.2953</v>
+      </c>
+      <c r="X146" t="n">
+        <v>31.9314</v>
+      </c>
+      <c r="Y146" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z146" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG146" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH146" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI146" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>1216</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>統一</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E147" t="n">
+        <v>71.53</v>
+      </c>
+      <c r="F147" t="n">
+        <v>40.66</v>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>Reject</t>
+        </is>
+      </c>
+      <c r="I147" t="b">
+        <v>0</v>
+      </c>
+      <c r="J147" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="K147" t="n">
+        <v>79.29000000000001</v>
+      </c>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>gap_MM_Target_Up</t>
+        </is>
+      </c>
+      <c r="M147" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="N147" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="O147" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="P147" t="n">
+        <v>74.95</v>
+      </c>
+      <c r="Q147" t="n">
+        <v>54.38</v>
+      </c>
+      <c r="R147" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S147" t="n">
+        <v>6.1977</v>
+      </c>
+      <c r="T147" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U147" t="inlineStr">
+        <is>
+          <t>unclassified</t>
+        </is>
+      </c>
+      <c r="V147" t="n">
+        <v>77.5</v>
+      </c>
+      <c r="W147" t="n">
+        <v>85.5526</v>
+      </c>
+      <c r="X147" t="n">
+        <v>72.6968</v>
+      </c>
+      <c r="Y147" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z147" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG147" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH147" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI147" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>1519</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>華城</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E148" t="n">
+        <v>72.48999999999999</v>
+      </c>
+      <c r="F148" t="n">
+        <v>50.38</v>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I148" t="b">
+        <v>0</v>
+      </c>
+      <c r="J148" t="n">
+        <v>10</v>
+      </c>
+      <c r="K148" t="n">
+        <v>789.8</v>
+      </c>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M148" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N148" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="O148" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="P148" t="n">
+        <v>676.3099999999999</v>
+      </c>
+      <c r="Q148" t="n">
+        <v>59.2</v>
+      </c>
+      <c r="R148" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S148" t="n">
+        <v>7</v>
+      </c>
+      <c r="T148" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U148" t="inlineStr">
+        <is>
+          <t>industrial</t>
+        </is>
+      </c>
+      <c r="V148" t="n">
+        <v>718</v>
+      </c>
+      <c r="W148" t="n">
+        <v>861.6</v>
+      </c>
+      <c r="X148" t="n">
+        <v>667.74</v>
+      </c>
+      <c r="Y148" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z148" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG148" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH148" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI148" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>2301</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>光寶科</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E149" t="n">
+        <v>79.95</v>
+      </c>
+      <c r="F149" t="n">
+        <v>46.17</v>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I149" t="b">
+        <v>0</v>
+      </c>
+      <c r="J149" t="n">
+        <v>10</v>
+      </c>
+      <c r="K149" t="n">
+        <v>300.85</v>
+      </c>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M149" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N149" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="O149" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P149" t="n">
+        <v>257.38</v>
+      </c>
+      <c r="Q149" t="n">
+        <v>64.48</v>
+      </c>
+      <c r="R149" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="S149" t="n">
+        <v>7</v>
+      </c>
+      <c r="T149" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U149" t="inlineStr">
+        <is>
+          <t>ai_hardware</t>
+        </is>
+      </c>
+      <c r="V149" t="n">
+        <v>273.5</v>
+      </c>
+      <c r="W149" t="n">
+        <v>328.2</v>
+      </c>
+      <c r="X149" t="n">
+        <v>254.355</v>
+      </c>
+      <c r="Y149" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z149" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG149" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH149" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI149" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>2603</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>長榮</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E150" t="n">
+        <v>84.33</v>
+      </c>
+      <c r="F150" t="n">
+        <v>29.55</v>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>Reject</t>
+        </is>
+      </c>
+      <c r="I150" t="b">
+        <v>0</v>
+      </c>
+      <c r="J150" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="K150" t="n">
+        <v>244</v>
+      </c>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M150" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="N150" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="O150" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P150" t="n">
+        <v>222</v>
+      </c>
+      <c r="Q150" t="n">
+        <v>80.34</v>
+      </c>
+      <c r="R150" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="S150" t="n">
+        <v>7</v>
+      </c>
+      <c r="T150" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U150" t="inlineStr">
+        <is>
+          <t>shipping</t>
+        </is>
+      </c>
+      <c r="V150" t="n">
+        <v>240.5</v>
+      </c>
+      <c r="W150" t="n">
+        <v>288.6</v>
+      </c>
+      <c r="X150" t="n">
+        <v>223.665</v>
+      </c>
+      <c r="Y150" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z150" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG150" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH150" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI150" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>3008</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>大立光</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E151" t="n">
+        <v>85.34</v>
+      </c>
+      <c r="F151" t="n">
+        <v>44.65</v>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I151" t="b">
+        <v>0</v>
+      </c>
+      <c r="J151" t="n">
+        <v>10</v>
+      </c>
+      <c r="K151" t="n">
+        <v>6105</v>
+      </c>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M151" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N151" t="n">
+        <v>3</v>
+      </c>
+      <c r="O151" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P151" t="n">
+        <v>4846.85</v>
+      </c>
+      <c r="Q151" t="n">
+        <v>84.36</v>
+      </c>
+      <c r="R151" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="S151" t="n">
+        <v>7</v>
+      </c>
+      <c r="T151" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U151" t="inlineStr">
+        <is>
+          <t>electronic_components</t>
+        </is>
+      </c>
+      <c r="V151" t="n">
+        <v>5550</v>
+      </c>
+      <c r="W151" t="n">
+        <v>6660</v>
+      </c>
+      <c r="X151" t="n">
+        <v>5161.5</v>
+      </c>
+      <c r="Y151" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z151" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG151" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH151" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI151" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>3037</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>欣興</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E152" t="n">
+        <v>77.18000000000001</v>
+      </c>
+      <c r="F152" t="n">
+        <v>46.72</v>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I152" t="b">
+        <v>0</v>
+      </c>
+      <c r="J152" t="n">
+        <v>10</v>
+      </c>
+      <c r="K152" t="n">
+        <v>1243</v>
+      </c>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M152" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N152" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="O152" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P152" t="n">
+        <v>1036.5</v>
+      </c>
+      <c r="Q152" t="n">
+        <v>74.81999999999999</v>
+      </c>
+      <c r="R152" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="S152" t="n">
+        <v>7</v>
+      </c>
+      <c r="T152" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U152" t="inlineStr">
+        <is>
+          <t>electronic_components</t>
+        </is>
+      </c>
+      <c r="V152" t="n">
+        <v>1130</v>
+      </c>
+      <c r="W152" t="n">
+        <v>1356</v>
+      </c>
+      <c r="X152" t="n">
+        <v>1050.9</v>
+      </c>
+      <c r="Y152" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z152" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG152" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH152" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI152" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AJ145"/>
+  <autoFilter ref="A1:AJ152"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -11334,7 +12190,7 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>2026-08-18 17:58:12</t>
+          <t>2026-08-19 14:24:13</t>
         </is>
       </c>
     </row>
@@ -11381,7 +12237,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>144</v>
+        <v>151</v>
       </c>
     </row>
     <row r="7">
@@ -11401,7 +12257,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>144</v>
+        <v>151</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-08-20 01:51:53
</commit_message>
<xml_diff>
--- a/data/swing_performance_analysis.xlsx
+++ b/data/swing_performance_analysis.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'T20_Tracking'!$A$1:$AJ$152</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'T20_Tracking'!$A$1:$AJ$163</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ152"/>
+  <dimension ref="A1:AJ163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -731,7 +731,7 @@
         </is>
       </c>
       <c r="Z2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA2" t="n">
         <v>-1.45</v>
@@ -800,7 +800,7 @@
         </is>
       </c>
       <c r="Z3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA3" t="n">
         <v>-5.5</v>
@@ -869,7 +869,7 @@
         </is>
       </c>
       <c r="Z4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA4" t="n">
         <v>21.91</v>
@@ -938,7 +938,7 @@
         </is>
       </c>
       <c r="Z5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA5" t="n">
         <v>3.92</v>
@@ -947,7 +947,7 @@
         <v>0</v>
       </c>
       <c r="AH5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI5" t="inlineStr">
         <is>
@@ -1007,7 +1007,7 @@
         </is>
       </c>
       <c r="Z6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA6" t="n">
         <v>7.73</v>
@@ -1076,7 +1076,7 @@
         </is>
       </c>
       <c r="Z7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA7" t="n">
         <v>5.54</v>
@@ -1145,7 +1145,7 @@
         </is>
       </c>
       <c r="Z8" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA8" t="n">
         <v>-11.56</v>
@@ -1214,7 +1214,7 @@
         </is>
       </c>
       <c r="Z9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA9" t="n">
         <v>-10.14</v>
@@ -1283,7 +1283,7 @@
         </is>
       </c>
       <c r="Z10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA10" t="n">
         <v>-12.27</v>
@@ -1352,7 +1352,7 @@
         </is>
       </c>
       <c r="Z11" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA11" t="n">
         <v>-6.97</v>
@@ -1421,7 +1421,7 @@
         </is>
       </c>
       <c r="Z12" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA12" t="n">
         <v>5.13</v>
@@ -1490,7 +1490,7 @@
         </is>
       </c>
       <c r="Z13" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA13" t="n">
         <v>-5.54</v>
@@ -1621,7 +1621,7 @@
         </is>
       </c>
       <c r="Z15" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA15" t="n">
         <v>3.09</v>
@@ -1690,7 +1690,7 @@
         </is>
       </c>
       <c r="Z16" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA16" t="n">
         <v>9.31</v>
@@ -1759,7 +1759,7 @@
         </is>
       </c>
       <c r="Z17" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA17" t="n">
         <v>-1.43</v>
@@ -1828,7 +1828,7 @@
         </is>
       </c>
       <c r="Z18" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA18" t="n">
         <v>-6.69</v>
@@ -1897,7 +1897,7 @@
         </is>
       </c>
       <c r="Z19" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA19" t="n">
         <v>-4.07</v>
@@ -1966,7 +1966,7 @@
         </is>
       </c>
       <c r="Z20" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA20" t="n">
         <v>-1.42</v>
@@ -2035,7 +2035,7 @@
         </is>
       </c>
       <c r="Z21" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA21" t="n">
         <v>-3.59</v>
@@ -2104,7 +2104,7 @@
         </is>
       </c>
       <c r="Z22" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA22" t="n">
         <v>14.67</v>
@@ -2173,7 +2173,7 @@
         </is>
       </c>
       <c r="Z23" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA23" t="n">
         <v>2.43</v>
@@ -2242,7 +2242,7 @@
         </is>
       </c>
       <c r="Z24" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA24" t="n">
         <v>1.05</v>
@@ -2311,13 +2311,13 @@
         </is>
       </c>
       <c r="Z25" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA25" t="n">
         <v>8.18</v>
       </c>
       <c r="AG25" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH25" t="b">
         <v>0</v>
@@ -2380,7 +2380,7 @@
         </is>
       </c>
       <c r="Z26" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA26" t="n">
         <v>6.01</v>
@@ -2449,7 +2449,7 @@
         </is>
       </c>
       <c r="Z27" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA27" t="n">
         <v>13.83</v>
@@ -2518,7 +2518,7 @@
         </is>
       </c>
       <c r="Z28" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA28" t="n">
         <v>-10.91</v>
@@ -2587,7 +2587,7 @@
         </is>
       </c>
       <c r="Z29" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA29" t="n">
         <v>-2.87</v>
@@ -2656,7 +2656,7 @@
         </is>
       </c>
       <c r="Z30" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA30" t="n">
         <v>-8.630000000000001</v>
@@ -2725,7 +2725,7 @@
         </is>
       </c>
       <c r="Z31" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA31" t="n">
         <v>-0.91</v>
@@ -2794,7 +2794,7 @@
         </is>
       </c>
       <c r="Z32" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA32" t="n">
         <v>-6.43</v>
@@ -2863,7 +2863,7 @@
         </is>
       </c>
       <c r="Z33" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA33" t="n">
         <v>-3.11</v>
@@ -3056,7 +3056,7 @@
         </is>
       </c>
       <c r="Z36" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA36" t="n">
         <v>-3.48</v>
@@ -3125,7 +3125,7 @@
         </is>
       </c>
       <c r="Z37" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA37" t="n">
         <v>10.15</v>
@@ -3194,7 +3194,7 @@
         </is>
       </c>
       <c r="Z38" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA38" t="n">
         <v>-5.23</v>
@@ -3263,7 +3263,7 @@
         </is>
       </c>
       <c r="Z39" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA39" t="n">
         <v>-5.13</v>
@@ -3332,7 +3332,7 @@
         </is>
       </c>
       <c r="Z40" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA40" t="n">
         <v>-3.13</v>
@@ -3401,7 +3401,7 @@
         </is>
       </c>
       <c r="Z41" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA41" t="n">
         <v>-4.05</v>
@@ -3470,7 +3470,7 @@
         </is>
       </c>
       <c r="Z42" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA42" t="n">
         <v>1.86</v>
@@ -3539,7 +3539,7 @@
         </is>
       </c>
       <c r="Z43" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA43" t="n">
         <v>8.460000000000001</v>
@@ -3608,7 +3608,7 @@
         </is>
       </c>
       <c r="Z44" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA44" t="n">
         <v>10.82</v>
@@ -3677,7 +3677,7 @@
         </is>
       </c>
       <c r="Z45" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA45" t="n">
         <v>-0.71</v>
@@ -3746,7 +3746,7 @@
         </is>
       </c>
       <c r="Z46" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA46" t="n">
         <v>12.1</v>
@@ -3815,7 +3815,7 @@
         </is>
       </c>
       <c r="Z47" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA47" t="n">
         <v>2.72</v>
@@ -3884,7 +3884,7 @@
         </is>
       </c>
       <c r="Z48" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA48" t="n">
         <v>5.32</v>
@@ -3953,7 +3953,7 @@
         </is>
       </c>
       <c r="Z49" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA49" t="n">
         <v>-3.36</v>
@@ -4022,7 +4022,7 @@
         </is>
       </c>
       <c r="Z50" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA50" t="n">
         <v>9.17</v>
@@ -4091,7 +4091,7 @@
         </is>
       </c>
       <c r="Z51" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA51" t="n">
         <v>8.08</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="Z52" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA52" t="n">
         <v>20.55</v>
@@ -4229,7 +4229,7 @@
         </is>
       </c>
       <c r="Z53" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA53" t="n">
         <v>-0.32</v>
@@ -4298,7 +4298,7 @@
         </is>
       </c>
       <c r="Z54" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA54" t="n">
         <v>-5.24</v>
@@ -4429,7 +4429,7 @@
         </is>
       </c>
       <c r="Z56" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA56" t="n">
         <v>-4.49</v>
@@ -4498,7 +4498,7 @@
         </is>
       </c>
       <c r="Z57" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA57" t="n">
         <v>-0.28</v>
@@ -4567,7 +4567,7 @@
         </is>
       </c>
       <c r="Z58" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA58" t="n">
         <v>-8.779999999999999</v>
@@ -4636,7 +4636,7 @@
         </is>
       </c>
       <c r="Z59" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA59" t="n">
         <v>-4.05</v>
@@ -4705,7 +4705,7 @@
         </is>
       </c>
       <c r="Z60" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA60" t="n">
         <v>-9.26</v>
@@ -4774,7 +4774,7 @@
         </is>
       </c>
       <c r="Z61" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA61" t="n">
         <v>8.57</v>
@@ -4843,7 +4843,7 @@
         </is>
       </c>
       <c r="Z62" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA62" t="n">
         <v>-3.42</v>
@@ -4912,7 +4912,7 @@
         </is>
       </c>
       <c r="Z63" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA63" t="n">
         <v>2.62</v>
@@ -4981,7 +4981,7 @@
         </is>
       </c>
       <c r="Z64" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA64" t="n">
         <v>1.17</v>
@@ -5050,13 +5050,13 @@
         </is>
       </c>
       <c r="Z65" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA65" t="n">
         <v>12.12</v>
       </c>
       <c r="AG65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH65" t="b">
         <v>0</v>
@@ -5119,7 +5119,7 @@
         </is>
       </c>
       <c r="Z66" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA66" t="n">
         <v>-1.13</v>
@@ -5188,7 +5188,7 @@
         </is>
       </c>
       <c r="Z67" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA67" t="n">
         <v>21.05</v>
@@ -5257,7 +5257,7 @@
         </is>
       </c>
       <c r="Z68" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA68" t="n">
         <v>6.36</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="Z69" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA69" t="n">
         <v>-5.94</v>
@@ -5457,7 +5457,7 @@
         </is>
       </c>
       <c r="Z71" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA71" t="n">
         <v>3.22</v>
@@ -5526,7 +5526,7 @@
         </is>
       </c>
       <c r="Z72" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA72" t="n">
         <v>-2.78</v>
@@ -5595,7 +5595,7 @@
         </is>
       </c>
       <c r="Z73" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA73" t="n">
         <v>5.81</v>
@@ -5664,7 +5664,7 @@
         </is>
       </c>
       <c r="Z74" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA74" t="n">
         <v>-5.04</v>
@@ -5733,7 +5733,10 @@
         </is>
       </c>
       <c r="Z75" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA75" t="n">
+        <v>-1.53</v>
       </c>
       <c r="AG75" t="b">
         <v>0</v>
@@ -5799,7 +5802,10 @@
         </is>
       </c>
       <c r="Z76" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA76" t="n">
+        <v>-1.02</v>
       </c>
       <c r="AG76" t="b">
         <v>0</v>
@@ -5865,7 +5871,10 @@
         </is>
       </c>
       <c r="Z77" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA77" t="n">
+        <v>0.37</v>
       </c>
       <c r="AG77" t="b">
         <v>0</v>
@@ -5931,7 +5940,10 @@
         </is>
       </c>
       <c r="Z78" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA78" t="n">
+        <v>-11.94</v>
       </c>
       <c r="AG78" t="b">
         <v>0</v>
@@ -5997,7 +6009,10 @@
         </is>
       </c>
       <c r="Z79" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA79" t="n">
+        <v>-2.44</v>
       </c>
       <c r="AG79" t="b">
         <v>0</v>
@@ -6063,7 +6078,10 @@
         </is>
       </c>
       <c r="Z80" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA80" t="n">
+        <v>0.58</v>
       </c>
       <c r="AG80" t="b">
         <v>0</v>
@@ -6129,10 +6147,13 @@
         </is>
       </c>
       <c r="Z81" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA81" t="n">
+        <v>12.3</v>
       </c>
       <c r="AG81" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH81" t="b">
         <v>0</v>
@@ -6195,7 +6216,10 @@
         </is>
       </c>
       <c r="Z82" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA82" t="n">
+        <v>23.43</v>
       </c>
       <c r="AG82" t="b">
         <v>1</v>
@@ -6261,7 +6285,10 @@
         </is>
       </c>
       <c r="Z83" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA83" t="n">
+        <v>-1.63</v>
       </c>
       <c r="AG83" t="b">
         <v>0</v>
@@ -6327,7 +6354,10 @@
         </is>
       </c>
       <c r="Z84" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA84" t="n">
+        <v>17.81</v>
       </c>
       <c r="AG84" t="b">
         <v>1</v>
@@ -6393,7 +6423,10 @@
         </is>
       </c>
       <c r="Z85" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA85" t="n">
+        <v>-8.880000000000001</v>
       </c>
       <c r="AG85" t="b">
         <v>0</v>
@@ -6459,7 +6492,10 @@
         </is>
       </c>
       <c r="Z86" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA86" t="n">
+        <v>-3.34</v>
       </c>
       <c r="AG86" t="b">
         <v>0</v>
@@ -6525,7 +6561,10 @@
         </is>
       </c>
       <c r="Z87" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA87" t="n">
+        <v>-11.46</v>
       </c>
       <c r="AG87" t="b">
         <v>0</v>
@@ -6591,7 +6630,10 @@
         </is>
       </c>
       <c r="Z88" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA88" t="n">
+        <v>-3.81</v>
       </c>
       <c r="AG88" t="b">
         <v>0</v>
@@ -6657,7 +6699,10 @@
         </is>
       </c>
       <c r="Z89" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA89" t="n">
+        <v>4.61</v>
       </c>
       <c r="AG89" t="b">
         <v>0</v>
@@ -6785,7 +6830,10 @@
         </is>
       </c>
       <c r="Z91" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA91" t="n">
+        <v>0</v>
       </c>
       <c r="AG91" t="b">
         <v>0</v>
@@ -6851,7 +6899,7 @@
         </is>
       </c>
       <c r="Z92" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG92" t="b">
         <v>0</v>
@@ -6917,7 +6965,7 @@
         </is>
       </c>
       <c r="Z93" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG93" t="b">
         <v>0</v>
@@ -6983,7 +7031,7 @@
         </is>
       </c>
       <c r="Z94" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG94" t="b">
         <v>0</v>
@@ -7049,7 +7097,7 @@
         </is>
       </c>
       <c r="Z95" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG95" t="b">
         <v>0</v>
@@ -7115,7 +7163,7 @@
         </is>
       </c>
       <c r="Z96" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG96" t="b">
         <v>0</v>
@@ -7181,7 +7229,7 @@
         </is>
       </c>
       <c r="Z97" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG97" t="b">
         <v>0</v>
@@ -7247,7 +7295,7 @@
         </is>
       </c>
       <c r="Z98" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG98" t="b">
         <v>0</v>
@@ -7313,7 +7361,7 @@
         </is>
       </c>
       <c r="Z99" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG99" t="b">
         <v>0</v>
@@ -7379,7 +7427,7 @@
         </is>
       </c>
       <c r="Z100" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG100" t="b">
         <v>0</v>
@@ -7445,7 +7493,7 @@
         </is>
       </c>
       <c r="Z101" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG101" t="b">
         <v>1</v>
@@ -7511,7 +7559,7 @@
         </is>
       </c>
       <c r="Z102" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG102" t="b">
         <v>1</v>
@@ -7577,7 +7625,7 @@
         </is>
       </c>
       <c r="Z103" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG103" t="b">
         <v>0</v>
@@ -7643,7 +7691,7 @@
         </is>
       </c>
       <c r="Z104" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG104" t="b">
         <v>0</v>
@@ -7709,7 +7757,7 @@
         </is>
       </c>
       <c r="Z105" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG105" t="b">
         <v>1</v>
@@ -7775,7 +7823,7 @@
         </is>
       </c>
       <c r="Z106" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG106" t="b">
         <v>0</v>
@@ -7841,7 +7889,7 @@
         </is>
       </c>
       <c r="Z107" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG107" t="b">
         <v>0</v>
@@ -7907,7 +7955,7 @@
         </is>
       </c>
       <c r="Z108" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG108" t="b">
         <v>0</v>
@@ -7973,7 +8021,7 @@
         </is>
       </c>
       <c r="Z109" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG109" t="b">
         <v>0</v>
@@ -8039,7 +8087,7 @@
         </is>
       </c>
       <c r="Z110" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG110" t="b">
         <v>0</v>
@@ -8105,7 +8153,7 @@
         </is>
       </c>
       <c r="Z111" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG111" t="b">
         <v>0</v>
@@ -8171,7 +8219,7 @@
         </is>
       </c>
       <c r="Z112" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG112" t="b">
         <v>0</v>
@@ -8237,7 +8285,7 @@
         </is>
       </c>
       <c r="Z113" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG113" t="b">
         <v>0</v>
@@ -8303,7 +8351,7 @@
         </is>
       </c>
       <c r="Z114" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG114" t="b">
         <v>0</v>
@@ -8369,7 +8417,7 @@
         </is>
       </c>
       <c r="Z115" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG115" t="b">
         <v>0</v>
@@ -8435,7 +8483,7 @@
         </is>
       </c>
       <c r="Z116" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG116" t="b">
         <v>0</v>
@@ -8501,7 +8549,7 @@
         </is>
       </c>
       <c r="Z117" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG117" t="b">
         <v>0</v>
@@ -8567,7 +8615,7 @@
         </is>
       </c>
       <c r="Z118" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG118" t="b">
         <v>0</v>
@@ -8633,7 +8681,7 @@
         </is>
       </c>
       <c r="Z119" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG119" t="b">
         <v>0</v>
@@ -8699,7 +8747,7 @@
         </is>
       </c>
       <c r="Z120" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG120" t="b">
         <v>0</v>
@@ -8765,7 +8813,7 @@
         </is>
       </c>
       <c r="Z121" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG121" t="b">
         <v>0</v>
@@ -8831,7 +8879,7 @@
         </is>
       </c>
       <c r="Z122" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG122" t="b">
         <v>0</v>
@@ -8897,7 +8945,7 @@
         </is>
       </c>
       <c r="Z123" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG123" t="b">
         <v>0</v>
@@ -8963,7 +9011,7 @@
         </is>
       </c>
       <c r="Z124" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG124" t="b">
         <v>0</v>
@@ -9029,7 +9077,7 @@
         </is>
       </c>
       <c r="Z125" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG125" t="b">
         <v>0</v>
@@ -9095,7 +9143,7 @@
         </is>
       </c>
       <c r="Z126" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG126" t="b">
         <v>0</v>
@@ -9161,7 +9209,7 @@
         </is>
       </c>
       <c r="Z127" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG127" t="b">
         <v>0</v>
@@ -9227,7 +9275,7 @@
         </is>
       </c>
       <c r="Z128" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG128" t="b">
         <v>0</v>
@@ -9293,7 +9341,7 @@
         </is>
       </c>
       <c r="Z129" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG129" t="b">
         <v>0</v>
@@ -9408,7 +9456,7 @@
         </is>
       </c>
       <c r="Z130" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG130" t="b">
         <v>0</v>
@@ -9523,7 +9571,7 @@
         </is>
       </c>
       <c r="Z131" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG131" t="b">
         <v>0</v>
@@ -9638,7 +9686,7 @@
         </is>
       </c>
       <c r="Z132" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG132" t="b">
         <v>0</v>
@@ -9753,7 +9801,7 @@
         </is>
       </c>
       <c r="Z133" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG133" t="b">
         <v>0</v>
@@ -9868,7 +9916,7 @@
         </is>
       </c>
       <c r="Z134" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG134" t="b">
         <v>0</v>
@@ -9983,7 +10031,7 @@
         </is>
       </c>
       <c r="Z135" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG135" t="b">
         <v>0</v>
@@ -10098,7 +10146,7 @@
         </is>
       </c>
       <c r="Z136" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG136" t="b">
         <v>0</v>
@@ -10210,7 +10258,7 @@
         </is>
       </c>
       <c r="Z137" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG137" t="b">
         <v>0</v>
@@ -10325,7 +10373,7 @@
         </is>
       </c>
       <c r="Z138" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG138" t="b">
         <v>0</v>
@@ -10440,7 +10488,7 @@
         </is>
       </c>
       <c r="Z139" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG139" t="b">
         <v>0</v>
@@ -10555,7 +10603,7 @@
         </is>
       </c>
       <c r="Z140" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG140" t="b">
         <v>0</v>
@@ -10670,7 +10718,7 @@
         </is>
       </c>
       <c r="Z141" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG141" t="b">
         <v>0</v>
@@ -10785,7 +10833,7 @@
         </is>
       </c>
       <c r="Z142" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG142" t="b">
         <v>0</v>
@@ -10900,7 +10948,7 @@
         </is>
       </c>
       <c r="Z143" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG143" t="b">
         <v>0</v>
@@ -11015,7 +11063,7 @@
         </is>
       </c>
       <c r="Z144" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG144" t="b">
         <v>0</v>
@@ -11130,7 +11178,7 @@
         </is>
       </c>
       <c r="Z145" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG145" t="b">
         <v>0</v>
@@ -11245,7 +11293,7 @@
         </is>
       </c>
       <c r="Z146" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG146" t="b">
         <v>0</v>
@@ -11360,7 +11408,7 @@
         </is>
       </c>
       <c r="Z147" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG147" t="b">
         <v>0</v>
@@ -11475,7 +11523,7 @@
         </is>
       </c>
       <c r="Z148" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG148" t="b">
         <v>0</v>
@@ -11590,7 +11638,7 @@
         </is>
       </c>
       <c r="Z149" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG149" t="b">
         <v>0</v>
@@ -11705,7 +11753,7 @@
         </is>
       </c>
       <c r="Z150" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG150" t="b">
         <v>0</v>
@@ -11820,7 +11868,7 @@
         </is>
       </c>
       <c r="Z151" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG151" t="b">
         <v>0</v>
@@ -11935,7 +11983,7 @@
         </is>
       </c>
       <c r="Z152" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG152" t="b">
         <v>0</v>
@@ -11949,8 +11997,1273 @@
         </is>
       </c>
     </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>1102</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>亞泥</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E153" t="n">
+        <v>73.31</v>
+      </c>
+      <c r="F153" t="n">
+        <v>36.03</v>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>Reject</t>
+        </is>
+      </c>
+      <c r="I153" t="b">
+        <v>0</v>
+      </c>
+      <c r="J153" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="K153" t="n">
+        <v>36</v>
+      </c>
+      <c r="L153" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M153" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="N153" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="O153" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="P153" t="n">
+        <v>33.22</v>
+      </c>
+      <c r="Q153" t="n">
+        <v>63.56</v>
+      </c>
+      <c r="R153" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="S153" t="n">
+        <v>7</v>
+      </c>
+      <c r="T153" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U153" t="inlineStr">
+        <is>
+          <t>materials</t>
+        </is>
+      </c>
+      <c r="V153" t="n">
+        <v>34.85</v>
+      </c>
+      <c r="W153" t="n">
+        <v>39.1688</v>
+      </c>
+      <c r="X153" t="n">
+        <v>32.4105</v>
+      </c>
+      <c r="Y153" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z153" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG153" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH153" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI153" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>2049</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>上銀</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E154" t="n">
+        <v>76.09</v>
+      </c>
+      <c r="F154" t="n">
+        <v>48.61</v>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I154" t="b">
+        <v>0</v>
+      </c>
+      <c r="J154" t="n">
+        <v>10</v>
+      </c>
+      <c r="K154" t="n">
+        <v>427.35</v>
+      </c>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M154" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N154" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="O154" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="P154" t="n">
+        <v>372.5</v>
+      </c>
+      <c r="Q154" t="n">
+        <v>60.7</v>
+      </c>
+      <c r="R154" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="S154" t="n">
+        <v>7</v>
+      </c>
+      <c r="T154" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U154" t="inlineStr">
+        <is>
+          <t>industrial</t>
+        </is>
+      </c>
+      <c r="V154" t="n">
+        <v>388.5</v>
+      </c>
+      <c r="W154" t="n">
+        <v>466.2</v>
+      </c>
+      <c r="X154" t="n">
+        <v>361.305</v>
+      </c>
+      <c r="Y154" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z154" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG154" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH154" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI154" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>2301</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>光寶科</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E155" t="n">
+        <v>72.55</v>
+      </c>
+      <c r="F155" t="n">
+        <v>45.83</v>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I155" t="b">
+        <v>0</v>
+      </c>
+      <c r="J155" t="n">
+        <v>10</v>
+      </c>
+      <c r="K155" t="n">
+        <v>298.1</v>
+      </c>
+      <c r="L155" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M155" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N155" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="O155" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P155" t="n">
+        <v>262.83</v>
+      </c>
+      <c r="Q155" t="n">
+        <v>48.84</v>
+      </c>
+      <c r="R155" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S155" t="n">
+        <v>7</v>
+      </c>
+      <c r="T155" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U155" t="inlineStr">
+        <is>
+          <t>ai_hardware</t>
+        </is>
+      </c>
+      <c r="V155" t="n">
+        <v>271</v>
+      </c>
+      <c r="W155" t="n">
+        <v>325.2</v>
+      </c>
+      <c r="X155" t="n">
+        <v>252.03</v>
+      </c>
+      <c r="Y155" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z155" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG155" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH155" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI155" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>2395</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>研華</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E156" t="n">
+        <v>70.29000000000001</v>
+      </c>
+      <c r="F156" t="n">
+        <v>47.11</v>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I156" t="b">
+        <v>0</v>
+      </c>
+      <c r="J156" t="n">
+        <v>10</v>
+      </c>
+      <c r="K156" t="n">
+        <v>750.2</v>
+      </c>
+      <c r="L156" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M156" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N156" t="n">
+        <v>5</v>
+      </c>
+      <c r="O156" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="P156" t="n">
+        <v>649.5</v>
+      </c>
+      <c r="Q156" t="n">
+        <v>54.08</v>
+      </c>
+      <c r="R156" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S156" t="n">
+        <v>7</v>
+      </c>
+      <c r="T156" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U156" t="inlineStr">
+        <is>
+          <t>ai_hardware</t>
+        </is>
+      </c>
+      <c r="V156" t="n">
+        <v>682</v>
+      </c>
+      <c r="W156" t="n">
+        <v>818.4</v>
+      </c>
+      <c r="X156" t="n">
+        <v>634.26</v>
+      </c>
+      <c r="Y156" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z156" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG156" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH156" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI156" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>2408</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>南亞科</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E157" t="n">
+        <v>73.59</v>
+      </c>
+      <c r="F157" t="n">
+        <v>42.65</v>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I157" t="b">
+        <v>0</v>
+      </c>
+      <c r="J157" t="n">
+        <v>10</v>
+      </c>
+      <c r="K157" t="n">
+        <v>572</v>
+      </c>
+      <c r="L157" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M157" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N157" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="O157" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P157" t="n">
+        <v>494.5</v>
+      </c>
+      <c r="Q157" t="n">
+        <v>54.36</v>
+      </c>
+      <c r="R157" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S157" t="n">
+        <v>7</v>
+      </c>
+      <c r="T157" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U157" t="inlineStr">
+        <is>
+          <t>semiconductor</t>
+        </is>
+      </c>
+      <c r="V157" t="n">
+        <v>520</v>
+      </c>
+      <c r="W157" t="n">
+        <v>624</v>
+      </c>
+      <c r="X157" t="n">
+        <v>483.6</v>
+      </c>
+      <c r="Y157" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z157" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG157" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH157" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI157" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>2603</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>長榮</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E158" t="n">
+        <v>77.81999999999999</v>
+      </c>
+      <c r="F158" t="n">
+        <v>40.03</v>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I158" t="b">
+        <v>0</v>
+      </c>
+      <c r="J158" t="n">
+        <v>9.24</v>
+      </c>
+      <c r="K158" t="n">
+        <v>266</v>
+      </c>
+      <c r="L158" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M158" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="N158" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="O158" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P158" t="n">
+        <v>225.5</v>
+      </c>
+      <c r="Q158" t="n">
+        <v>70.2</v>
+      </c>
+      <c r="R158" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="S158" t="n">
+        <v>7</v>
+      </c>
+      <c r="T158" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U158" t="inlineStr">
+        <is>
+          <t>shipping</t>
+        </is>
+      </c>
+      <c r="V158" t="n">
+        <v>243.5</v>
+      </c>
+      <c r="W158" t="n">
+        <v>292.2</v>
+      </c>
+      <c r="X158" t="n">
+        <v>226.455</v>
+      </c>
+      <c r="Y158" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z158" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG158" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH158" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI158" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>2609</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>陽明</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E159" t="n">
+        <v>76.16</v>
+      </c>
+      <c r="F159" t="n">
+        <v>25.69</v>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>Reject</t>
+        </is>
+      </c>
+      <c r="I159" t="b">
+        <v>0</v>
+      </c>
+      <c r="J159" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="K159" t="n">
+        <v>60.1</v>
+      </c>
+      <c r="L159" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M159" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="N159" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="O159" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P159" t="n">
+        <v>55.3</v>
+      </c>
+      <c r="Q159" t="n">
+        <v>67.93000000000001</v>
+      </c>
+      <c r="R159" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="S159" t="n">
+        <v>7</v>
+      </c>
+      <c r="T159" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U159" t="inlineStr">
+        <is>
+          <t>shipping</t>
+        </is>
+      </c>
+      <c r="V159" t="n">
+        <v>59.7</v>
+      </c>
+      <c r="W159" t="n">
+        <v>71.64</v>
+      </c>
+      <c r="X159" t="n">
+        <v>55.521</v>
+      </c>
+      <c r="Y159" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z159" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG159" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH159" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI159" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>2615</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>萬海</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E160" t="n">
+        <v>84.39</v>
+      </c>
+      <c r="F160" t="n">
+        <v>39.6</v>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I160" t="b">
+        <v>0</v>
+      </c>
+      <c r="J160" t="n">
+        <v>8.890000000000001</v>
+      </c>
+      <c r="K160" t="n">
+        <v>117.6</v>
+      </c>
+      <c r="L160" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M160" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="N160" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="O160" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P160" t="n">
+        <v>96.40000000000001</v>
+      </c>
+      <c r="Q160" t="n">
+        <v>80.68000000000001</v>
+      </c>
+      <c r="R160" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="S160" t="n">
+        <v>7</v>
+      </c>
+      <c r="T160" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U160" t="inlineStr">
+        <is>
+          <t>shipping</t>
+        </is>
+      </c>
+      <c r="V160" t="n">
+        <v>108</v>
+      </c>
+      <c r="W160" t="n">
+        <v>129.6</v>
+      </c>
+      <c r="X160" t="n">
+        <v>100.44</v>
+      </c>
+      <c r="Y160" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z160" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG160" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH160" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI160" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>3008</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>大立光</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E161" t="n">
+        <v>77.73</v>
+      </c>
+      <c r="F161" t="n">
+        <v>42.98</v>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I161" t="b">
+        <v>0</v>
+      </c>
+      <c r="J161" t="n">
+        <v>10</v>
+      </c>
+      <c r="K161" t="n">
+        <v>6028</v>
+      </c>
+      <c r="L161" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M161" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N161" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="O161" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P161" t="n">
+        <v>4955.86</v>
+      </c>
+      <c r="Q161" t="n">
+        <v>69.89</v>
+      </c>
+      <c r="R161" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="S161" t="n">
+        <v>7</v>
+      </c>
+      <c r="T161" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U161" t="inlineStr">
+        <is>
+          <t>electronic_components</t>
+        </is>
+      </c>
+      <c r="V161" t="n">
+        <v>5480</v>
+      </c>
+      <c r="W161" t="n">
+        <v>6576</v>
+      </c>
+      <c r="X161" t="n">
+        <v>5096.4</v>
+      </c>
+      <c r="Y161" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z161" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG161" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH161" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI161" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>3037</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>欣興</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E162" t="n">
+        <v>70.59</v>
+      </c>
+      <c r="F162" t="n">
+        <v>43.04</v>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I162" t="b">
+        <v>0</v>
+      </c>
+      <c r="J162" t="n">
+        <v>10</v>
+      </c>
+      <c r="K162" t="n">
+        <v>1210</v>
+      </c>
+      <c r="L162" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M162" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N162" t="n">
+        <v>1</v>
+      </c>
+      <c r="O162" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P162" t="n">
+        <v>1064</v>
+      </c>
+      <c r="Q162" t="n">
+        <v>60.28</v>
+      </c>
+      <c r="R162" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="S162" t="n">
+        <v>7</v>
+      </c>
+      <c r="T162" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U162" t="inlineStr">
+        <is>
+          <t>electronic_components</t>
+        </is>
+      </c>
+      <c r="V162" t="n">
+        <v>1100</v>
+      </c>
+      <c r="W162" t="n">
+        <v>1320</v>
+      </c>
+      <c r="X162" t="n">
+        <v>1023</v>
+      </c>
+      <c r="Y162" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z162" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG162" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH162" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI162" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>6669</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>緯穎</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E163" t="n">
+        <v>74.44</v>
+      </c>
+      <c r="F163" t="n">
+        <v>54.53</v>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I163" t="b">
+        <v>0</v>
+      </c>
+      <c r="J163" t="n">
+        <v>10</v>
+      </c>
+      <c r="K163" t="n">
+        <v>6990.5</v>
+      </c>
+      <c r="L163" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M163" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N163" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="O163" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="P163" t="n">
+        <v>6297.5</v>
+      </c>
+      <c r="Q163" t="n">
+        <v>53.52</v>
+      </c>
+      <c r="R163" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S163" t="n">
+        <v>7</v>
+      </c>
+      <c r="T163" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U163" t="inlineStr">
+        <is>
+          <t>semiconductor</t>
+        </is>
+      </c>
+      <c r="V163" t="n">
+        <v>6355</v>
+      </c>
+      <c r="W163" t="n">
+        <v>7626</v>
+      </c>
+      <c r="X163" t="n">
+        <v>5910.15</v>
+      </c>
+      <c r="Y163" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z163" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG163" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH163" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI163" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AJ152"/>
+  <autoFilter ref="A1:AJ163"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -12190,7 +13503,7 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>2026-08-19 14:24:13</t>
+          <t>2026-08-20 09:51:49</t>
         </is>
       </c>
     </row>
@@ -12237,7 +13550,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>151</v>
+        <v>162</v>
       </c>
     </row>
     <row r="7">
@@ -12257,7 +13570,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>151</v>
+        <v>162</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-08-20 06:22:15
</commit_message>
<xml_diff>
--- a/data/swing_performance_analysis.xlsx
+++ b/data/swing_performance_analysis.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'T20_Tracking'!$A$1:$AJ$163</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'T20_Tracking'!$A$1:$AJ$171</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ163"/>
+  <dimension ref="A1:AJ171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3962,7 +3962,7 @@
         <v>0</v>
       </c>
       <c r="AH49" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI49" t="inlineStr">
         <is>
@@ -5736,7 +5736,7 @@
         <v>5</v>
       </c>
       <c r="AA75" t="n">
-        <v>-1.53</v>
+        <v>0.97</v>
       </c>
       <c r="AG75" t="b">
         <v>0</v>
@@ -5805,7 +5805,7 @@
         <v>5</v>
       </c>
       <c r="AA76" t="n">
-        <v>-1.02</v>
+        <v>-3.4</v>
       </c>
       <c r="AG76" t="b">
         <v>0</v>
@@ -5874,7 +5874,7 @@
         <v>5</v>
       </c>
       <c r="AA77" t="n">
-        <v>0.37</v>
+        <v>-0.93</v>
       </c>
       <c r="AG77" t="b">
         <v>0</v>
@@ -5943,7 +5943,7 @@
         <v>5</v>
       </c>
       <c r="AA78" t="n">
-        <v>-11.94</v>
+        <v>-12.58</v>
       </c>
       <c r="AG78" t="b">
         <v>0</v>
@@ -6012,7 +6012,7 @@
         <v>5</v>
       </c>
       <c r="AA79" t="n">
-        <v>-2.44</v>
+        <v>-3.58</v>
       </c>
       <c r="AG79" t="b">
         <v>0</v>
@@ -6150,7 +6150,7 @@
         <v>5</v>
       </c>
       <c r="AA81" t="n">
-        <v>12.3</v>
+        <v>14.15</v>
       </c>
       <c r="AG81" t="b">
         <v>1</v>
@@ -6219,7 +6219,7 @@
         <v>5</v>
       </c>
       <c r="AA82" t="n">
-        <v>23.43</v>
+        <v>29.71</v>
       </c>
       <c r="AG82" t="b">
         <v>1</v>
@@ -6288,7 +6288,7 @@
         <v>5</v>
       </c>
       <c r="AA83" t="n">
-        <v>-1.63</v>
+        <v>-1.5</v>
       </c>
       <c r="AG83" t="b">
         <v>0</v>
@@ -6357,7 +6357,7 @@
         <v>5</v>
       </c>
       <c r="AA84" t="n">
-        <v>17.81</v>
+        <v>18.35</v>
       </c>
       <c r="AG84" t="b">
         <v>1</v>
@@ -6426,7 +6426,7 @@
         <v>5</v>
       </c>
       <c r="AA85" t="n">
-        <v>-8.880000000000001</v>
+        <v>-8.630000000000001</v>
       </c>
       <c r="AG85" t="b">
         <v>0</v>
@@ -6495,7 +6495,7 @@
         <v>5</v>
       </c>
       <c r="AA86" t="n">
-        <v>-3.34</v>
+        <v>1.62</v>
       </c>
       <c r="AG86" t="b">
         <v>0</v>
@@ -6564,7 +6564,7 @@
         <v>5</v>
       </c>
       <c r="AA87" t="n">
-        <v>-11.46</v>
+        <v>-10.5</v>
       </c>
       <c r="AG87" t="b">
         <v>0</v>
@@ -6633,7 +6633,7 @@
         <v>5</v>
       </c>
       <c r="AA88" t="n">
-        <v>-3.81</v>
+        <v>-4.84</v>
       </c>
       <c r="AG88" t="b">
         <v>0</v>
@@ -6702,7 +6702,7 @@
         <v>5</v>
       </c>
       <c r="AA89" t="n">
-        <v>4.61</v>
+        <v>4.2</v>
       </c>
       <c r="AG89" t="b">
         <v>0</v>
@@ -6833,7 +6833,7 @@
         <v>5</v>
       </c>
       <c r="AA91" t="n">
-        <v>0</v>
+        <v>0.95</v>
       </c>
       <c r="AG91" t="b">
         <v>0</v>
@@ -12005,12 +12005,12 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>1102</t>
+          <t>1101</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>亞泥</t>
+          <t>台泥</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -12019,10 +12019,10 @@
         </is>
       </c>
       <c r="E153" t="n">
-        <v>73.31</v>
+        <v>79.08</v>
       </c>
       <c r="F153" t="n">
-        <v>36.03</v>
+        <v>40.69</v>
       </c>
       <c r="G153" t="inlineStr">
         <is>
@@ -12038,40 +12038,40 @@
         <v>0</v>
       </c>
       <c r="J153" t="n">
-        <v>3.3</v>
+        <v>3.83</v>
       </c>
       <c r="K153" t="n">
-        <v>36</v>
+        <v>25.75</v>
       </c>
       <c r="L153" t="inlineStr">
         <is>
-          <t>measured_move_target_up</t>
+          <t>gap_MM_Target_Up</t>
         </is>
       </c>
       <c r="M153" t="n">
-        <v>0.47</v>
+        <v>0.89</v>
       </c>
       <c r="N153" t="n">
-        <v>8.5</v>
+        <v>10</v>
       </c>
       <c r="O153" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="P153" t="n">
-        <v>33.22</v>
+        <v>24.27</v>
       </c>
       <c r="Q153" t="n">
-        <v>63.56</v>
+        <v>57.96</v>
       </c>
       <c r="R153" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="S153" t="n">
-        <v>7</v>
+        <v>4.3115</v>
       </c>
       <c r="T153" t="inlineStr">
         <is>
@@ -12084,13 +12084,13 @@
         </is>
       </c>
       <c r="V153" t="n">
-        <v>34.85</v>
+        <v>24.8</v>
       </c>
       <c r="W153" t="n">
-        <v>39.1688</v>
+        <v>27.0889</v>
       </c>
       <c r="X153" t="n">
-        <v>32.4105</v>
+        <v>23.7308</v>
       </c>
       <c r="Y153" t="inlineStr">
         <is>
@@ -12120,12 +12120,12 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2049</t>
+          <t>1102</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>上銀</t>
+          <t>亞泥</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -12134,10 +12134,10 @@
         </is>
       </c>
       <c r="E154" t="n">
-        <v>76.09</v>
+        <v>79.06999999999999</v>
       </c>
       <c r="F154" t="n">
-        <v>48.61</v>
+        <v>36.73</v>
       </c>
       <c r="G154" t="inlineStr">
         <is>
@@ -12146,17 +12146,17 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>WaitPullback</t>
+          <t>Reject</t>
         </is>
       </c>
       <c r="I154" t="b">
         <v>0</v>
       </c>
       <c r="J154" t="n">
-        <v>10</v>
+        <v>3.75</v>
       </c>
       <c r="K154" t="n">
-        <v>427.35</v>
+        <v>36</v>
       </c>
       <c r="L154" t="inlineStr">
         <is>
@@ -12164,10 +12164,10 @@
         </is>
       </c>
       <c r="M154" t="n">
-        <v>1.43</v>
+        <v>0.54</v>
       </c>
       <c r="N154" t="n">
-        <v>2.5</v>
+        <v>8.5</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -12175,10 +12175,10 @@
         </is>
       </c>
       <c r="P154" t="n">
-        <v>372.5</v>
+        <v>33.25</v>
       </c>
       <c r="Q154" t="n">
-        <v>60.7</v>
+        <v>68.17</v>
       </c>
       <c r="R154" t="inlineStr">
         <is>
@@ -12195,17 +12195,17 @@
       </c>
       <c r="U154" t="inlineStr">
         <is>
-          <t>industrial</t>
+          <t>materials</t>
         </is>
       </c>
       <c r="V154" t="n">
-        <v>388.5</v>
+        <v>34.7</v>
       </c>
       <c r="W154" t="n">
-        <v>466.2</v>
+        <v>39.0431</v>
       </c>
       <c r="X154" t="n">
-        <v>361.305</v>
+        <v>32.271</v>
       </c>
       <c r="Y154" t="inlineStr">
         <is>
@@ -12235,12 +12235,12 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2301</t>
+          <t>1216</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>光寶科</t>
+          <t>統一</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -12249,10 +12249,10 @@
         </is>
       </c>
       <c r="E155" t="n">
-        <v>72.55</v>
+        <v>74.12</v>
       </c>
       <c r="F155" t="n">
-        <v>45.83</v>
+        <v>42.35</v>
       </c>
       <c r="G155" t="inlineStr">
         <is>
@@ -12261,47 +12261,47 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>WaitPullback</t>
+          <t>Reject</t>
         </is>
       </c>
       <c r="I155" t="b">
         <v>0</v>
       </c>
       <c r="J155" t="n">
-        <v>10</v>
+        <v>1.39</v>
       </c>
       <c r="K155" t="n">
-        <v>298.1</v>
+        <v>79.29000000000001</v>
       </c>
       <c r="L155" t="inlineStr">
         <is>
-          <t>measured_move_target_up</t>
+          <t>gap_MM_Target_Up</t>
         </is>
       </c>
       <c r="M155" t="n">
-        <v>1.43</v>
+        <v>0.21</v>
       </c>
       <c r="N155" t="n">
-        <v>4.5</v>
+        <v>8.5</v>
       </c>
       <c r="O155" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="P155" t="n">
-        <v>262.83</v>
+        <v>75.34999999999999</v>
       </c>
       <c r="Q155" t="n">
-        <v>48.84</v>
+        <v>65.65000000000001</v>
       </c>
       <c r="R155" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="S155" t="n">
-        <v>7</v>
+        <v>6.4802</v>
       </c>
       <c r="T155" t="inlineStr">
         <is>
@@ -12310,17 +12310,17 @@
       </c>
       <c r="U155" t="inlineStr">
         <is>
-          <t>ai_hardware</t>
+          <t>unclassified</t>
         </is>
       </c>
       <c r="V155" t="n">
-        <v>271</v>
+        <v>78.2</v>
       </c>
       <c r="W155" t="n">
-        <v>325.2</v>
+        <v>86.5274</v>
       </c>
       <c r="X155" t="n">
-        <v>252.03</v>
+        <v>73.13249999999999</v>
       </c>
       <c r="Y155" t="inlineStr">
         <is>
@@ -12350,12 +12350,12 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2395</t>
+          <t>1402</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>研華</t>
+          <t>遠東新</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -12364,10 +12364,10 @@
         </is>
       </c>
       <c r="E156" t="n">
-        <v>70.29000000000001</v>
+        <v>76.83</v>
       </c>
       <c r="F156" t="n">
-        <v>47.11</v>
+        <v>50.2</v>
       </c>
       <c r="G156" t="inlineStr">
         <is>
@@ -12383,21 +12383,21 @@
         <v>0</v>
       </c>
       <c r="J156" t="n">
-        <v>10</v>
+        <v>9.76</v>
       </c>
       <c r="K156" t="n">
-        <v>750.2</v>
+        <v>32.05</v>
       </c>
       <c r="L156" t="inlineStr">
         <is>
-          <t>measured_move_target_up</t>
+          <t>wedge_failure_measured_move_target</t>
         </is>
       </c>
       <c r="M156" t="n">
-        <v>1.43</v>
+        <v>1.39</v>
       </c>
       <c r="N156" t="n">
-        <v>5</v>
+        <v>8.5</v>
       </c>
       <c r="O156" t="inlineStr">
         <is>
@@ -12405,14 +12405,14 @@
         </is>
       </c>
       <c r="P156" t="n">
-        <v>649.5</v>
+        <v>28.03</v>
       </c>
       <c r="Q156" t="n">
-        <v>54.08</v>
+        <v>64.68000000000001</v>
       </c>
       <c r="R156" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="S156" t="n">
@@ -12425,17 +12425,17 @@
       </c>
       <c r="U156" t="inlineStr">
         <is>
-          <t>ai_hardware</t>
+          <t>unclassified</t>
         </is>
       </c>
       <c r="V156" t="n">
-        <v>682</v>
+        <v>29.2</v>
       </c>
       <c r="W156" t="n">
-        <v>818.4</v>
+        <v>33.2614</v>
       </c>
       <c r="X156" t="n">
-        <v>634.26</v>
+        <v>27.156</v>
       </c>
       <c r="Y156" t="inlineStr">
         <is>
@@ -12465,12 +12465,12 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2408</t>
+          <t>1519</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>南亞科</t>
+          <t>華城</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -12479,10 +12479,10 @@
         </is>
       </c>
       <c r="E157" t="n">
-        <v>73.59</v>
+        <v>78.98999999999999</v>
       </c>
       <c r="F157" t="n">
-        <v>42.65</v>
+        <v>55.46</v>
       </c>
       <c r="G157" t="inlineStr">
         <is>
@@ -12501,7 +12501,7 @@
         <v>10</v>
       </c>
       <c r="K157" t="n">
-        <v>572</v>
+        <v>799.7</v>
       </c>
       <c r="L157" t="inlineStr">
         <is>
@@ -12512,22 +12512,22 @@
         <v>1.43</v>
       </c>
       <c r="N157" t="n">
-        <v>2.5</v>
+        <v>6.5</v>
       </c>
       <c r="O157" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="P157" t="n">
-        <v>494.5</v>
+        <v>693</v>
       </c>
       <c r="Q157" t="n">
-        <v>54.36</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="R157" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="S157" t="n">
@@ -12540,17 +12540,17 @@
       </c>
       <c r="U157" t="inlineStr">
         <is>
-          <t>semiconductor</t>
+          <t>industrial</t>
         </is>
       </c>
       <c r="V157" t="n">
-        <v>520</v>
+        <v>727</v>
       </c>
       <c r="W157" t="n">
-        <v>624</v>
+        <v>872.4</v>
       </c>
       <c r="X157" t="n">
-        <v>483.6</v>
+        <v>676.11</v>
       </c>
       <c r="Y157" t="inlineStr">
         <is>
@@ -12580,12 +12580,12 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2603</t>
+          <t>2049</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>長榮</t>
+          <t>上銀</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -12594,10 +12594,10 @@
         </is>
       </c>
       <c r="E158" t="n">
-        <v>77.81999999999999</v>
+        <v>79.54000000000001</v>
       </c>
       <c r="F158" t="n">
-        <v>40.03</v>
+        <v>51.68</v>
       </c>
       <c r="G158" t="inlineStr">
         <is>
@@ -12613,40 +12613,40 @@
         <v>0</v>
       </c>
       <c r="J158" t="n">
-        <v>9.24</v>
+        <v>8.32</v>
       </c>
       <c r="K158" t="n">
-        <v>266</v>
+        <v>397</v>
       </c>
       <c r="L158" t="inlineStr">
         <is>
-          <t>measured_move_target_up</t>
+          <t>gap_MM_Target_Up</t>
         </is>
       </c>
       <c r="M158" t="n">
-        <v>1.32</v>
+        <v>1.67</v>
       </c>
       <c r="N158" t="n">
-        <v>4.5</v>
+        <v>10</v>
       </c>
       <c r="O158" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="P158" t="n">
-        <v>225.5</v>
+        <v>372.5</v>
       </c>
       <c r="Q158" t="n">
-        <v>70.2</v>
+        <v>44.52</v>
       </c>
       <c r="R158" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="S158" t="n">
-        <v>7</v>
+        <v>4.9795</v>
       </c>
       <c r="T158" t="inlineStr">
         <is>
@@ -12655,17 +12655,17 @@
       </c>
       <c r="U158" t="inlineStr">
         <is>
-          <t>shipping</t>
+          <t>industrial</t>
         </is>
       </c>
       <c r="V158" t="n">
-        <v>243.5</v>
+        <v>366.5</v>
       </c>
       <c r="W158" t="n">
-        <v>292.2</v>
+        <v>439.8</v>
       </c>
       <c r="X158" t="n">
-        <v>226.455</v>
+        <v>348.25</v>
       </c>
       <c r="Y158" t="inlineStr">
         <is>
@@ -12695,12 +12695,12 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2609</t>
+          <t>2301</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>陽明</t>
+          <t>光寶科</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -12709,10 +12709,10 @@
         </is>
       </c>
       <c r="E159" t="n">
-        <v>76.16</v>
+        <v>72.55</v>
       </c>
       <c r="F159" t="n">
-        <v>25.69</v>
+        <v>45.83</v>
       </c>
       <c r="G159" t="inlineStr">
         <is>
@@ -12721,17 +12721,17 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>Reject</t>
+          <t>WaitPullback</t>
         </is>
       </c>
       <c r="I159" t="b">
         <v>0</v>
       </c>
       <c r="J159" t="n">
-        <v>0.67</v>
+        <v>10</v>
       </c>
       <c r="K159" t="n">
-        <v>60.1</v>
+        <v>298.1</v>
       </c>
       <c r="L159" t="inlineStr">
         <is>
@@ -12739,7 +12739,7 @@
         </is>
       </c>
       <c r="M159" t="n">
-        <v>0.1</v>
+        <v>1.43</v>
       </c>
       <c r="N159" t="n">
         <v>4.5</v>
@@ -12750,14 +12750,14 @@
         </is>
       </c>
       <c r="P159" t="n">
-        <v>55.3</v>
+        <v>262.83</v>
       </c>
       <c r="Q159" t="n">
-        <v>67.93000000000001</v>
+        <v>48.84</v>
       </c>
       <c r="R159" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="S159" t="n">
@@ -12770,17 +12770,17 @@
       </c>
       <c r="U159" t="inlineStr">
         <is>
-          <t>shipping</t>
+          <t>ai_hardware</t>
         </is>
       </c>
       <c r="V159" t="n">
-        <v>59.7</v>
+        <v>271</v>
       </c>
       <c r="W159" t="n">
-        <v>71.64</v>
+        <v>325.2</v>
       </c>
       <c r="X159" t="n">
-        <v>55.521</v>
+        <v>252.03</v>
       </c>
       <c r="Y159" t="inlineStr">
         <is>
@@ -12810,12 +12810,12 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2615</t>
+          <t>2383</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>萬海</t>
+          <t>台光電</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -12824,10 +12824,10 @@
         </is>
       </c>
       <c r="E160" t="n">
-        <v>84.39</v>
+        <v>75.29000000000001</v>
       </c>
       <c r="F160" t="n">
-        <v>39.6</v>
+        <v>49.32</v>
       </c>
       <c r="G160" t="inlineStr">
         <is>
@@ -12843,10 +12843,10 @@
         <v>0</v>
       </c>
       <c r="J160" t="n">
-        <v>8.890000000000001</v>
+        <v>10</v>
       </c>
       <c r="K160" t="n">
-        <v>117.6</v>
+        <v>6583.5</v>
       </c>
       <c r="L160" t="inlineStr">
         <is>
@@ -12854,7 +12854,7 @@
         </is>
       </c>
       <c r="M160" t="n">
-        <v>1.27</v>
+        <v>1.43</v>
       </c>
       <c r="N160" t="n">
         <v>4.5</v>
@@ -12865,14 +12865,14 @@
         </is>
       </c>
       <c r="P160" t="n">
-        <v>96.40000000000001</v>
+        <v>5787.5</v>
       </c>
       <c r="Q160" t="n">
-        <v>80.68000000000001</v>
+        <v>65.48</v>
       </c>
       <c r="R160" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="S160" t="n">
@@ -12885,17 +12885,17 @@
       </c>
       <c r="U160" t="inlineStr">
         <is>
-          <t>shipping</t>
+          <t>electronic_components</t>
         </is>
       </c>
       <c r="V160" t="n">
-        <v>108</v>
+        <v>5985</v>
       </c>
       <c r="W160" t="n">
-        <v>129.6</v>
+        <v>7182</v>
       </c>
       <c r="X160" t="n">
-        <v>100.44</v>
+        <v>5566.05</v>
       </c>
       <c r="Y160" t="inlineStr">
         <is>
@@ -12925,12 +12925,12 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>3008</t>
+          <t>2395</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>大立光</t>
+          <t>研華</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -12939,10 +12939,10 @@
         </is>
       </c>
       <c r="E161" t="n">
-        <v>77.73</v>
+        <v>70.29000000000001</v>
       </c>
       <c r="F161" t="n">
-        <v>42.98</v>
+        <v>47.11</v>
       </c>
       <c r="G161" t="inlineStr">
         <is>
@@ -12961,7 +12961,7 @@
         <v>10</v>
       </c>
       <c r="K161" t="n">
-        <v>6028</v>
+        <v>750.2</v>
       </c>
       <c r="L161" t="inlineStr">
         <is>
@@ -12972,22 +12972,22 @@
         <v>1.43</v>
       </c>
       <c r="N161" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="O161" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="P161" t="n">
-        <v>4955.86</v>
+        <v>649.5</v>
       </c>
       <c r="Q161" t="n">
-        <v>69.89</v>
+        <v>54.08</v>
       </c>
       <c r="R161" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="S161" t="n">
@@ -13000,17 +13000,17 @@
       </c>
       <c r="U161" t="inlineStr">
         <is>
-          <t>electronic_components</t>
+          <t>ai_hardware</t>
         </is>
       </c>
       <c r="V161" t="n">
-        <v>5480</v>
+        <v>682</v>
       </c>
       <c r="W161" t="n">
-        <v>6576</v>
+        <v>818.4</v>
       </c>
       <c r="X161" t="n">
-        <v>5096.4</v>
+        <v>634.26</v>
       </c>
       <c r="Y161" t="inlineStr">
         <is>
@@ -13040,12 +13040,12 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>3037</t>
+          <t>2408</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>欣興</t>
+          <t>南亞科</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -13054,10 +13054,10 @@
         </is>
       </c>
       <c r="E162" t="n">
-        <v>70.59</v>
+        <v>75.48999999999999</v>
       </c>
       <c r="F162" t="n">
-        <v>43.04</v>
+        <v>43.38</v>
       </c>
       <c r="G162" t="inlineStr">
         <is>
@@ -13076,7 +13076,7 @@
         <v>10</v>
       </c>
       <c r="K162" t="n">
-        <v>1210</v>
+        <v>568.7</v>
       </c>
       <c r="L162" t="inlineStr">
         <is>
@@ -13087,7 +13087,7 @@
         <v>1.43</v>
       </c>
       <c r="N162" t="n">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="O162" t="inlineStr">
         <is>
@@ -13095,14 +13095,14 @@
         </is>
       </c>
       <c r="P162" t="n">
-        <v>1064</v>
+        <v>494.5</v>
       </c>
       <c r="Q162" t="n">
-        <v>60.28</v>
+        <v>59.2</v>
       </c>
       <c r="R162" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="S162" t="n">
@@ -13115,17 +13115,17 @@
       </c>
       <c r="U162" t="inlineStr">
         <is>
-          <t>electronic_components</t>
+          <t>semiconductor</t>
         </is>
       </c>
       <c r="V162" t="n">
-        <v>1100</v>
+        <v>517</v>
       </c>
       <c r="W162" t="n">
-        <v>1320</v>
+        <v>620.4</v>
       </c>
       <c r="X162" t="n">
-        <v>1023</v>
+        <v>480.81</v>
       </c>
       <c r="Y162" t="inlineStr">
         <is>
@@ -13155,115 +13155,1031 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
+          <t>2603</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>長榮</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E163" t="n">
+        <v>77.81999999999999</v>
+      </c>
+      <c r="F163" t="n">
+        <v>40.03</v>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I163" t="b">
+        <v>0</v>
+      </c>
+      <c r="J163" t="n">
+        <v>9.24</v>
+      </c>
+      <c r="K163" t="n">
+        <v>266</v>
+      </c>
+      <c r="L163" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M163" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="N163" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="O163" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P163" t="n">
+        <v>225.5</v>
+      </c>
+      <c r="Q163" t="n">
+        <v>70.2</v>
+      </c>
+      <c r="R163" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="S163" t="n">
+        <v>7</v>
+      </c>
+      <c r="T163" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U163" t="inlineStr">
+        <is>
+          <t>shipping</t>
+        </is>
+      </c>
+      <c r="V163" t="n">
+        <v>243.5</v>
+      </c>
+      <c r="W163" t="n">
+        <v>292.2</v>
+      </c>
+      <c r="X163" t="n">
+        <v>226.455</v>
+      </c>
+      <c r="Y163" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z163" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG163" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH163" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI163" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>2609</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>陽明</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E164" t="n">
+        <v>76.16</v>
+      </c>
+      <c r="F164" t="n">
+        <v>25.69</v>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>Reject</t>
+        </is>
+      </c>
+      <c r="I164" t="b">
+        <v>0</v>
+      </c>
+      <c r="J164" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="K164" t="n">
+        <v>60.1</v>
+      </c>
+      <c r="L164" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M164" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="N164" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="O164" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P164" t="n">
+        <v>55.3</v>
+      </c>
+      <c r="Q164" t="n">
+        <v>67.93000000000001</v>
+      </c>
+      <c r="R164" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="S164" t="n">
+        <v>7</v>
+      </c>
+      <c r="T164" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U164" t="inlineStr">
+        <is>
+          <t>shipping</t>
+        </is>
+      </c>
+      <c r="V164" t="n">
+        <v>59.7</v>
+      </c>
+      <c r="W164" t="n">
+        <v>71.64</v>
+      </c>
+      <c r="X164" t="n">
+        <v>55.521</v>
+      </c>
+      <c r="Y164" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z164" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG164" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH164" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI164" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>2615</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>萬海</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E165" t="n">
+        <v>84.39</v>
+      </c>
+      <c r="F165" t="n">
+        <v>39.6</v>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I165" t="b">
+        <v>0</v>
+      </c>
+      <c r="J165" t="n">
+        <v>8.890000000000001</v>
+      </c>
+      <c r="K165" t="n">
+        <v>117.6</v>
+      </c>
+      <c r="L165" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M165" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="N165" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="O165" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P165" t="n">
+        <v>96.40000000000001</v>
+      </c>
+      <c r="Q165" t="n">
+        <v>80.68000000000001</v>
+      </c>
+      <c r="R165" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="S165" t="n">
+        <v>7</v>
+      </c>
+      <c r="T165" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U165" t="inlineStr">
+        <is>
+          <t>shipping</t>
+        </is>
+      </c>
+      <c r="V165" t="n">
+        <v>108</v>
+      </c>
+      <c r="W165" t="n">
+        <v>129.6</v>
+      </c>
+      <c r="X165" t="n">
+        <v>100.44</v>
+      </c>
+      <c r="Y165" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z165" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG165" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH165" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI165" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>3008</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>大立光</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E166" t="n">
+        <v>81.23</v>
+      </c>
+      <c r="F166" t="n">
+        <v>42.23</v>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I166" t="b">
+        <v>0</v>
+      </c>
+      <c r="J166" t="n">
+        <v>10</v>
+      </c>
+      <c r="K166" t="n">
+        <v>6066.5</v>
+      </c>
+      <c r="L166" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M166" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N166" t="n">
+        <v>3</v>
+      </c>
+      <c r="O166" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P166" t="n">
+        <v>4955.86</v>
+      </c>
+      <c r="Q166" t="n">
+        <v>74.89</v>
+      </c>
+      <c r="R166" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="S166" t="n">
+        <v>7</v>
+      </c>
+      <c r="T166" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U166" t="inlineStr">
+        <is>
+          <t>electronic_components</t>
+        </is>
+      </c>
+      <c r="V166" t="n">
+        <v>5515</v>
+      </c>
+      <c r="W166" t="n">
+        <v>6618</v>
+      </c>
+      <c r="X166" t="n">
+        <v>5128.95</v>
+      </c>
+      <c r="Y166" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z166" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG166" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH166" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI166" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>3037</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>欣興</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E167" t="n">
+        <v>78.62</v>
+      </c>
+      <c r="F167" t="n">
+        <v>44.31</v>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I167" t="b">
+        <v>0</v>
+      </c>
+      <c r="J167" t="n">
+        <v>10</v>
+      </c>
+      <c r="K167" t="n">
+        <v>1254</v>
+      </c>
+      <c r="L167" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M167" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N167" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="O167" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P167" t="n">
+        <v>1064</v>
+      </c>
+      <c r="Q167" t="n">
+        <v>65.40000000000001</v>
+      </c>
+      <c r="R167" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="S167" t="n">
+        <v>7</v>
+      </c>
+      <c r="T167" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U167" t="inlineStr">
+        <is>
+          <t>electronic_components</t>
+        </is>
+      </c>
+      <c r="V167" t="n">
+        <v>1140</v>
+      </c>
+      <c r="W167" t="n">
+        <v>1368</v>
+      </c>
+      <c r="X167" t="n">
+        <v>1060.2</v>
+      </c>
+      <c r="Y167" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z167" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG167" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH167" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI167" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>3081</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>聯亞</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E168" t="n">
+        <v>77.04000000000001</v>
+      </c>
+      <c r="F168" t="n">
+        <v>46.13</v>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I168" t="b">
+        <v>0</v>
+      </c>
+      <c r="J168" t="n">
+        <v>10</v>
+      </c>
+      <c r="K168" t="n">
+        <v>3058</v>
+      </c>
+      <c r="L168" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M168" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N168" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="O168" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P168" t="n">
+        <v>2612.5</v>
+      </c>
+      <c r="Q168" t="n">
+        <v>50.86</v>
+      </c>
+      <c r="R168" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S168" t="n">
+        <v>7</v>
+      </c>
+      <c r="T168" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U168" t="inlineStr">
+        <is>
+          <t>unclassified</t>
+        </is>
+      </c>
+      <c r="V168" t="n">
+        <v>2780</v>
+      </c>
+      <c r="W168" t="n">
+        <v>3336</v>
+      </c>
+      <c r="X168" t="n">
+        <v>2585.4</v>
+      </c>
+      <c r="Y168" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="AI168" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="AJ168" t="inlineStr">
+        <is>
+          <t>market_data_temporarily_unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>3189</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>景碩</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E169" t="n">
+        <v>72.84999999999999</v>
+      </c>
+      <c r="F169" t="n">
+        <v>54.7</v>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I169" t="b">
+        <v>0</v>
+      </c>
+      <c r="J169" t="n">
+        <v>10</v>
+      </c>
+      <c r="K169" t="n">
+        <v>936.1</v>
+      </c>
+      <c r="L169" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M169" t="n">
+        <v>1.77</v>
+      </c>
+      <c r="N169" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="O169" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="P169" t="n">
+        <v>869</v>
+      </c>
+      <c r="Q169" t="n">
+        <v>41.32</v>
+      </c>
+      <c r="R169" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S169" t="n">
+        <v>5.6445</v>
+      </c>
+      <c r="T169" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U169" t="inlineStr">
+        <is>
+          <t>unclassified</t>
+        </is>
+      </c>
+      <c r="V169" t="n">
+        <v>851</v>
+      </c>
+      <c r="W169" t="n">
+        <v>1021.2</v>
+      </c>
+      <c r="X169" t="n">
+        <v>802.965</v>
+      </c>
+      <c r="Y169" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z169" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG169" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH169" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI169" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>3443</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>創意</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E170" t="n">
+        <v>78.89</v>
+      </c>
+      <c r="F170" t="n">
+        <v>43.48</v>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I170" t="b">
+        <v>0</v>
+      </c>
+      <c r="J170" t="n">
+        <v>10</v>
+      </c>
+      <c r="K170" t="n">
+        <v>6193</v>
+      </c>
+      <c r="L170" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M170" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N170" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="O170" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P170" t="n">
+        <v>5120</v>
+      </c>
+      <c r="Q170" t="n">
+        <v>59.84</v>
+      </c>
+      <c r="R170" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S170" t="n">
+        <v>7</v>
+      </c>
+      <c r="T170" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U170" t="inlineStr">
+        <is>
+          <t>semiconductor</t>
+        </is>
+      </c>
+      <c r="V170" t="n">
+        <v>5630</v>
+      </c>
+      <c r="W170" t="n">
+        <v>6756</v>
+      </c>
+      <c r="X170" t="n">
+        <v>5235.9</v>
+      </c>
+      <c r="Y170" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z170" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG170" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH170" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI170" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
           <t>6669</t>
         </is>
       </c>
-      <c r="C163" t="inlineStr">
+      <c r="C171" t="inlineStr">
         <is>
           <t>緯穎</t>
         </is>
       </c>
-      <c r="D163" t="inlineStr">
-        <is>
-          <t>swing_accumulation_ready</t>
-        </is>
-      </c>
-      <c r="E163" t="n">
-        <v>74.44</v>
-      </c>
-      <c r="F163" t="n">
-        <v>54.53</v>
-      </c>
-      <c r="G163" t="inlineStr">
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E171" t="n">
+        <v>74.25</v>
+      </c>
+      <c r="F171" t="n">
+        <v>53.42</v>
+      </c>
+      <c r="G171" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H163" t="inlineStr">
+      <c r="H171" t="inlineStr">
         <is>
           <t>WaitPullback</t>
         </is>
       </c>
-      <c r="I163" t="b">
-        <v>0</v>
-      </c>
-      <c r="J163" t="n">
+      <c r="I171" t="b">
+        <v>0</v>
+      </c>
+      <c r="J171" t="n">
         <v>10</v>
       </c>
-      <c r="K163" t="n">
-        <v>6990.5</v>
-      </c>
-      <c r="L163" t="inlineStr">
+      <c r="K171" t="n">
+        <v>6957.5</v>
+      </c>
+      <c r="L171" t="inlineStr">
         <is>
           <t>measured_move_target_up</t>
         </is>
       </c>
-      <c r="M163" t="n">
+      <c r="M171" t="n">
         <v>1.43</v>
       </c>
-      <c r="N163" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="O163" t="inlineStr">
+      <c r="N171" t="n">
+        <v>7</v>
+      </c>
+      <c r="O171" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="P163" t="n">
+      <c r="P171" t="n">
         <v>6297.5</v>
       </c>
-      <c r="Q163" t="n">
-        <v>53.52</v>
-      </c>
-      <c r="R163" t="inlineStr">
+      <c r="Q171" t="n">
+        <v>56.16</v>
+      </c>
+      <c r="R171" t="inlineStr">
         <is>
           <t>Weak</t>
         </is>
       </c>
-      <c r="S163" t="n">
-        <v>7</v>
-      </c>
-      <c r="T163" t="inlineStr">
-        <is>
-          <t>RangeRotation</t>
-        </is>
-      </c>
-      <c r="U163" t="inlineStr">
+      <c r="S171" t="n">
+        <v>7</v>
+      </c>
+      <c r="T171" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U171" t="inlineStr">
         <is>
           <t>semiconductor</t>
         </is>
       </c>
-      <c r="V163" t="n">
-        <v>6355</v>
-      </c>
-      <c r="W163" t="n">
-        <v>7626</v>
-      </c>
-      <c r="X163" t="n">
-        <v>5910.15</v>
-      </c>
-      <c r="Y163" t="inlineStr">
-        <is>
-          <t>Tracking</t>
-        </is>
-      </c>
-      <c r="Z163" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG163" t="b">
-        <v>0</v>
-      </c>
-      <c r="AH163" t="b">
-        <v>0</v>
-      </c>
-      <c r="AI163" t="inlineStr">
+      <c r="V171" t="n">
+        <v>6325</v>
+      </c>
+      <c r="W171" t="n">
+        <v>7590</v>
+      </c>
+      <c r="X171" t="n">
+        <v>5882.25</v>
+      </c>
+      <c r="Y171" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z171" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG171" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH171" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI171" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AJ163"/>
+  <autoFilter ref="A1:AJ171"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -13370,7 +14286,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -13458,10 +14374,20 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>Unknown</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13503,7 +14429,7 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>2026-08-20 09:51:49</t>
+          <t>2026-08-20 14:22:09</t>
         </is>
       </c>
     </row>
@@ -13550,7 +14476,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>162</v>
+        <v>170</v>
       </c>
     </row>
     <row r="7">
@@ -13570,7 +14496,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>162</v>
+        <v>170</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-08-21 06:24:02
</commit_message>
<xml_diff>
--- a/data/swing_performance_analysis.xlsx
+++ b/data/swing_performance_analysis.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'T20_Tracking'!$A$1:$AJ$171</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'T20_Tracking'!$A$1:$AJ$180</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ171"/>
+  <dimension ref="A1:AJ180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -731,13 +731,16 @@
         </is>
       </c>
       <c r="Z2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA2" t="n">
         <v>-1.45</v>
       </c>
+      <c r="AB2" t="n">
+        <v>10.36</v>
+      </c>
       <c r="AG2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH2" t="b">
         <v>0</v>
@@ -800,11 +803,14 @@
         </is>
       </c>
       <c r="Z3" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA3" t="n">
         <v>-5.5</v>
       </c>
+      <c r="AB3" t="n">
+        <v>-7.12</v>
+      </c>
       <c r="AG3" t="b">
         <v>0</v>
       </c>
@@ -869,11 +875,14 @@
         </is>
       </c>
       <c r="Z4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA4" t="n">
         <v>21.91</v>
       </c>
+      <c r="AB4" t="n">
+        <v>12.73</v>
+      </c>
       <c r="AG4" t="b">
         <v>1</v>
       </c>
@@ -938,11 +947,14 @@
         </is>
       </c>
       <c r="Z5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA5" t="n">
         <v>3.92</v>
       </c>
+      <c r="AB5" t="n">
+        <v>-7.52</v>
+      </c>
       <c r="AG5" t="b">
         <v>0</v>
       </c>
@@ -1007,11 +1019,14 @@
         </is>
       </c>
       <c r="Z6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA6" t="n">
         <v>7.73</v>
       </c>
+      <c r="AB6" t="n">
+        <v>2.37</v>
+      </c>
       <c r="AG6" t="b">
         <v>0</v>
       </c>
@@ -1076,11 +1091,14 @@
         </is>
       </c>
       <c r="Z7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA7" t="n">
         <v>5.54</v>
       </c>
+      <c r="AB7" t="n">
+        <v>21.2</v>
+      </c>
       <c r="AG7" t="b">
         <v>1</v>
       </c>
@@ -1145,11 +1163,14 @@
         </is>
       </c>
       <c r="Z8" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA8" t="n">
         <v>-11.56</v>
       </c>
+      <c r="AB8" t="n">
+        <v>-9.33</v>
+      </c>
       <c r="AG8" t="b">
         <v>0</v>
       </c>
@@ -1214,11 +1235,14 @@
         </is>
       </c>
       <c r="Z9" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA9" t="n">
         <v>-10.14</v>
       </c>
+      <c r="AB9" t="n">
+        <v>-4.05</v>
+      </c>
       <c r="AG9" t="b">
         <v>0</v>
       </c>
@@ -1283,11 +1307,14 @@
         </is>
       </c>
       <c r="Z10" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA10" t="n">
         <v>-12.27</v>
       </c>
+      <c r="AB10" t="n">
+        <v>-10.81</v>
+      </c>
       <c r="AG10" t="b">
         <v>0</v>
       </c>
@@ -1352,11 +1379,14 @@
         </is>
       </c>
       <c r="Z11" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA11" t="n">
         <v>-6.97</v>
       </c>
+      <c r="AB11" t="n">
+        <v>-7.76</v>
+      </c>
       <c r="AG11" t="b">
         <v>0</v>
       </c>
@@ -1421,11 +1451,14 @@
         </is>
       </c>
       <c r="Z12" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA12" t="n">
         <v>5.13</v>
       </c>
+      <c r="AB12" t="n">
+        <v>27.94</v>
+      </c>
       <c r="AG12" t="b">
         <v>1</v>
       </c>
@@ -1490,11 +1523,14 @@
         </is>
       </c>
       <c r="Z13" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA13" t="n">
         <v>-5.54</v>
       </c>
+      <c r="AB13" t="n">
+        <v>-2.21</v>
+      </c>
       <c r="AG13" t="b">
         <v>0</v>
       </c>
@@ -1621,11 +1657,14 @@
         </is>
       </c>
       <c r="Z15" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA15" t="n">
         <v>3.09</v>
       </c>
+      <c r="AB15" t="n">
+        <v>8.66</v>
+      </c>
       <c r="AG15" t="b">
         <v>0</v>
       </c>
@@ -1690,11 +1729,14 @@
         </is>
       </c>
       <c r="Z16" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA16" t="n">
         <v>9.31</v>
       </c>
+      <c r="AB16" t="n">
+        <v>16.34</v>
+      </c>
       <c r="AG16" t="b">
         <v>1</v>
       </c>
@@ -1759,7 +1801,7 @@
         </is>
       </c>
       <c r="Z17" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA17" t="n">
         <v>-1.43</v>
@@ -1828,7 +1870,7 @@
         </is>
       </c>
       <c r="Z18" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA18" t="n">
         <v>-6.69</v>
@@ -1897,7 +1939,7 @@
         </is>
       </c>
       <c r="Z19" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA19" t="n">
         <v>-4.07</v>
@@ -1966,7 +2008,7 @@
         </is>
       </c>
       <c r="Z20" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA20" t="n">
         <v>-1.42</v>
@@ -2035,7 +2077,7 @@
         </is>
       </c>
       <c r="Z21" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA21" t="n">
         <v>-3.59</v>
@@ -2104,7 +2146,7 @@
         </is>
       </c>
       <c r="Z22" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA22" t="n">
         <v>14.67</v>
@@ -2173,7 +2215,7 @@
         </is>
       </c>
       <c r="Z23" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA23" t="n">
         <v>2.43</v>
@@ -2242,7 +2284,7 @@
         </is>
       </c>
       <c r="Z24" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA24" t="n">
         <v>1.05</v>
@@ -2311,7 +2353,7 @@
         </is>
       </c>
       <c r="Z25" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA25" t="n">
         <v>8.18</v>
@@ -2380,7 +2422,7 @@
         </is>
       </c>
       <c r="Z26" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA26" t="n">
         <v>6.01</v>
@@ -2449,7 +2491,7 @@
         </is>
       </c>
       <c r="Z27" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA27" t="n">
         <v>13.83</v>
@@ -2518,7 +2560,7 @@
         </is>
       </c>
       <c r="Z28" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA28" t="n">
         <v>-10.91</v>
@@ -2587,7 +2629,7 @@
         </is>
       </c>
       <c r="Z29" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA29" t="n">
         <v>-2.87</v>
@@ -2656,7 +2698,7 @@
         </is>
       </c>
       <c r="Z30" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA30" t="n">
         <v>-8.630000000000001</v>
@@ -2725,7 +2767,7 @@
         </is>
       </c>
       <c r="Z31" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA31" t="n">
         <v>-0.91</v>
@@ -2794,7 +2836,7 @@
         </is>
       </c>
       <c r="Z32" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA32" t="n">
         <v>-6.43</v>
@@ -2863,7 +2905,7 @@
         </is>
       </c>
       <c r="Z33" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA33" t="n">
         <v>-3.11</v>
@@ -3056,7 +3098,7 @@
         </is>
       </c>
       <c r="Z36" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA36" t="n">
         <v>-3.48</v>
@@ -3125,7 +3167,7 @@
         </is>
       </c>
       <c r="Z37" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA37" t="n">
         <v>10.15</v>
@@ -3194,7 +3236,7 @@
         </is>
       </c>
       <c r="Z38" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA38" t="n">
         <v>-5.23</v>
@@ -3263,7 +3305,7 @@
         </is>
       </c>
       <c r="Z39" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA39" t="n">
         <v>-5.13</v>
@@ -3332,7 +3374,7 @@
         </is>
       </c>
       <c r="Z40" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA40" t="n">
         <v>-3.13</v>
@@ -3401,7 +3443,7 @@
         </is>
       </c>
       <c r="Z41" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA41" t="n">
         <v>-4.05</v>
@@ -3470,7 +3512,7 @@
         </is>
       </c>
       <c r="Z42" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA42" t="n">
         <v>1.86</v>
@@ -3539,7 +3581,7 @@
         </is>
       </c>
       <c r="Z43" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA43" t="n">
         <v>8.460000000000001</v>
@@ -3608,7 +3650,7 @@
         </is>
       </c>
       <c r="Z44" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA44" t="n">
         <v>10.82</v>
@@ -3677,7 +3719,7 @@
         </is>
       </c>
       <c r="Z45" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA45" t="n">
         <v>-0.71</v>
@@ -3746,7 +3788,7 @@
         </is>
       </c>
       <c r="Z46" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA46" t="n">
         <v>12.1</v>
@@ -3815,7 +3857,7 @@
         </is>
       </c>
       <c r="Z47" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA47" t="n">
         <v>2.72</v>
@@ -3884,7 +3926,7 @@
         </is>
       </c>
       <c r="Z48" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA48" t="n">
         <v>5.32</v>
@@ -3953,7 +3995,7 @@
         </is>
       </c>
       <c r="Z49" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA49" t="n">
         <v>-3.36</v>
@@ -4022,13 +4064,13 @@
         </is>
       </c>
       <c r="Z50" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA50" t="n">
         <v>9.17</v>
       </c>
       <c r="AG50" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH50" t="b">
         <v>0</v>
@@ -4091,7 +4133,7 @@
         </is>
       </c>
       <c r="Z51" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA51" t="n">
         <v>8.08</v>
@@ -4160,7 +4202,7 @@
         </is>
       </c>
       <c r="Z52" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA52" t="n">
         <v>20.55</v>
@@ -4229,7 +4271,7 @@
         </is>
       </c>
       <c r="Z53" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA53" t="n">
         <v>-0.32</v>
@@ -4298,7 +4340,7 @@
         </is>
       </c>
       <c r="Z54" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA54" t="n">
         <v>-5.24</v>
@@ -4429,7 +4471,7 @@
         </is>
       </c>
       <c r="Z56" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA56" t="n">
         <v>-4.49</v>
@@ -4498,7 +4540,7 @@
         </is>
       </c>
       <c r="Z57" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA57" t="n">
         <v>-0.28</v>
@@ -4567,7 +4609,7 @@
         </is>
       </c>
       <c r="Z58" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA58" t="n">
         <v>-8.779999999999999</v>
@@ -4636,7 +4678,7 @@
         </is>
       </c>
       <c r="Z59" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA59" t="n">
         <v>-4.05</v>
@@ -4705,7 +4747,7 @@
         </is>
       </c>
       <c r="Z60" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA60" t="n">
         <v>-9.26</v>
@@ -4774,7 +4816,7 @@
         </is>
       </c>
       <c r="Z61" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA61" t="n">
         <v>8.57</v>
@@ -4843,7 +4885,7 @@
         </is>
       </c>
       <c r="Z62" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA62" t="n">
         <v>-3.42</v>
@@ -4912,7 +4954,7 @@
         </is>
       </c>
       <c r="Z63" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA63" t="n">
         <v>2.62</v>
@@ -4981,7 +5023,7 @@
         </is>
       </c>
       <c r="Z64" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA64" t="n">
         <v>1.17</v>
@@ -5050,7 +5092,7 @@
         </is>
       </c>
       <c r="Z65" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA65" t="n">
         <v>12.12</v>
@@ -5119,7 +5161,7 @@
         </is>
       </c>
       <c r="Z66" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA66" t="n">
         <v>-1.13</v>
@@ -5188,7 +5230,7 @@
         </is>
       </c>
       <c r="Z67" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA67" t="n">
         <v>21.05</v>
@@ -5257,7 +5299,7 @@
         </is>
       </c>
       <c r="Z68" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA68" t="n">
         <v>6.36</v>
@@ -5326,7 +5368,7 @@
         </is>
       </c>
       <c r="Z69" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA69" t="n">
         <v>-5.94</v>
@@ -5457,7 +5499,7 @@
         </is>
       </c>
       <c r="Z71" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA71" t="n">
         <v>3.22</v>
@@ -5526,7 +5568,7 @@
         </is>
       </c>
       <c r="Z72" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA72" t="n">
         <v>-2.78</v>
@@ -5595,7 +5637,7 @@
         </is>
       </c>
       <c r="Z73" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA73" t="n">
         <v>5.81</v>
@@ -5664,7 +5706,7 @@
         </is>
       </c>
       <c r="Z74" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA74" t="n">
         <v>-5.04</v>
@@ -5733,7 +5775,7 @@
         </is>
       </c>
       <c r="Z75" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA75" t="n">
         <v>0.97</v>
@@ -5802,7 +5844,7 @@
         </is>
       </c>
       <c r="Z76" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA76" t="n">
         <v>-3.4</v>
@@ -5871,7 +5913,7 @@
         </is>
       </c>
       <c r="Z77" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA77" t="n">
         <v>-0.93</v>
@@ -5940,7 +5982,7 @@
         </is>
       </c>
       <c r="Z78" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA78" t="n">
         <v>-12.58</v>
@@ -6009,7 +6051,7 @@
         </is>
       </c>
       <c r="Z79" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA79" t="n">
         <v>-3.58</v>
@@ -6018,7 +6060,7 @@
         <v>0</v>
       </c>
       <c r="AH79" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI79" t="inlineStr">
         <is>
@@ -6078,7 +6120,7 @@
         </is>
       </c>
       <c r="Z80" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA80" t="n">
         <v>0.58</v>
@@ -6147,7 +6189,7 @@
         </is>
       </c>
       <c r="Z81" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA81" t="n">
         <v>14.15</v>
@@ -6216,7 +6258,7 @@
         </is>
       </c>
       <c r="Z82" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA82" t="n">
         <v>29.71</v>
@@ -6285,7 +6327,7 @@
         </is>
       </c>
       <c r="Z83" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA83" t="n">
         <v>-1.5</v>
@@ -6354,7 +6396,7 @@
         </is>
       </c>
       <c r="Z84" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA84" t="n">
         <v>18.35</v>
@@ -6423,7 +6465,7 @@
         </is>
       </c>
       <c r="Z85" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA85" t="n">
         <v>-8.630000000000001</v>
@@ -6492,7 +6534,7 @@
         </is>
       </c>
       <c r="Z86" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA86" t="n">
         <v>1.62</v>
@@ -6561,7 +6603,7 @@
         </is>
       </c>
       <c r="Z87" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA87" t="n">
         <v>-10.5</v>
@@ -6630,7 +6672,7 @@
         </is>
       </c>
       <c r="Z88" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA88" t="n">
         <v>-4.84</v>
@@ -6699,7 +6741,7 @@
         </is>
       </c>
       <c r="Z89" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA89" t="n">
         <v>4.2</v>
@@ -6830,7 +6872,7 @@
         </is>
       </c>
       <c r="Z91" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA91" t="n">
         <v>0.95</v>
@@ -6899,7 +6941,10 @@
         </is>
       </c>
       <c r="Z92" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA92" t="n">
+        <v>1.83</v>
       </c>
       <c r="AG92" t="b">
         <v>0</v>
@@ -6965,7 +7010,10 @@
         </is>
       </c>
       <c r="Z93" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA93" t="n">
+        <v>-1.71</v>
       </c>
       <c r="AG93" t="b">
         <v>0</v>
@@ -7031,7 +7079,10 @@
         </is>
       </c>
       <c r="Z94" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA94" t="n">
+        <v>-2.25</v>
       </c>
       <c r="AG94" t="b">
         <v>0</v>
@@ -7097,7 +7148,10 @@
         </is>
       </c>
       <c r="Z95" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA95" t="n">
+        <v>-14.59</v>
       </c>
       <c r="AG95" t="b">
         <v>0</v>
@@ -7163,7 +7217,10 @@
         </is>
       </c>
       <c r="Z96" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA96" t="n">
+        <v>-11.01</v>
       </c>
       <c r="AG96" t="b">
         <v>0</v>
@@ -7229,13 +7286,16 @@
         </is>
       </c>
       <c r="Z97" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA97" t="n">
+        <v>-7.87</v>
       </c>
       <c r="AG97" t="b">
         <v>0</v>
       </c>
       <c r="AH97" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI97" t="inlineStr">
         <is>
@@ -7295,7 +7355,10 @@
         </is>
       </c>
       <c r="Z98" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA98" t="n">
+        <v>3.12</v>
       </c>
       <c r="AG98" t="b">
         <v>0</v>
@@ -7361,7 +7424,10 @@
         </is>
       </c>
       <c r="Z99" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA99" t="n">
+        <v>-9.98</v>
       </c>
       <c r="AG99" t="b">
         <v>0</v>
@@ -7427,10 +7493,13 @@
         </is>
       </c>
       <c r="Z100" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA100" t="n">
+        <v>14.84</v>
       </c>
       <c r="AG100" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH100" t="b">
         <v>0</v>
@@ -7493,7 +7562,10 @@
         </is>
       </c>
       <c r="Z101" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA101" t="n">
+        <v>24.03</v>
       </c>
       <c r="AG101" t="b">
         <v>1</v>
@@ -7559,7 +7631,10 @@
         </is>
       </c>
       <c r="Z102" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA102" t="n">
+        <v>37.42</v>
       </c>
       <c r="AG102" t="b">
         <v>1</v>
@@ -7625,7 +7700,10 @@
         </is>
       </c>
       <c r="Z103" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA103" t="n">
+        <v>-0.32</v>
       </c>
       <c r="AG103" t="b">
         <v>0</v>
@@ -7691,7 +7769,10 @@
         </is>
       </c>
       <c r="Z104" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA104" t="n">
+        <v>-1.32</v>
       </c>
       <c r="AG104" t="b">
         <v>0</v>
@@ -7757,7 +7838,10 @@
         </is>
       </c>
       <c r="Z105" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA105" t="n">
+        <v>21.69</v>
       </c>
       <c r="AG105" t="b">
         <v>1</v>
@@ -7823,7 +7907,10 @@
         </is>
       </c>
       <c r="Z106" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA106" t="n">
+        <v>-11.44</v>
       </c>
       <c r="AG106" t="b">
         <v>0</v>
@@ -7889,7 +7976,10 @@
         </is>
       </c>
       <c r="Z107" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA107" t="n">
+        <v>6.37</v>
       </c>
       <c r="AG107" t="b">
         <v>0</v>
@@ -7955,13 +8045,16 @@
         </is>
       </c>
       <c r="Z108" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA108" t="n">
+        <v>-5.92</v>
       </c>
       <c r="AG108" t="b">
         <v>0</v>
       </c>
       <c r="AH108" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI108" t="inlineStr">
         <is>
@@ -8021,7 +8114,10 @@
         </is>
       </c>
       <c r="Z109" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA109" t="n">
+        <v>-9.300000000000001</v>
       </c>
       <c r="AG109" t="b">
         <v>0</v>
@@ -8087,7 +8183,10 @@
         </is>
       </c>
       <c r="Z110" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA110" t="n">
+        <v>2.47</v>
       </c>
       <c r="AG110" t="b">
         <v>0</v>
@@ -8153,7 +8252,10 @@
         </is>
       </c>
       <c r="Z111" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA111" t="n">
+        <v>-6.67</v>
       </c>
       <c r="AG111" t="b">
         <v>0</v>
@@ -8219,7 +8321,10 @@
         </is>
       </c>
       <c r="Z112" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA112" t="n">
+        <v>-2.8</v>
       </c>
       <c r="AG112" t="b">
         <v>0</v>
@@ -8285,7 +8390,7 @@
         </is>
       </c>
       <c r="Z113" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG113" t="b">
         <v>0</v>
@@ -8351,7 +8456,7 @@
         </is>
       </c>
       <c r="Z114" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG114" t="b">
         <v>0</v>
@@ -8417,7 +8522,7 @@
         </is>
       </c>
       <c r="Z115" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG115" t="b">
         <v>0</v>
@@ -8483,7 +8588,7 @@
         </is>
       </c>
       <c r="Z116" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG116" t="b">
         <v>0</v>
@@ -8549,7 +8654,7 @@
         </is>
       </c>
       <c r="Z117" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG117" t="b">
         <v>0</v>
@@ -8615,7 +8720,7 @@
         </is>
       </c>
       <c r="Z118" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG118" t="b">
         <v>0</v>
@@ -8681,7 +8786,7 @@
         </is>
       </c>
       <c r="Z119" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG119" t="b">
         <v>0</v>
@@ -8747,7 +8852,7 @@
         </is>
       </c>
       <c r="Z120" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG120" t="b">
         <v>0</v>
@@ -8813,7 +8918,7 @@
         </is>
       </c>
       <c r="Z121" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG121" t="b">
         <v>0</v>
@@ -8879,10 +8984,10 @@
         </is>
       </c>
       <c r="Z122" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG122" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH122" t="b">
         <v>0</v>
@@ -8945,7 +9050,7 @@
         </is>
       </c>
       <c r="Z123" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG123" t="b">
         <v>0</v>
@@ -9011,7 +9116,7 @@
         </is>
       </c>
       <c r="Z124" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG124" t="b">
         <v>0</v>
@@ -9077,7 +9182,7 @@
         </is>
       </c>
       <c r="Z125" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG125" t="b">
         <v>0</v>
@@ -9143,7 +9248,7 @@
         </is>
       </c>
       <c r="Z126" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG126" t="b">
         <v>0</v>
@@ -9209,7 +9314,7 @@
         </is>
       </c>
       <c r="Z127" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG127" t="b">
         <v>0</v>
@@ -9275,7 +9380,7 @@
         </is>
       </c>
       <c r="Z128" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG128" t="b">
         <v>0</v>
@@ -9341,7 +9446,7 @@
         </is>
       </c>
       <c r="Z129" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG129" t="b">
         <v>0</v>
@@ -9456,7 +9561,7 @@
         </is>
       </c>
       <c r="Z130" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG130" t="b">
         <v>0</v>
@@ -9571,13 +9676,13 @@
         </is>
       </c>
       <c r="Z131" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG131" t="b">
         <v>0</v>
       </c>
       <c r="AH131" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI131" t="inlineStr">
         <is>
@@ -9686,7 +9791,7 @@
         </is>
       </c>
       <c r="Z132" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG132" t="b">
         <v>0</v>
@@ -9801,13 +9906,13 @@
         </is>
       </c>
       <c r="Z133" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG133" t="b">
         <v>0</v>
       </c>
       <c r="AH133" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI133" t="inlineStr">
         <is>
@@ -9916,13 +10021,13 @@
         </is>
       </c>
       <c r="Z134" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG134" t="b">
         <v>0</v>
       </c>
       <c r="AH134" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI134" t="inlineStr">
         <is>
@@ -10031,7 +10136,7 @@
         </is>
       </c>
       <c r="Z135" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG135" t="b">
         <v>0</v>
@@ -10146,7 +10251,7 @@
         </is>
       </c>
       <c r="Z136" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG136" t="b">
         <v>0</v>
@@ -10258,7 +10363,7 @@
         </is>
       </c>
       <c r="Z137" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG137" t="b">
         <v>0</v>
@@ -10373,7 +10478,7 @@
         </is>
       </c>
       <c r="Z138" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG138" t="b">
         <v>0</v>
@@ -10488,7 +10593,7 @@
         </is>
       </c>
       <c r="Z139" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG139" t="b">
         <v>0</v>
@@ -10603,7 +10708,7 @@
         </is>
       </c>
       <c r="Z140" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG140" t="b">
         <v>0</v>
@@ -10718,13 +10823,13 @@
         </is>
       </c>
       <c r="Z141" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG141" t="b">
         <v>0</v>
       </c>
       <c r="AH141" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI141" t="inlineStr">
         <is>
@@ -10833,13 +10938,13 @@
         </is>
       </c>
       <c r="Z142" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG142" t="b">
         <v>0</v>
       </c>
       <c r="AH142" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI142" t="inlineStr">
         <is>
@@ -10948,7 +11053,7 @@
         </is>
       </c>
       <c r="Z143" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG143" t="b">
         <v>0</v>
@@ -11063,7 +11168,7 @@
         </is>
       </c>
       <c r="Z144" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG144" t="b">
         <v>0</v>
@@ -11178,7 +11283,7 @@
         </is>
       </c>
       <c r="Z145" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG145" t="b">
         <v>0</v>
@@ -11293,7 +11398,7 @@
         </is>
       </c>
       <c r="Z146" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG146" t="b">
         <v>0</v>
@@ -11408,7 +11513,7 @@
         </is>
       </c>
       <c r="Z147" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG147" t="b">
         <v>0</v>
@@ -11523,7 +11628,7 @@
         </is>
       </c>
       <c r="Z148" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG148" t="b">
         <v>0</v>
@@ -11638,13 +11743,13 @@
         </is>
       </c>
       <c r="Z149" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG149" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH149" t="b">
         <v>1</v>
-      </c>
-      <c r="AG149" t="b">
-        <v>0</v>
-      </c>
-      <c r="AH149" t="b">
-        <v>0</v>
       </c>
       <c r="AI149" t="inlineStr">
         <is>
@@ -11753,7 +11858,7 @@
         </is>
       </c>
       <c r="Z150" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG150" t="b">
         <v>0</v>
@@ -11868,7 +11973,7 @@
         </is>
       </c>
       <c r="Z151" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG151" t="b">
         <v>0</v>
@@ -11983,13 +12088,13 @@
         </is>
       </c>
       <c r="Z152" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG152" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH152" t="b">
         <v>1</v>
-      </c>
-      <c r="AG152" t="b">
-        <v>0</v>
-      </c>
-      <c r="AH152" t="b">
-        <v>0</v>
       </c>
       <c r="AI152" t="inlineStr">
         <is>
@@ -12098,7 +12203,7 @@
         </is>
       </c>
       <c r="Z153" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG153" t="b">
         <v>0</v>
@@ -12213,7 +12318,7 @@
         </is>
       </c>
       <c r="Z154" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG154" t="b">
         <v>0</v>
@@ -12328,7 +12433,7 @@
         </is>
       </c>
       <c r="Z155" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG155" t="b">
         <v>0</v>
@@ -12443,7 +12548,7 @@
         </is>
       </c>
       <c r="Z156" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG156" t="b">
         <v>0</v>
@@ -12558,7 +12663,7 @@
         </is>
       </c>
       <c r="Z157" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG157" t="b">
         <v>0</v>
@@ -12673,13 +12778,13 @@
         </is>
       </c>
       <c r="Z158" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG158" t="b">
         <v>0</v>
       </c>
       <c r="AH158" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI158" t="inlineStr">
         <is>
@@ -12788,13 +12893,13 @@
         </is>
       </c>
       <c r="Z159" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG159" t="b">
         <v>0</v>
       </c>
       <c r="AH159" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI159" t="inlineStr">
         <is>
@@ -12903,7 +13008,7 @@
         </is>
       </c>
       <c r="Z160" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG160" t="b">
         <v>0</v>
@@ -13018,7 +13123,7 @@
         </is>
       </c>
       <c r="Z161" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG161" t="b">
         <v>0</v>
@@ -13133,7 +13238,7 @@
         </is>
       </c>
       <c r="Z162" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG162" t="b">
         <v>0</v>
@@ -13248,7 +13353,7 @@
         </is>
       </c>
       <c r="Z163" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG163" t="b">
         <v>0</v>
@@ -13363,7 +13468,7 @@
         </is>
       </c>
       <c r="Z164" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG164" t="b">
         <v>0</v>
@@ -13478,7 +13583,7 @@
         </is>
       </c>
       <c r="Z165" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG165" t="b">
         <v>0</v>
@@ -13593,7 +13698,7 @@
         </is>
       </c>
       <c r="Z166" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG166" t="b">
         <v>0</v>
@@ -13708,13 +13813,13 @@
         </is>
       </c>
       <c r="Z167" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG167" t="b">
         <v>0</v>
       </c>
       <c r="AH167" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI167" t="inlineStr">
         <is>
@@ -13934,13 +14039,13 @@
         </is>
       </c>
       <c r="Z169" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG169" t="b">
         <v>0</v>
       </c>
       <c r="AH169" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI169" t="inlineStr">
         <is>
@@ -14049,7 +14154,7 @@
         </is>
       </c>
       <c r="Z170" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG170" t="b">
         <v>0</v>
@@ -14164,7 +14269,7 @@
         </is>
       </c>
       <c r="Z171" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG171" t="b">
         <v>0</v>
@@ -14178,8 +14283,1039 @@
         </is>
       </c>
     </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>1101</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>台泥</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E172" t="n">
+        <v>72.77</v>
+      </c>
+      <c r="F172" t="n">
+        <v>41.95</v>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>Reject</t>
+        </is>
+      </c>
+      <c r="I172" t="b">
+        <v>0</v>
+      </c>
+      <c r="J172" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="K172" t="n">
+        <v>25.75</v>
+      </c>
+      <c r="L172" t="inlineStr">
+        <is>
+          <t>gap_MM_Target_Up</t>
+        </is>
+      </c>
+      <c r="M172" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="N172" t="n">
+        <v>10</v>
+      </c>
+      <c r="O172" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="P172" t="n">
+        <v>24.43</v>
+      </c>
+      <c r="Q172" t="n">
+        <v>52.98</v>
+      </c>
+      <c r="R172" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S172" t="n">
+        <v>4.504</v>
+      </c>
+      <c r="T172" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U172" t="inlineStr">
+        <is>
+          <t>materials</t>
+        </is>
+      </c>
+      <c r="V172" t="n">
+        <v>24.85</v>
+      </c>
+      <c r="W172" t="n">
+        <v>27.108</v>
+      </c>
+      <c r="X172" t="n">
+        <v>23.7308</v>
+      </c>
+      <c r="Y172" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z172" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG172" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH172" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI172" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>1102</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>亞泥</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>swing_buy_confirmed</t>
+        </is>
+      </c>
+      <c r="E173" t="n">
+        <v>80.47</v>
+      </c>
+      <c r="F173" t="n">
+        <v>42.38</v>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>Reject</t>
+        </is>
+      </c>
+      <c r="I173" t="b">
+        <v>0</v>
+      </c>
+      <c r="J173" t="n">
+        <v>3</v>
+      </c>
+      <c r="K173" t="n">
+        <v>36</v>
+      </c>
+      <c r="L173" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M173" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="N173" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="O173" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="P173" t="n">
+        <v>33.32</v>
+      </c>
+      <c r="Q173" t="n">
+        <v>79.17</v>
+      </c>
+      <c r="R173" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="S173" t="n">
+        <v>7</v>
+      </c>
+      <c r="T173" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U173" t="inlineStr">
+        <is>
+          <t>materials</t>
+        </is>
+      </c>
+      <c r="V173" t="n">
+        <v>34.95</v>
+      </c>
+      <c r="W173" t="n">
+        <v>39.0268</v>
+      </c>
+      <c r="X173" t="n">
+        <v>32.5035</v>
+      </c>
+      <c r="Y173" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z173" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG173" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH173" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI173" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>1402</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>遠東新</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E174" t="n">
+        <v>76.19</v>
+      </c>
+      <c r="F174" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I174" t="b">
+        <v>0</v>
+      </c>
+      <c r="J174" t="n">
+        <v>10.02</v>
+      </c>
+      <c r="K174" t="n">
+        <v>33.39</v>
+      </c>
+      <c r="L174" t="inlineStr">
+        <is>
+          <t>gap_MM_Target_Up</t>
+        </is>
+      </c>
+      <c r="M174" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N174" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="O174" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="P174" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="Q174" t="n">
+        <v>73.31999999999999</v>
+      </c>
+      <c r="R174" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="S174" t="n">
+        <v>7</v>
+      </c>
+      <c r="T174" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U174" t="inlineStr">
+        <is>
+          <t>unclassified</t>
+        </is>
+      </c>
+      <c r="V174" t="n">
+        <v>30.35</v>
+      </c>
+      <c r="W174" t="n">
+        <v>35.5963</v>
+      </c>
+      <c r="X174" t="n">
+        <v>28.2255</v>
+      </c>
+      <c r="Y174" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z174" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG174" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH174" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI174" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>2408</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>南亞科</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E175" t="n">
+        <v>75.04000000000001</v>
+      </c>
+      <c r="F175" t="n">
+        <v>44.37</v>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I175" t="b">
+        <v>0</v>
+      </c>
+      <c r="J175" t="n">
+        <v>10</v>
+      </c>
+      <c r="K175" t="n">
+        <v>580.8</v>
+      </c>
+      <c r="L175" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M175" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N175" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="O175" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P175" t="n">
+        <v>494.5</v>
+      </c>
+      <c r="Q175" t="n">
+        <v>52.48</v>
+      </c>
+      <c r="R175" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S175" t="n">
+        <v>7</v>
+      </c>
+      <c r="T175" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U175" t="inlineStr">
+        <is>
+          <t>semiconductor</t>
+        </is>
+      </c>
+      <c r="V175" t="n">
+        <v>528</v>
+      </c>
+      <c r="W175" t="n">
+        <v>633.6</v>
+      </c>
+      <c r="X175" t="n">
+        <v>491.04</v>
+      </c>
+      <c r="Y175" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z175" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG175" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH175" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI175" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>2881</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>富邦金</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E176" t="n">
+        <v>74.78</v>
+      </c>
+      <c r="F176" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>Reject</t>
+        </is>
+      </c>
+      <c r="I176" t="b">
+        <v>0</v>
+      </c>
+      <c r="J176" t="n">
+        <v>7.84</v>
+      </c>
+      <c r="K176" t="n">
+        <v>144.5</v>
+      </c>
+      <c r="L176" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M176" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="N176" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="O176" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="P176" t="n">
+        <v>129.5</v>
+      </c>
+      <c r="Q176" t="n">
+        <v>62.7</v>
+      </c>
+      <c r="R176" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="S176" t="n">
+        <v>7</v>
+      </c>
+      <c r="T176" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U176" t="inlineStr">
+        <is>
+          <t>finance</t>
+        </is>
+      </c>
+      <c r="V176" t="n">
+        <v>134</v>
+      </c>
+      <c r="W176" t="n">
+        <v>151.2218</v>
+      </c>
+      <c r="X176" t="n">
+        <v>124.62</v>
+      </c>
+      <c r="Y176" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z176" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG176" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH176" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI176" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>2887</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>台新金</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E177" t="n">
+        <v>75.45</v>
+      </c>
+      <c r="F177" t="n">
+        <v>52.96</v>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I177" t="b">
+        <v>0</v>
+      </c>
+      <c r="J177" t="n">
+        <v>10.01</v>
+      </c>
+      <c r="K177" t="n">
+        <v>40.98</v>
+      </c>
+      <c r="L177" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M177" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N177" t="n">
+        <v>7</v>
+      </c>
+      <c r="O177" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="P177" t="n">
+        <v>36.15</v>
+      </c>
+      <c r="Q177" t="n">
+        <v>53.08</v>
+      </c>
+      <c r="R177" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S177" t="n">
+        <v>7</v>
+      </c>
+      <c r="T177" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U177" t="inlineStr">
+        <is>
+          <t>finance</t>
+        </is>
+      </c>
+      <c r="V177" t="n">
+        <v>37.25</v>
+      </c>
+      <c r="W177" t="n">
+        <v>42.8264</v>
+      </c>
+      <c r="X177" t="n">
+        <v>34.6425</v>
+      </c>
+      <c r="Y177" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z177" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG177" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH177" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI177" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>3008</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>大立光</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E178" t="n">
+        <v>86.58</v>
+      </c>
+      <c r="F178" t="n">
+        <v>44.17</v>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I178" t="b">
+        <v>0</v>
+      </c>
+      <c r="J178" t="n">
+        <v>10</v>
+      </c>
+      <c r="K178" t="n">
+        <v>6171</v>
+      </c>
+      <c r="L178" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M178" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N178" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="O178" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P178" t="n">
+        <v>4970.86</v>
+      </c>
+      <c r="Q178" t="n">
+        <v>77.81999999999999</v>
+      </c>
+      <c r="R178" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="S178" t="n">
+        <v>7</v>
+      </c>
+      <c r="T178" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U178" t="inlineStr">
+        <is>
+          <t>electronic_components</t>
+        </is>
+      </c>
+      <c r="V178" t="n">
+        <v>5610</v>
+      </c>
+      <c r="W178" t="n">
+        <v>6732</v>
+      </c>
+      <c r="X178" t="n">
+        <v>5217.3</v>
+      </c>
+      <c r="Y178" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z178" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG178" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH178" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI178" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>3081</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>聯亞</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E179" t="n">
+        <v>74.95</v>
+      </c>
+      <c r="F179" t="n">
+        <v>40.15</v>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I179" t="b">
+        <v>0</v>
+      </c>
+      <c r="J179" t="n">
+        <v>10</v>
+      </c>
+      <c r="K179" t="n">
+        <v>3212</v>
+      </c>
+      <c r="L179" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M179" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N179" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="O179" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P179" t="n">
+        <v>2622.5</v>
+      </c>
+      <c r="Q179" t="n">
+        <v>57.68</v>
+      </c>
+      <c r="R179" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S179" t="n">
+        <v>7</v>
+      </c>
+      <c r="T179" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U179" t="inlineStr">
+        <is>
+          <t>unclassified</t>
+        </is>
+      </c>
+      <c r="V179" t="n">
+        <v>2920</v>
+      </c>
+      <c r="W179" t="n">
+        <v>3504</v>
+      </c>
+      <c r="X179" t="n">
+        <v>2715.6</v>
+      </c>
+      <c r="Y179" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="AI179" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="AJ179" t="inlineStr">
+        <is>
+          <t>market_data_temporarily_unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>3443</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>創意</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E180" t="n">
+        <v>74.23999999999999</v>
+      </c>
+      <c r="F180" t="n">
+        <v>42.95</v>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I180" t="b">
+        <v>0</v>
+      </c>
+      <c r="J180" t="n">
+        <v>10</v>
+      </c>
+      <c r="K180" t="n">
+        <v>6160</v>
+      </c>
+      <c r="L180" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M180" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N180" t="n">
+        <v>3</v>
+      </c>
+      <c r="O180" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P180" t="n">
+        <v>5120</v>
+      </c>
+      <c r="Q180" t="n">
+        <v>53</v>
+      </c>
+      <c r="R180" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S180" t="n">
+        <v>7</v>
+      </c>
+      <c r="T180" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U180" t="inlineStr">
+        <is>
+          <t>semiconductor</t>
+        </is>
+      </c>
+      <c r="V180" t="n">
+        <v>5600</v>
+      </c>
+      <c r="W180" t="n">
+        <v>6720</v>
+      </c>
+      <c r="X180" t="n">
+        <v>5208</v>
+      </c>
+      <c r="Y180" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z180" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG180" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH180" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI180" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AJ171"/>
+  <autoFilter ref="A1:AJ180"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -14429,7 +15565,7 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>2026-08-20 14:22:09</t>
+          <t>2026-08-21 14:23:57</t>
         </is>
       </c>
     </row>
@@ -14476,7 +15612,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>170</v>
+        <v>179</v>
       </c>
     </row>
     <row r="7">
@@ -14496,7 +15632,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>170</v>
+        <v>179</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-08-24 06:50:53
</commit_message>
<xml_diff>
--- a/data/swing_performance_analysis.xlsx
+++ b/data/swing_performance_analysis.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'T20_Tracking'!$A$1:$AJ$180</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'T20_Tracking'!$A$1:$AJ$186</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ180"/>
+  <dimension ref="A1:AJ186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -731,7 +731,7 @@
         </is>
       </c>
       <c r="Z2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA2" t="n">
         <v>-1.45</v>
@@ -803,7 +803,7 @@
         </is>
       </c>
       <c r="Z3" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA3" t="n">
         <v>-5.5</v>
@@ -875,7 +875,7 @@
         </is>
       </c>
       <c r="Z4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA4" t="n">
         <v>21.91</v>
@@ -947,7 +947,7 @@
         </is>
       </c>
       <c r="Z5" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA5" t="n">
         <v>3.92</v>
@@ -1019,7 +1019,7 @@
         </is>
       </c>
       <c r="Z6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA6" t="n">
         <v>7.73</v>
@@ -1091,7 +1091,7 @@
         </is>
       </c>
       <c r="Z7" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA7" t="n">
         <v>5.54</v>
@@ -1163,7 +1163,7 @@
         </is>
       </c>
       <c r="Z8" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA8" t="n">
         <v>-11.56</v>
@@ -1235,7 +1235,7 @@
         </is>
       </c>
       <c r="Z9" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA9" t="n">
         <v>-10.14</v>
@@ -1307,7 +1307,7 @@
         </is>
       </c>
       <c r="Z10" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA10" t="n">
         <v>-12.27</v>
@@ -1379,7 +1379,7 @@
         </is>
       </c>
       <c r="Z11" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA11" t="n">
         <v>-6.97</v>
@@ -1451,7 +1451,7 @@
         </is>
       </c>
       <c r="Z12" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA12" t="n">
         <v>5.13</v>
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="Z13" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA13" t="n">
         <v>-5.54</v>
@@ -1657,7 +1657,7 @@
         </is>
       </c>
       <c r="Z15" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA15" t="n">
         <v>3.09</v>
@@ -1729,7 +1729,7 @@
         </is>
       </c>
       <c r="Z16" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA16" t="n">
         <v>9.31</v>
@@ -1801,11 +1801,14 @@
         </is>
       </c>
       <c r="Z17" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA17" t="n">
         <v>-1.43</v>
       </c>
+      <c r="AB17" t="n">
+        <v>0.61</v>
+      </c>
       <c r="AG17" t="b">
         <v>0</v>
       </c>
@@ -1870,11 +1873,14 @@
         </is>
       </c>
       <c r="Z18" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA18" t="n">
         <v>-6.69</v>
       </c>
+      <c r="AB18" t="n">
+        <v>-8.6</v>
+      </c>
       <c r="AG18" t="b">
         <v>0</v>
       </c>
@@ -1939,11 +1945,14 @@
         </is>
       </c>
       <c r="Z19" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA19" t="n">
         <v>-4.07</v>
       </c>
+      <c r="AB19" t="n">
+        <v>-2.29</v>
+      </c>
       <c r="AG19" t="b">
         <v>0</v>
       </c>
@@ -2008,11 +2017,14 @@
         </is>
       </c>
       <c r="Z20" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA20" t="n">
         <v>-1.42</v>
       </c>
+      <c r="AB20" t="n">
+        <v>-11.24</v>
+      </c>
       <c r="AG20" t="b">
         <v>0</v>
       </c>
@@ -2077,11 +2089,14 @@
         </is>
       </c>
       <c r="Z21" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA21" t="n">
         <v>-3.59</v>
       </c>
+      <c r="AB21" t="n">
+        <v>-7.94</v>
+      </c>
       <c r="AG21" t="b">
         <v>0</v>
       </c>
@@ -2146,11 +2161,14 @@
         </is>
       </c>
       <c r="Z22" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA22" t="n">
         <v>14.67</v>
       </c>
+      <c r="AB22" t="n">
+        <v>12.84</v>
+      </c>
       <c r="AG22" t="b">
         <v>1</v>
       </c>
@@ -2215,11 +2233,14 @@
         </is>
       </c>
       <c r="Z23" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA23" t="n">
         <v>2.43</v>
       </c>
+      <c r="AB23" t="n">
+        <v>-2.43</v>
+      </c>
       <c r="AG23" t="b">
         <v>0</v>
       </c>
@@ -2284,11 +2305,14 @@
         </is>
       </c>
       <c r="Z24" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA24" t="n">
         <v>1.05</v>
       </c>
+      <c r="AB24" t="n">
+        <v>-1.35</v>
+      </c>
       <c r="AG24" t="b">
         <v>0</v>
       </c>
@@ -2353,11 +2377,14 @@
         </is>
       </c>
       <c r="Z25" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA25" t="n">
         <v>8.18</v>
       </c>
+      <c r="AB25" t="n">
+        <v>17.06</v>
+      </c>
       <c r="AG25" t="b">
         <v>1</v>
       </c>
@@ -2422,11 +2449,14 @@
         </is>
       </c>
       <c r="Z26" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA26" t="n">
         <v>6.01</v>
       </c>
+      <c r="AB26" t="n">
+        <v>25</v>
+      </c>
       <c r="AG26" t="b">
         <v>1</v>
       </c>
@@ -2491,11 +2521,14 @@
         </is>
       </c>
       <c r="Z27" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA27" t="n">
         <v>13.83</v>
       </c>
+      <c r="AB27" t="n">
+        <v>42.29</v>
+      </c>
       <c r="AG27" t="b">
         <v>1</v>
       </c>
@@ -2560,11 +2593,14 @@
         </is>
       </c>
       <c r="Z28" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA28" t="n">
         <v>-10.91</v>
       </c>
+      <c r="AB28" t="n">
+        <v>-10.8</v>
+      </c>
       <c r="AG28" t="b">
         <v>0</v>
       </c>
@@ -2629,11 +2665,14 @@
         </is>
       </c>
       <c r="Z29" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA29" t="n">
         <v>-2.87</v>
       </c>
+      <c r="AB29" t="n">
+        <v>-2.08</v>
+      </c>
       <c r="AG29" t="b">
         <v>0</v>
       </c>
@@ -2698,11 +2737,14 @@
         </is>
       </c>
       <c r="Z30" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA30" t="n">
         <v>-8.630000000000001</v>
       </c>
+      <c r="AB30" t="n">
+        <v>-8.140000000000001</v>
+      </c>
       <c r="AG30" t="b">
         <v>0</v>
       </c>
@@ -2767,11 +2809,14 @@
         </is>
       </c>
       <c r="Z31" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA31" t="n">
         <v>-0.91</v>
       </c>
+      <c r="AB31" t="n">
+        <v>2.36</v>
+      </c>
       <c r="AG31" t="b">
         <v>0</v>
       </c>
@@ -2836,11 +2881,14 @@
         </is>
       </c>
       <c r="Z32" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA32" t="n">
         <v>-6.43</v>
       </c>
+      <c r="AB32" t="n">
+        <v>-0.37</v>
+      </c>
       <c r="AG32" t="b">
         <v>0</v>
       </c>
@@ -2905,11 +2953,14 @@
         </is>
       </c>
       <c r="Z33" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA33" t="n">
         <v>-3.11</v>
       </c>
+      <c r="AB33" t="n">
+        <v>-9.07</v>
+      </c>
       <c r="AG33" t="b">
         <v>0</v>
       </c>
@@ -3098,11 +3149,14 @@
         </is>
       </c>
       <c r="Z36" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA36" t="n">
         <v>-3.48</v>
       </c>
+      <c r="AB36" t="n">
+        <v>5.1</v>
+      </c>
       <c r="AG36" t="b">
         <v>0</v>
       </c>
@@ -3167,11 +3221,14 @@
         </is>
       </c>
       <c r="Z37" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA37" t="n">
         <v>10.15</v>
       </c>
+      <c r="AB37" t="n">
+        <v>4.83</v>
+      </c>
       <c r="AG37" t="b">
         <v>0</v>
       </c>
@@ -3236,11 +3293,14 @@
         </is>
       </c>
       <c r="Z38" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA38" t="n">
         <v>-5.23</v>
       </c>
+      <c r="AB38" t="n">
+        <v>-1.74</v>
+      </c>
       <c r="AG38" t="b">
         <v>0</v>
       </c>
@@ -3305,7 +3365,7 @@
         </is>
       </c>
       <c r="Z39" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA39" t="n">
         <v>-5.13</v>
@@ -3374,7 +3434,7 @@
         </is>
       </c>
       <c r="Z40" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA40" t="n">
         <v>-3.13</v>
@@ -3443,7 +3503,7 @@
         </is>
       </c>
       <c r="Z41" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA41" t="n">
         <v>-4.05</v>
@@ -3512,7 +3572,7 @@
         </is>
       </c>
       <c r="Z42" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA42" t="n">
         <v>1.86</v>
@@ -3581,7 +3641,7 @@
         </is>
       </c>
       <c r="Z43" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA43" t="n">
         <v>8.460000000000001</v>
@@ -3650,7 +3710,7 @@
         </is>
       </c>
       <c r="Z44" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA44" t="n">
         <v>10.82</v>
@@ -3719,7 +3779,7 @@
         </is>
       </c>
       <c r="Z45" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA45" t="n">
         <v>-0.71</v>
@@ -3788,7 +3848,7 @@
         </is>
       </c>
       <c r="Z46" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA46" t="n">
         <v>12.1</v>
@@ -3857,7 +3917,7 @@
         </is>
       </c>
       <c r="Z47" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA47" t="n">
         <v>2.72</v>
@@ -3926,7 +3986,7 @@
         </is>
       </c>
       <c r="Z48" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA48" t="n">
         <v>5.32</v>
@@ -3995,7 +4055,7 @@
         </is>
       </c>
       <c r="Z49" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA49" t="n">
         <v>-3.36</v>
@@ -4064,7 +4124,7 @@
         </is>
       </c>
       <c r="Z50" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA50" t="n">
         <v>9.17</v>
@@ -4133,7 +4193,7 @@
         </is>
       </c>
       <c r="Z51" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA51" t="n">
         <v>8.08</v>
@@ -4202,7 +4262,7 @@
         </is>
       </c>
       <c r="Z52" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA52" t="n">
         <v>20.55</v>
@@ -4271,7 +4331,7 @@
         </is>
       </c>
       <c r="Z53" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA53" t="n">
         <v>-0.32</v>
@@ -4340,7 +4400,7 @@
         </is>
       </c>
       <c r="Z54" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA54" t="n">
         <v>-5.24</v>
@@ -4471,7 +4531,7 @@
         </is>
       </c>
       <c r="Z56" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA56" t="n">
         <v>-4.49</v>
@@ -4540,7 +4600,7 @@
         </is>
       </c>
       <c r="Z57" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA57" t="n">
         <v>-0.28</v>
@@ -4609,7 +4669,7 @@
         </is>
       </c>
       <c r="Z58" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA58" t="n">
         <v>-8.779999999999999</v>
@@ -4678,7 +4738,7 @@
         </is>
       </c>
       <c r="Z59" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA59" t="n">
         <v>-4.05</v>
@@ -4747,7 +4807,7 @@
         </is>
       </c>
       <c r="Z60" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA60" t="n">
         <v>-9.26</v>
@@ -4816,7 +4876,7 @@
         </is>
       </c>
       <c r="Z61" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA61" t="n">
         <v>8.57</v>
@@ -4885,7 +4945,7 @@
         </is>
       </c>
       <c r="Z62" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA62" t="n">
         <v>-3.42</v>
@@ -4954,7 +5014,7 @@
         </is>
       </c>
       <c r="Z63" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA63" t="n">
         <v>2.62</v>
@@ -5023,7 +5083,7 @@
         </is>
       </c>
       <c r="Z64" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA64" t="n">
         <v>1.17</v>
@@ -5092,7 +5152,7 @@
         </is>
       </c>
       <c r="Z65" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA65" t="n">
         <v>12.12</v>
@@ -5161,7 +5221,7 @@
         </is>
       </c>
       <c r="Z66" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA66" t="n">
         <v>-1.13</v>
@@ -5230,7 +5290,7 @@
         </is>
       </c>
       <c r="Z67" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA67" t="n">
         <v>21.05</v>
@@ -5299,7 +5359,7 @@
         </is>
       </c>
       <c r="Z68" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA68" t="n">
         <v>6.36</v>
@@ -5368,7 +5428,7 @@
         </is>
       </c>
       <c r="Z69" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA69" t="n">
         <v>-5.94</v>
@@ -5499,7 +5559,7 @@
         </is>
       </c>
       <c r="Z71" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA71" t="n">
         <v>3.22</v>
@@ -5568,7 +5628,7 @@
         </is>
       </c>
       <c r="Z72" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA72" t="n">
         <v>-2.78</v>
@@ -5637,7 +5697,7 @@
         </is>
       </c>
       <c r="Z73" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA73" t="n">
         <v>5.81</v>
@@ -5706,7 +5766,7 @@
         </is>
       </c>
       <c r="Z74" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA74" t="n">
         <v>-5.04</v>
@@ -5775,7 +5835,7 @@
         </is>
       </c>
       <c r="Z75" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA75" t="n">
         <v>0.97</v>
@@ -5844,7 +5904,7 @@
         </is>
       </c>
       <c r="Z76" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA76" t="n">
         <v>-3.4</v>
@@ -5913,7 +5973,7 @@
         </is>
       </c>
       <c r="Z77" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA77" t="n">
         <v>-0.93</v>
@@ -5982,7 +6042,7 @@
         </is>
       </c>
       <c r="Z78" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA78" t="n">
         <v>-12.58</v>
@@ -6051,7 +6111,7 @@
         </is>
       </c>
       <c r="Z79" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA79" t="n">
         <v>-3.58</v>
@@ -6120,7 +6180,7 @@
         </is>
       </c>
       <c r="Z80" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA80" t="n">
         <v>0.58</v>
@@ -6189,7 +6249,7 @@
         </is>
       </c>
       <c r="Z81" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA81" t="n">
         <v>14.15</v>
@@ -6258,7 +6318,7 @@
         </is>
       </c>
       <c r="Z82" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA82" t="n">
         <v>29.71</v>
@@ -6327,7 +6387,7 @@
         </is>
       </c>
       <c r="Z83" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA83" t="n">
         <v>-1.5</v>
@@ -6396,7 +6456,7 @@
         </is>
       </c>
       <c r="Z84" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA84" t="n">
         <v>18.35</v>
@@ -6465,7 +6525,7 @@
         </is>
       </c>
       <c r="Z85" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA85" t="n">
         <v>-8.630000000000001</v>
@@ -6534,7 +6594,7 @@
         </is>
       </c>
       <c r="Z86" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA86" t="n">
         <v>1.62</v>
@@ -6603,7 +6663,7 @@
         </is>
       </c>
       <c r="Z87" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA87" t="n">
         <v>-10.5</v>
@@ -6672,7 +6732,7 @@
         </is>
       </c>
       <c r="Z88" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA88" t="n">
         <v>-4.84</v>
@@ -6741,7 +6801,7 @@
         </is>
       </c>
       <c r="Z89" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA89" t="n">
         <v>4.2</v>
@@ -6872,7 +6932,7 @@
         </is>
       </c>
       <c r="Z91" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA91" t="n">
         <v>0.95</v>
@@ -6941,7 +7001,7 @@
         </is>
       </c>
       <c r="Z92" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA92" t="n">
         <v>1.83</v>
@@ -7010,7 +7070,7 @@
         </is>
       </c>
       <c r="Z93" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA93" t="n">
         <v>-1.71</v>
@@ -7079,7 +7139,7 @@
         </is>
       </c>
       <c r="Z94" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA94" t="n">
         <v>-2.25</v>
@@ -7148,7 +7208,7 @@
         </is>
       </c>
       <c r="Z95" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA95" t="n">
         <v>-14.59</v>
@@ -7217,7 +7277,7 @@
         </is>
       </c>
       <c r="Z96" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA96" t="n">
         <v>-11.01</v>
@@ -7286,7 +7346,7 @@
         </is>
       </c>
       <c r="Z97" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA97" t="n">
         <v>-7.87</v>
@@ -7355,7 +7415,7 @@
         </is>
       </c>
       <c r="Z98" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA98" t="n">
         <v>3.12</v>
@@ -7424,7 +7484,7 @@
         </is>
       </c>
       <c r="Z99" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA99" t="n">
         <v>-9.98</v>
@@ -7493,7 +7553,7 @@
         </is>
       </c>
       <c r="Z100" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA100" t="n">
         <v>14.84</v>
@@ -7562,7 +7622,7 @@
         </is>
       </c>
       <c r="Z101" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA101" t="n">
         <v>24.03</v>
@@ -7631,7 +7691,7 @@
         </is>
       </c>
       <c r="Z102" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA102" t="n">
         <v>37.42</v>
@@ -7700,7 +7760,7 @@
         </is>
       </c>
       <c r="Z103" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA103" t="n">
         <v>-0.32</v>
@@ -7769,7 +7829,7 @@
         </is>
       </c>
       <c r="Z104" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA104" t="n">
         <v>-1.32</v>
@@ -7838,7 +7898,7 @@
         </is>
       </c>
       <c r="Z105" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA105" t="n">
         <v>21.69</v>
@@ -7907,7 +7967,7 @@
         </is>
       </c>
       <c r="Z106" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA106" t="n">
         <v>-11.44</v>
@@ -7976,7 +8036,7 @@
         </is>
       </c>
       <c r="Z107" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA107" t="n">
         <v>6.37</v>
@@ -8045,7 +8105,7 @@
         </is>
       </c>
       <c r="Z108" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA108" t="n">
         <v>-5.92</v>
@@ -8114,7 +8174,7 @@
         </is>
       </c>
       <c r="Z109" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA109" t="n">
         <v>-9.300000000000001</v>
@@ -8183,7 +8243,7 @@
         </is>
       </c>
       <c r="Z110" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA110" t="n">
         <v>2.47</v>
@@ -8252,7 +8312,7 @@
         </is>
       </c>
       <c r="Z111" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA111" t="n">
         <v>-6.67</v>
@@ -8321,7 +8381,7 @@
         </is>
       </c>
       <c r="Z112" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA112" t="n">
         <v>-2.8</v>
@@ -8390,7 +8450,10 @@
         </is>
       </c>
       <c r="Z113" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA113" t="n">
+        <v>-1.11</v>
       </c>
       <c r="AG113" t="b">
         <v>0</v>
@@ -8456,7 +8519,10 @@
         </is>
       </c>
       <c r="Z114" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA114" t="n">
+        <v>-2.05</v>
       </c>
       <c r="AG114" t="b">
         <v>0</v>
@@ -8522,7 +8588,10 @@
         </is>
       </c>
       <c r="Z115" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA115" t="n">
+        <v>-9.960000000000001</v>
       </c>
       <c r="AG115" t="b">
         <v>0</v>
@@ -8588,7 +8657,10 @@
         </is>
       </c>
       <c r="Z116" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA116" t="n">
+        <v>8.92</v>
       </c>
       <c r="AG116" t="b">
         <v>0</v>
@@ -8654,7 +8726,10 @@
         </is>
       </c>
       <c r="Z117" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA117" t="n">
+        <v>-1.6</v>
       </c>
       <c r="AG117" t="b">
         <v>0</v>
@@ -8720,7 +8795,10 @@
         </is>
       </c>
       <c r="Z118" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA118" t="n">
+        <v>-12.29</v>
       </c>
       <c r="AG118" t="b">
         <v>0</v>
@@ -8786,7 +8864,10 @@
         </is>
       </c>
       <c r="Z119" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA119" t="n">
+        <v>-14.49</v>
       </c>
       <c r="AG119" t="b">
         <v>0</v>
@@ -8852,7 +8933,10 @@
         </is>
       </c>
       <c r="Z120" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA120" t="n">
+        <v>-4.39</v>
       </c>
       <c r="AG120" t="b">
         <v>0</v>
@@ -8918,7 +9002,10 @@
         </is>
       </c>
       <c r="Z121" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA121" t="n">
+        <v>8.210000000000001</v>
       </c>
       <c r="AG121" t="b">
         <v>0</v>
@@ -8984,7 +9071,10 @@
         </is>
       </c>
       <c r="Z122" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA122" t="n">
+        <v>17.92</v>
       </c>
       <c r="AG122" t="b">
         <v>1</v>
@@ -9050,7 +9140,10 @@
         </is>
       </c>
       <c r="Z123" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA123" t="n">
+        <v>-1.27</v>
       </c>
       <c r="AG123" t="b">
         <v>0</v>
@@ -9116,7 +9209,10 @@
         </is>
       </c>
       <c r="Z124" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA124" t="n">
+        <v>-8.640000000000001</v>
       </c>
       <c r="AG124" t="b">
         <v>0</v>
@@ -9182,7 +9278,10 @@
         </is>
       </c>
       <c r="Z125" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA125" t="n">
+        <v>-1.75</v>
       </c>
       <c r="AG125" t="b">
         <v>0</v>
@@ -9248,7 +9347,10 @@
         </is>
       </c>
       <c r="Z126" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA126" t="n">
+        <v>-9.369999999999999</v>
       </c>
       <c r="AG126" t="b">
         <v>0</v>
@@ -9314,7 +9416,10 @@
         </is>
       </c>
       <c r="Z127" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA127" t="n">
+        <v>-6.15</v>
       </c>
       <c r="AG127" t="b">
         <v>0</v>
@@ -9380,7 +9485,10 @@
         </is>
       </c>
       <c r="Z128" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA128" t="n">
+        <v>-8.289999999999999</v>
       </c>
       <c r="AG128" t="b">
         <v>0</v>
@@ -9446,7 +9554,10 @@
         </is>
       </c>
       <c r="Z129" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA129" t="n">
+        <v>-4.83</v>
       </c>
       <c r="AG129" t="b">
         <v>0</v>
@@ -9561,7 +9672,7 @@
         </is>
       </c>
       <c r="Z130" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG130" t="b">
         <v>0</v>
@@ -9676,7 +9787,7 @@
         </is>
       </c>
       <c r="Z131" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG131" t="b">
         <v>0</v>
@@ -9791,7 +9902,7 @@
         </is>
       </c>
       <c r="Z132" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG132" t="b">
         <v>0</v>
@@ -9906,7 +10017,7 @@
         </is>
       </c>
       <c r="Z133" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG133" t="b">
         <v>0</v>
@@ -10021,7 +10132,7 @@
         </is>
       </c>
       <c r="Z134" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG134" t="b">
         <v>0</v>
@@ -10136,7 +10247,7 @@
         </is>
       </c>
       <c r="Z135" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG135" t="b">
         <v>0</v>
@@ -10251,10 +10362,10 @@
         </is>
       </c>
       <c r="Z136" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG136" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH136" t="b">
         <v>0</v>
@@ -10363,7 +10474,7 @@
         </is>
       </c>
       <c r="Z137" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG137" t="b">
         <v>0</v>
@@ -10478,7 +10589,7 @@
         </is>
       </c>
       <c r="Z138" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG138" t="b">
         <v>0</v>
@@ -10593,7 +10704,7 @@
         </is>
       </c>
       <c r="Z139" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG139" t="b">
         <v>0</v>
@@ -10708,7 +10819,7 @@
         </is>
       </c>
       <c r="Z140" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG140" t="b">
         <v>0</v>
@@ -10823,7 +10934,7 @@
         </is>
       </c>
       <c r="Z141" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG141" t="b">
         <v>0</v>
@@ -10938,7 +11049,7 @@
         </is>
       </c>
       <c r="Z142" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG142" t="b">
         <v>0</v>
@@ -11053,7 +11164,7 @@
         </is>
       </c>
       <c r="Z143" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG143" t="b">
         <v>0</v>
@@ -11168,7 +11279,7 @@
         </is>
       </c>
       <c r="Z144" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG144" t="b">
         <v>0</v>
@@ -11283,7 +11394,7 @@
         </is>
       </c>
       <c r="Z145" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG145" t="b">
         <v>0</v>
@@ -11398,7 +11509,7 @@
         </is>
       </c>
       <c r="Z146" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG146" t="b">
         <v>0</v>
@@ -11513,7 +11624,7 @@
         </is>
       </c>
       <c r="Z147" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG147" t="b">
         <v>0</v>
@@ -11628,7 +11739,7 @@
         </is>
       </c>
       <c r="Z148" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG148" t="b">
         <v>0</v>
@@ -11743,7 +11854,7 @@
         </is>
       </c>
       <c r="Z149" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG149" t="b">
         <v>0</v>
@@ -11858,7 +11969,7 @@
         </is>
       </c>
       <c r="Z150" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG150" t="b">
         <v>0</v>
@@ -11973,7 +12084,7 @@
         </is>
       </c>
       <c r="Z151" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG151" t="b">
         <v>0</v>
@@ -12088,7 +12199,7 @@
         </is>
       </c>
       <c r="Z152" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG152" t="b">
         <v>0</v>
@@ -12203,7 +12314,7 @@
         </is>
       </c>
       <c r="Z153" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG153" t="b">
         <v>0</v>
@@ -12318,7 +12429,7 @@
         </is>
       </c>
       <c r="Z154" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG154" t="b">
         <v>0</v>
@@ -12433,7 +12544,7 @@
         </is>
       </c>
       <c r="Z155" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG155" t="b">
         <v>0</v>
@@ -12548,7 +12659,7 @@
         </is>
       </c>
       <c r="Z156" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG156" t="b">
         <v>0</v>
@@ -12663,7 +12774,7 @@
         </is>
       </c>
       <c r="Z157" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG157" t="b">
         <v>0</v>
@@ -12778,7 +12889,7 @@
         </is>
       </c>
       <c r="Z158" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG158" t="b">
         <v>0</v>
@@ -12893,7 +13004,7 @@
         </is>
       </c>
       <c r="Z159" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG159" t="b">
         <v>0</v>
@@ -13008,13 +13119,13 @@
         </is>
       </c>
       <c r="Z160" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG160" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH160" t="b">
         <v>1</v>
-      </c>
-      <c r="AG160" t="b">
-        <v>0</v>
-      </c>
-      <c r="AH160" t="b">
-        <v>0</v>
       </c>
       <c r="AI160" t="inlineStr">
         <is>
@@ -13123,7 +13234,7 @@
         </is>
       </c>
       <c r="Z161" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG161" t="b">
         <v>0</v>
@@ -13238,7 +13349,7 @@
         </is>
       </c>
       <c r="Z162" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG162" t="b">
         <v>0</v>
@@ -13353,7 +13464,7 @@
         </is>
       </c>
       <c r="Z163" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG163" t="b">
         <v>0</v>
@@ -13468,7 +13579,7 @@
         </is>
       </c>
       <c r="Z164" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG164" t="b">
         <v>0</v>
@@ -13583,10 +13694,10 @@
         </is>
       </c>
       <c r="Z165" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG165" t="b">
         <v>1</v>
-      </c>
-      <c r="AG165" t="b">
-        <v>0</v>
       </c>
       <c r="AH165" t="b">
         <v>0</v>
@@ -13698,7 +13809,7 @@
         </is>
       </c>
       <c r="Z166" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG166" t="b">
         <v>0</v>
@@ -13813,7 +13924,7 @@
         </is>
       </c>
       <c r="Z167" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG167" t="b">
         <v>0</v>
@@ -14039,7 +14150,7 @@
         </is>
       </c>
       <c r="Z169" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG169" t="b">
         <v>0</v>
@@ -14154,7 +14265,7 @@
         </is>
       </c>
       <c r="Z170" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG170" t="b">
         <v>0</v>
@@ -14269,7 +14380,7 @@
         </is>
       </c>
       <c r="Z171" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG171" t="b">
         <v>0</v>
@@ -14384,7 +14495,7 @@
         </is>
       </c>
       <c r="Z172" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG172" t="b">
         <v>0</v>
@@ -14499,7 +14610,7 @@
         </is>
       </c>
       <c r="Z173" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG173" t="b">
         <v>0</v>
@@ -14614,7 +14725,7 @@
         </is>
       </c>
       <c r="Z174" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG174" t="b">
         <v>0</v>
@@ -14729,7 +14840,7 @@
         </is>
       </c>
       <c r="Z175" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG175" t="b">
         <v>0</v>
@@ -14844,7 +14955,7 @@
         </is>
       </c>
       <c r="Z176" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG176" t="b">
         <v>0</v>
@@ -14959,7 +15070,7 @@
         </is>
       </c>
       <c r="Z177" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG177" t="b">
         <v>0</v>
@@ -15074,7 +15185,7 @@
         </is>
       </c>
       <c r="Z178" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG178" t="b">
         <v>0</v>
@@ -15300,7 +15411,7 @@
         </is>
       </c>
       <c r="Z180" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG180" t="b">
         <v>0</v>
@@ -15314,8 +15425,698 @@
         </is>
       </c>
     </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>1402</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>遠東新</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E181" t="n">
+        <v>72.39</v>
+      </c>
+      <c r="F181" t="n">
+        <v>37.15</v>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>Reject</t>
+        </is>
+      </c>
+      <c r="I181" t="b">
+        <v>0</v>
+      </c>
+      <c r="J181" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="K181" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="L181" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M181" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="N181" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="O181" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="P181" t="n">
+        <v>28.65</v>
+      </c>
+      <c r="Q181" t="n">
+        <v>71.03</v>
+      </c>
+      <c r="R181" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="S181" t="n">
+        <v>7</v>
+      </c>
+      <c r="T181" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U181" t="inlineStr">
+        <is>
+          <t>unclassified</t>
+        </is>
+      </c>
+      <c r="V181" t="n">
+        <v>29.45</v>
+      </c>
+      <c r="W181" t="n">
+        <v>33.8455</v>
+      </c>
+      <c r="X181" t="n">
+        <v>27.3885</v>
+      </c>
+      <c r="Y181" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z181" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG181" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH181" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI181" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>2324</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>仁寶</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E182" t="n">
+        <v>78.75</v>
+      </c>
+      <c r="F182" t="n">
+        <v>41.48</v>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I182" t="b">
+        <v>0</v>
+      </c>
+      <c r="J182" t="n">
+        <v>9.98</v>
+      </c>
+      <c r="K182" t="n">
+        <v>45.75</v>
+      </c>
+      <c r="L182" t="inlineStr">
+        <is>
+          <t>gap_MM_Target_Up</t>
+        </is>
+      </c>
+      <c r="M182" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N182" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="O182" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="P182" t="n">
+        <v>40.3</v>
+      </c>
+      <c r="Q182" t="n">
+        <v>59.86</v>
+      </c>
+      <c r="R182" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S182" t="n">
+        <v>7</v>
+      </c>
+      <c r="T182" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U182" t="inlineStr">
+        <is>
+          <t>ai_hardware</t>
+        </is>
+      </c>
+      <c r="V182" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="W182" t="n">
+        <v>49.92</v>
+      </c>
+      <c r="X182" t="n">
+        <v>38.688</v>
+      </c>
+      <c r="Y182" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z182" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG182" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH182" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI182" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>2603</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>長榮</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E183" t="n">
+        <v>74.61</v>
+      </c>
+      <c r="F183" t="n">
+        <v>48.62</v>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I183" t="b">
+        <v>0</v>
+      </c>
+      <c r="J183" t="n">
+        <v>10</v>
+      </c>
+      <c r="K183" t="n">
+        <v>275.55</v>
+      </c>
+      <c r="L183" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M183" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N183" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="O183" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P183" t="n">
+        <v>230.25</v>
+      </c>
+      <c r="Q183" t="n">
+        <v>67.45999999999999</v>
+      </c>
+      <c r="R183" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="S183" t="n">
+        <v>7</v>
+      </c>
+      <c r="T183" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U183" t="inlineStr">
+        <is>
+          <t>shipping</t>
+        </is>
+      </c>
+      <c r="V183" t="n">
+        <v>250.5</v>
+      </c>
+      <c r="W183" t="n">
+        <v>300.6</v>
+      </c>
+      <c r="X183" t="n">
+        <v>232.965</v>
+      </c>
+      <c r="Y183" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z183" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG183" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH183" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI183" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>3008</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>大立光</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E184" t="n">
+        <v>73.04000000000001</v>
+      </c>
+      <c r="F184" t="n">
+        <v>44.42</v>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I184" t="b">
+        <v>0</v>
+      </c>
+      <c r="J184" t="n">
+        <v>10</v>
+      </c>
+      <c r="K184" t="n">
+        <v>5923.5</v>
+      </c>
+      <c r="L184" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M184" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N184" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="O184" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P184" t="n">
+        <v>4970.86</v>
+      </c>
+      <c r="Q184" t="n">
+        <v>59.48</v>
+      </c>
+      <c r="R184" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S184" t="n">
+        <v>7</v>
+      </c>
+      <c r="T184" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U184" t="inlineStr">
+        <is>
+          <t>electronic_components</t>
+        </is>
+      </c>
+      <c r="V184" t="n">
+        <v>5385</v>
+      </c>
+      <c r="W184" t="n">
+        <v>6462</v>
+      </c>
+      <c r="X184" t="n">
+        <v>5008.05</v>
+      </c>
+      <c r="Y184" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z184" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG184" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH184" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI184" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>6472</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>保瑞</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E185" t="n">
+        <v>80.95999999999999</v>
+      </c>
+      <c r="F185" t="n">
+        <v>48.47</v>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I185" t="b">
+        <v>0</v>
+      </c>
+      <c r="J185" t="n">
+        <v>10</v>
+      </c>
+      <c r="K185" t="n">
+        <v>498.3</v>
+      </c>
+      <c r="L185" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M185" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N185" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="O185" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="P185" t="n">
+        <v>431</v>
+      </c>
+      <c r="Q185" t="n">
+        <v>66.45999999999999</v>
+      </c>
+      <c r="R185" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="S185" t="n">
+        <v>7</v>
+      </c>
+      <c r="T185" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U185" t="inlineStr">
+        <is>
+          <t>unclassified</t>
+        </is>
+      </c>
+      <c r="V185" t="n">
+        <v>453</v>
+      </c>
+      <c r="W185" t="n">
+        <v>543.6</v>
+      </c>
+      <c r="X185" t="n">
+        <v>421.29</v>
+      </c>
+      <c r="Y185" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z185" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG185" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH185" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI185" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>6669</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>緯穎</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E186" t="n">
+        <v>71.09999999999999</v>
+      </c>
+      <c r="F186" t="n">
+        <v>49.74</v>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I186" t="b">
+        <v>0</v>
+      </c>
+      <c r="J186" t="n">
+        <v>10</v>
+      </c>
+      <c r="K186" t="n">
+        <v>6930</v>
+      </c>
+      <c r="L186" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M186" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N186" t="n">
+        <v>7</v>
+      </c>
+      <c r="O186" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="P186" t="n">
+        <v>6297.5</v>
+      </c>
+      <c r="Q186" t="n">
+        <v>44.92</v>
+      </c>
+      <c r="R186" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S186" t="n">
+        <v>7</v>
+      </c>
+      <c r="T186" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U186" t="inlineStr">
+        <is>
+          <t>semiconductor</t>
+        </is>
+      </c>
+      <c r="V186" t="n">
+        <v>6300</v>
+      </c>
+      <c r="W186" t="n">
+        <v>7489.4557</v>
+      </c>
+      <c r="X186" t="n">
+        <v>5859</v>
+      </c>
+      <c r="Y186" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z186" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG186" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH186" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI186" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AJ180"/>
+  <autoFilter ref="A1:AJ186"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -15565,7 +16366,7 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>2026-08-21 14:23:57</t>
+          <t>2026-08-24 14:50:49</t>
         </is>
       </c>
     </row>
@@ -15612,7 +16413,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>179</v>
+        <v>185</v>
       </c>
     </row>
     <row r="7">
@@ -15632,7 +16433,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>179</v>
+        <v>185</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-08-25 06:23:14
</commit_message>
<xml_diff>
--- a/data/swing_performance_analysis.xlsx
+++ b/data/swing_performance_analysis.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'T20_Tracking'!$A$1:$AJ$186</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'T20_Tracking'!$A$1:$AJ$202</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ186"/>
+  <dimension ref="A1:AJ202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -731,7 +731,7 @@
         </is>
       </c>
       <c r="Z2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA2" t="n">
         <v>-1.45</v>
@@ -803,7 +803,7 @@
         </is>
       </c>
       <c r="Z3" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA3" t="n">
         <v>-5.5</v>
@@ -875,7 +875,7 @@
         </is>
       </c>
       <c r="Z4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA4" t="n">
         <v>21.91</v>
@@ -947,7 +947,7 @@
         </is>
       </c>
       <c r="Z5" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA5" t="n">
         <v>3.92</v>
@@ -1019,7 +1019,7 @@
         </is>
       </c>
       <c r="Z6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA6" t="n">
         <v>7.73</v>
@@ -1091,7 +1091,7 @@
         </is>
       </c>
       <c r="Z7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA7" t="n">
         <v>5.54</v>
@@ -1163,7 +1163,7 @@
         </is>
       </c>
       <c r="Z8" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA8" t="n">
         <v>-11.56</v>
@@ -1235,7 +1235,7 @@
         </is>
       </c>
       <c r="Z9" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA9" t="n">
         <v>-10.14</v>
@@ -1307,7 +1307,7 @@
         </is>
       </c>
       <c r="Z10" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA10" t="n">
         <v>-12.27</v>
@@ -1379,7 +1379,7 @@
         </is>
       </c>
       <c r="Z11" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA11" t="n">
         <v>-6.97</v>
@@ -1451,7 +1451,7 @@
         </is>
       </c>
       <c r="Z12" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA12" t="n">
         <v>5.13</v>
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="Z13" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA13" t="n">
         <v>-5.54</v>
@@ -1657,7 +1657,7 @@
         </is>
       </c>
       <c r="Z15" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA15" t="n">
         <v>3.09</v>
@@ -1729,7 +1729,7 @@
         </is>
       </c>
       <c r="Z16" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA16" t="n">
         <v>9.31</v>
@@ -1801,7 +1801,7 @@
         </is>
       </c>
       <c r="Z17" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA17" t="n">
         <v>-1.43</v>
@@ -1873,7 +1873,7 @@
         </is>
       </c>
       <c r="Z18" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA18" t="n">
         <v>-6.69</v>
@@ -1945,7 +1945,7 @@
         </is>
       </c>
       <c r="Z19" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA19" t="n">
         <v>-4.07</v>
@@ -2017,7 +2017,7 @@
         </is>
       </c>
       <c r="Z20" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA20" t="n">
         <v>-1.42</v>
@@ -2089,7 +2089,7 @@
         </is>
       </c>
       <c r="Z21" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA21" t="n">
         <v>-3.59</v>
@@ -2161,7 +2161,7 @@
         </is>
       </c>
       <c r="Z22" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA22" t="n">
         <v>14.67</v>
@@ -2233,7 +2233,7 @@
         </is>
       </c>
       <c r="Z23" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA23" t="n">
         <v>2.43</v>
@@ -2305,7 +2305,7 @@
         </is>
       </c>
       <c r="Z24" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA24" t="n">
         <v>1.05</v>
@@ -2377,7 +2377,7 @@
         </is>
       </c>
       <c r="Z25" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA25" t="n">
         <v>8.18</v>
@@ -2449,7 +2449,7 @@
         </is>
       </c>
       <c r="Z26" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA26" t="n">
         <v>6.01</v>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="Z27" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA27" t="n">
         <v>13.83</v>
@@ -2593,7 +2593,7 @@
         </is>
       </c>
       <c r="Z28" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA28" t="n">
         <v>-10.91</v>
@@ -2665,7 +2665,7 @@
         </is>
       </c>
       <c r="Z29" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA29" t="n">
         <v>-2.87</v>
@@ -2737,7 +2737,7 @@
         </is>
       </c>
       <c r="Z30" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA30" t="n">
         <v>-8.630000000000001</v>
@@ -2809,7 +2809,7 @@
         </is>
       </c>
       <c r="Z31" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA31" t="n">
         <v>-0.91</v>
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Z32" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA32" t="n">
         <v>-6.43</v>
@@ -2953,7 +2953,7 @@
         </is>
       </c>
       <c r="Z33" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA33" t="n">
         <v>-3.11</v>
@@ -3149,7 +3149,7 @@
         </is>
       </c>
       <c r="Z36" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA36" t="n">
         <v>-3.48</v>
@@ -3221,7 +3221,7 @@
         </is>
       </c>
       <c r="Z37" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA37" t="n">
         <v>10.15</v>
@@ -3293,7 +3293,7 @@
         </is>
       </c>
       <c r="Z38" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA38" t="n">
         <v>-5.23</v>
@@ -3365,11 +3365,14 @@
         </is>
       </c>
       <c r="Z39" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA39" t="n">
         <v>-5.13</v>
       </c>
+      <c r="AB39" t="n">
+        <v>-6.41</v>
+      </c>
       <c r="AG39" t="b">
         <v>0</v>
       </c>
@@ -3434,11 +3437,14 @@
         </is>
       </c>
       <c r="Z40" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA40" t="n">
         <v>-3.13</v>
       </c>
+      <c r="AB40" t="n">
+        <v>0.39</v>
+      </c>
       <c r="AG40" t="b">
         <v>0</v>
       </c>
@@ -3503,11 +3509,14 @@
         </is>
       </c>
       <c r="Z41" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA41" t="n">
         <v>-4.05</v>
       </c>
+      <c r="AB41" t="n">
+        <v>-3.54</v>
+      </c>
       <c r="AG41" t="b">
         <v>0</v>
       </c>
@@ -3572,11 +3581,14 @@
         </is>
       </c>
       <c r="Z42" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA42" t="n">
         <v>1.86</v>
       </c>
+      <c r="AB42" t="n">
+        <v>10.24</v>
+      </c>
       <c r="AG42" t="b">
         <v>0</v>
       </c>
@@ -3641,11 +3653,14 @@
         </is>
       </c>
       <c r="Z43" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA43" t="n">
         <v>8.460000000000001</v>
       </c>
+      <c r="AB43" t="n">
+        <v>10.25</v>
+      </c>
       <c r="AG43" t="b">
         <v>1</v>
       </c>
@@ -3710,16 +3725,19 @@
         </is>
       </c>
       <c r="Z44" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA44" t="n">
         <v>10.82</v>
       </c>
+      <c r="AB44" t="n">
+        <v>-5.53</v>
+      </c>
       <c r="AG44" t="b">
         <v>0</v>
       </c>
       <c r="AH44" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI44" t="inlineStr">
         <is>
@@ -3779,11 +3797,14 @@
         </is>
       </c>
       <c r="Z45" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA45" t="n">
         <v>-0.71</v>
       </c>
+      <c r="AB45" t="n">
+        <v>-0.86</v>
+      </c>
       <c r="AG45" t="b">
         <v>0</v>
       </c>
@@ -3848,11 +3869,14 @@
         </is>
       </c>
       <c r="Z46" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA46" t="n">
         <v>12.1</v>
       </c>
+      <c r="AB46" t="n">
+        <v>1.08</v>
+      </c>
       <c r="AG46" t="b">
         <v>0</v>
       </c>
@@ -3917,11 +3941,14 @@
         </is>
       </c>
       <c r="Z47" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA47" t="n">
         <v>2.72</v>
       </c>
+      <c r="AB47" t="n">
+        <v>1.36</v>
+      </c>
       <c r="AG47" t="b">
         <v>0</v>
       </c>
@@ -3986,11 +4013,14 @@
         </is>
       </c>
       <c r="Z48" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA48" t="n">
         <v>5.32</v>
       </c>
+      <c r="AB48" t="n">
+        <v>4.29</v>
+      </c>
       <c r="AG48" t="b">
         <v>0</v>
       </c>
@@ -4055,11 +4085,14 @@
         </is>
       </c>
       <c r="Z49" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA49" t="n">
         <v>-3.36</v>
       </c>
+      <c r="AB49" t="n">
+        <v>-7.09</v>
+      </c>
       <c r="AG49" t="b">
         <v>0</v>
       </c>
@@ -4124,11 +4157,14 @@
         </is>
       </c>
       <c r="Z50" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA50" t="n">
         <v>9.17</v>
       </c>
+      <c r="AB50" t="n">
+        <v>12.84</v>
+      </c>
       <c r="AG50" t="b">
         <v>1</v>
       </c>
@@ -4193,11 +4229,14 @@
         </is>
       </c>
       <c r="Z51" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA51" t="n">
         <v>8.08</v>
       </c>
+      <c r="AB51" t="n">
+        <v>22.31</v>
+      </c>
       <c r="AG51" t="b">
         <v>1</v>
       </c>
@@ -4262,11 +4301,14 @@
         </is>
       </c>
       <c r="Z52" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA52" t="n">
         <v>20.55</v>
       </c>
+      <c r="AB52" t="n">
+        <v>45.24</v>
+      </c>
       <c r="AG52" t="b">
         <v>1</v>
       </c>
@@ -4331,11 +4373,14 @@
         </is>
       </c>
       <c r="Z53" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA53" t="n">
         <v>-0.32</v>
       </c>
+      <c r="AB53" t="n">
+        <v>2.09</v>
+      </c>
       <c r="AG53" t="b">
         <v>0</v>
       </c>
@@ -4400,11 +4445,14 @@
         </is>
       </c>
       <c r="Z54" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA54" t="n">
         <v>-5.24</v>
       </c>
+      <c r="AB54" t="n">
+        <v>-6.54</v>
+      </c>
       <c r="AG54" t="b">
         <v>0</v>
       </c>
@@ -4531,11 +4579,14 @@
         </is>
       </c>
       <c r="Z56" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA56" t="n">
         <v>-4.49</v>
       </c>
+      <c r="AB56" t="n">
+        <v>10.98</v>
+      </c>
       <c r="AG56" t="b">
         <v>0</v>
       </c>
@@ -4600,7 +4651,7 @@
         </is>
       </c>
       <c r="Z57" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA57" t="n">
         <v>-0.28</v>
@@ -4669,7 +4720,7 @@
         </is>
       </c>
       <c r="Z58" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA58" t="n">
         <v>-8.779999999999999</v>
@@ -4738,7 +4789,7 @@
         </is>
       </c>
       <c r="Z59" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA59" t="n">
         <v>-4.05</v>
@@ -4807,7 +4858,7 @@
         </is>
       </c>
       <c r="Z60" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA60" t="n">
         <v>-9.26</v>
@@ -4876,7 +4927,7 @@
         </is>
       </c>
       <c r="Z61" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA61" t="n">
         <v>8.57</v>
@@ -4945,7 +4996,7 @@
         </is>
       </c>
       <c r="Z62" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA62" t="n">
         <v>-3.42</v>
@@ -4954,7 +5005,7 @@
         <v>0</v>
       </c>
       <c r="AH62" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI62" t="inlineStr">
         <is>
@@ -5014,7 +5065,7 @@
         </is>
       </c>
       <c r="Z63" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA63" t="n">
         <v>2.62</v>
@@ -5023,7 +5074,7 @@
         <v>0</v>
       </c>
       <c r="AH63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI63" t="inlineStr">
         <is>
@@ -5083,7 +5134,7 @@
         </is>
       </c>
       <c r="Z64" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA64" t="n">
         <v>1.17</v>
@@ -5152,7 +5203,7 @@
         </is>
       </c>
       <c r="Z65" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA65" t="n">
         <v>12.12</v>
@@ -5221,7 +5272,7 @@
         </is>
       </c>
       <c r="Z66" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA66" t="n">
         <v>-1.13</v>
@@ -5290,7 +5341,7 @@
         </is>
       </c>
       <c r="Z67" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA67" t="n">
         <v>21.05</v>
@@ -5359,7 +5410,7 @@
         </is>
       </c>
       <c r="Z68" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA68" t="n">
         <v>6.36</v>
@@ -5428,7 +5479,7 @@
         </is>
       </c>
       <c r="Z69" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA69" t="n">
         <v>-5.94</v>
@@ -5559,7 +5610,7 @@
         </is>
       </c>
       <c r="Z71" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA71" t="n">
         <v>3.22</v>
@@ -5628,7 +5679,7 @@
         </is>
       </c>
       <c r="Z72" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA72" t="n">
         <v>-2.78</v>
@@ -5697,7 +5748,7 @@
         </is>
       </c>
       <c r="Z73" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA73" t="n">
         <v>5.81</v>
@@ -5766,7 +5817,7 @@
         </is>
       </c>
       <c r="Z74" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA74" t="n">
         <v>-5.04</v>
@@ -5835,7 +5886,7 @@
         </is>
       </c>
       <c r="Z75" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA75" t="n">
         <v>0.97</v>
@@ -5904,7 +5955,7 @@
         </is>
       </c>
       <c r="Z76" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA76" t="n">
         <v>-3.4</v>
@@ -5973,7 +6024,7 @@
         </is>
       </c>
       <c r="Z77" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA77" t="n">
         <v>-0.93</v>
@@ -6042,7 +6093,7 @@
         </is>
       </c>
       <c r="Z78" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA78" t="n">
         <v>-12.58</v>
@@ -6111,7 +6162,7 @@
         </is>
       </c>
       <c r="Z79" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA79" t="n">
         <v>-3.58</v>
@@ -6180,7 +6231,7 @@
         </is>
       </c>
       <c r="Z80" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA80" t="n">
         <v>0.58</v>
@@ -6249,7 +6300,7 @@
         </is>
       </c>
       <c r="Z81" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA81" t="n">
         <v>14.15</v>
@@ -6318,7 +6369,7 @@
         </is>
       </c>
       <c r="Z82" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA82" t="n">
         <v>29.71</v>
@@ -6387,7 +6438,7 @@
         </is>
       </c>
       <c r="Z83" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA83" t="n">
         <v>-1.5</v>
@@ -6456,7 +6507,7 @@
         </is>
       </c>
       <c r="Z84" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA84" t="n">
         <v>18.35</v>
@@ -6525,7 +6576,7 @@
         </is>
       </c>
       <c r="Z85" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA85" t="n">
         <v>-8.630000000000001</v>
@@ -6594,7 +6645,7 @@
         </is>
       </c>
       <c r="Z86" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA86" t="n">
         <v>1.62</v>
@@ -6663,7 +6714,7 @@
         </is>
       </c>
       <c r="Z87" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA87" t="n">
         <v>-10.5</v>
@@ -6732,7 +6783,7 @@
         </is>
       </c>
       <c r="Z88" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA88" t="n">
         <v>-4.84</v>
@@ -6801,7 +6852,7 @@
         </is>
       </c>
       <c r="Z89" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA89" t="n">
         <v>4.2</v>
@@ -6932,7 +6983,7 @@
         </is>
       </c>
       <c r="Z91" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA91" t="n">
         <v>0.95</v>
@@ -7001,7 +7052,7 @@
         </is>
       </c>
       <c r="Z92" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA92" t="n">
         <v>1.83</v>
@@ -7070,7 +7121,7 @@
         </is>
       </c>
       <c r="Z93" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA93" t="n">
         <v>-1.71</v>
@@ -7139,7 +7190,7 @@
         </is>
       </c>
       <c r="Z94" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA94" t="n">
         <v>-2.25</v>
@@ -7208,7 +7259,7 @@
         </is>
       </c>
       <c r="Z95" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA95" t="n">
         <v>-14.59</v>
@@ -7277,7 +7328,7 @@
         </is>
       </c>
       <c r="Z96" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA96" t="n">
         <v>-11.01</v>
@@ -7346,7 +7397,7 @@
         </is>
       </c>
       <c r="Z97" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA97" t="n">
         <v>-7.87</v>
@@ -7415,7 +7466,7 @@
         </is>
       </c>
       <c r="Z98" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA98" t="n">
         <v>3.12</v>
@@ -7484,7 +7535,7 @@
         </is>
       </c>
       <c r="Z99" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA99" t="n">
         <v>-9.98</v>
@@ -7553,7 +7604,7 @@
         </is>
       </c>
       <c r="Z100" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA100" t="n">
         <v>14.84</v>
@@ -7622,7 +7673,7 @@
         </is>
       </c>
       <c r="Z101" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA101" t="n">
         <v>24.03</v>
@@ -7691,7 +7742,7 @@
         </is>
       </c>
       <c r="Z102" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA102" t="n">
         <v>37.42</v>
@@ -7760,7 +7811,7 @@
         </is>
       </c>
       <c r="Z103" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA103" t="n">
         <v>-0.32</v>
@@ -7829,7 +7880,7 @@
         </is>
       </c>
       <c r="Z104" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA104" t="n">
         <v>-1.32</v>
@@ -7898,7 +7949,7 @@
         </is>
       </c>
       <c r="Z105" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA105" t="n">
         <v>21.69</v>
@@ -7967,7 +8018,7 @@
         </is>
       </c>
       <c r="Z106" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA106" t="n">
         <v>-11.44</v>
@@ -8036,7 +8087,7 @@
         </is>
       </c>
       <c r="Z107" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA107" t="n">
         <v>6.37</v>
@@ -8105,7 +8156,7 @@
         </is>
       </c>
       <c r="Z108" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA108" t="n">
         <v>-5.92</v>
@@ -8174,7 +8225,7 @@
         </is>
       </c>
       <c r="Z109" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA109" t="n">
         <v>-9.300000000000001</v>
@@ -8243,7 +8294,7 @@
         </is>
       </c>
       <c r="Z110" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA110" t="n">
         <v>2.47</v>
@@ -8312,7 +8363,7 @@
         </is>
       </c>
       <c r="Z111" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA111" t="n">
         <v>-6.67</v>
@@ -8381,7 +8432,7 @@
         </is>
       </c>
       <c r="Z112" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA112" t="n">
         <v>-2.8</v>
@@ -8450,7 +8501,7 @@
         </is>
       </c>
       <c r="Z113" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA113" t="n">
         <v>-1.11</v>
@@ -8519,7 +8570,7 @@
         </is>
       </c>
       <c r="Z114" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA114" t="n">
         <v>-2.05</v>
@@ -8588,7 +8639,7 @@
         </is>
       </c>
       <c r="Z115" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA115" t="n">
         <v>-9.960000000000001</v>
@@ -8657,7 +8708,7 @@
         </is>
       </c>
       <c r="Z116" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA116" t="n">
         <v>8.92</v>
@@ -8726,7 +8777,7 @@
         </is>
       </c>
       <c r="Z117" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA117" t="n">
         <v>-1.6</v>
@@ -8795,7 +8846,7 @@
         </is>
       </c>
       <c r="Z118" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA118" t="n">
         <v>-12.29</v>
@@ -8864,7 +8915,7 @@
         </is>
       </c>
       <c r="Z119" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA119" t="n">
         <v>-14.49</v>
@@ -8933,7 +8984,7 @@
         </is>
       </c>
       <c r="Z120" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA120" t="n">
         <v>-4.39</v>
@@ -9002,7 +9053,7 @@
         </is>
       </c>
       <c r="Z121" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA121" t="n">
         <v>8.210000000000001</v>
@@ -9071,7 +9122,7 @@
         </is>
       </c>
       <c r="Z122" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA122" t="n">
         <v>17.92</v>
@@ -9140,7 +9191,7 @@
         </is>
       </c>
       <c r="Z123" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA123" t="n">
         <v>-1.27</v>
@@ -9209,7 +9260,7 @@
         </is>
       </c>
       <c r="Z124" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA124" t="n">
         <v>-8.640000000000001</v>
@@ -9278,7 +9329,7 @@
         </is>
       </c>
       <c r="Z125" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA125" t="n">
         <v>-1.75</v>
@@ -9347,7 +9398,7 @@
         </is>
       </c>
       <c r="Z126" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA126" t="n">
         <v>-9.369999999999999</v>
@@ -9416,7 +9467,7 @@
         </is>
       </c>
       <c r="Z127" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA127" t="n">
         <v>-6.15</v>
@@ -9485,7 +9536,7 @@
         </is>
       </c>
       <c r="Z128" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA128" t="n">
         <v>-8.289999999999999</v>
@@ -9554,7 +9605,7 @@
         </is>
       </c>
       <c r="Z129" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA129" t="n">
         <v>-4.83</v>
@@ -9563,7 +9614,7 @@
         <v>0</v>
       </c>
       <c r="AH129" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI129" t="inlineStr">
         <is>
@@ -9672,7 +9723,10 @@
         </is>
       </c>
       <c r="Z130" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA130" t="n">
+        <v>0.42</v>
       </c>
       <c r="AG130" t="b">
         <v>0</v>
@@ -9787,7 +9841,10 @@
         </is>
       </c>
       <c r="Z131" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA131" t="n">
+        <v>8.23</v>
       </c>
       <c r="AG131" t="b">
         <v>0</v>
@@ -9902,7 +9959,10 @@
         </is>
       </c>
       <c r="Z132" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA132" t="n">
+        <v>0.49</v>
       </c>
       <c r="AG132" t="b">
         <v>0</v>
@@ -10017,7 +10077,10 @@
         </is>
       </c>
       <c r="Z133" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA133" t="n">
+        <v>-9.25</v>
       </c>
       <c r="AG133" t="b">
         <v>0</v>
@@ -10132,7 +10195,10 @@
         </is>
       </c>
       <c r="Z134" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA134" t="n">
+        <v>-9.83</v>
       </c>
       <c r="AG134" t="b">
         <v>0</v>
@@ -10247,7 +10313,10 @@
         </is>
       </c>
       <c r="Z135" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA135" t="n">
+        <v>-0.97</v>
       </c>
       <c r="AG135" t="b">
         <v>0</v>
@@ -10362,7 +10431,10 @@
         </is>
       </c>
       <c r="Z136" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA136" t="n">
+        <v>13.17</v>
       </c>
       <c r="AG136" t="b">
         <v>1</v>
@@ -10474,7 +10546,10 @@
         </is>
       </c>
       <c r="Z137" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA137" t="n">
+        <v>9.27</v>
       </c>
       <c r="AG137" t="b">
         <v>0</v>
@@ -10589,7 +10664,10 @@
         </is>
       </c>
       <c r="Z138" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA138" t="n">
+        <v>2.36</v>
       </c>
       <c r="AG138" t="b">
         <v>0</v>
@@ -10704,7 +10782,10 @@
         </is>
       </c>
       <c r="Z139" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA139" t="n">
+        <v>0.68</v>
       </c>
       <c r="AG139" t="b">
         <v>0</v>
@@ -10819,7 +10900,10 @@
         </is>
       </c>
       <c r="Z140" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA140" t="n">
+        <v>8.130000000000001</v>
       </c>
       <c r="AG140" t="b">
         <v>0</v>
@@ -10934,7 +11018,10 @@
         </is>
       </c>
       <c r="Z141" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA141" t="n">
+        <v>-4.37</v>
       </c>
       <c r="AG141" t="b">
         <v>0</v>
@@ -11049,7 +11136,10 @@
         </is>
       </c>
       <c r="Z142" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA142" t="n">
+        <v>-3.47</v>
       </c>
       <c r="AG142" t="b">
         <v>0</v>
@@ -11164,7 +11254,10 @@
         </is>
       </c>
       <c r="Z143" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA143" t="n">
+        <v>0.63</v>
       </c>
       <c r="AG143" t="b">
         <v>0</v>
@@ -11279,7 +11372,10 @@
         </is>
       </c>
       <c r="Z144" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA144" t="n">
+        <v>6.43</v>
       </c>
       <c r="AG144" t="b">
         <v>0</v>
@@ -11394,7 +11490,10 @@
         </is>
       </c>
       <c r="Z145" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA145" t="n">
+        <v>0.63</v>
       </c>
       <c r="AG145" t="b">
         <v>0</v>
@@ -11509,7 +11608,7 @@
         </is>
       </c>
       <c r="Z146" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG146" t="b">
         <v>0</v>
@@ -11624,7 +11723,7 @@
         </is>
       </c>
       <c r="Z147" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG147" t="b">
         <v>0</v>
@@ -11739,7 +11838,7 @@
         </is>
       </c>
       <c r="Z148" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG148" t="b">
         <v>0</v>
@@ -11854,7 +11953,7 @@
         </is>
       </c>
       <c r="Z149" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG149" t="b">
         <v>0</v>
@@ -11969,7 +12068,7 @@
         </is>
       </c>
       <c r="Z150" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG150" t="b">
         <v>0</v>
@@ -12084,7 +12183,7 @@
         </is>
       </c>
       <c r="Z151" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG151" t="b">
         <v>0</v>
@@ -12199,7 +12298,7 @@
         </is>
       </c>
       <c r="Z152" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG152" t="b">
         <v>0</v>
@@ -12314,7 +12413,7 @@
         </is>
       </c>
       <c r="Z153" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG153" t="b">
         <v>0</v>
@@ -12429,7 +12528,7 @@
         </is>
       </c>
       <c r="Z154" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG154" t="b">
         <v>0</v>
@@ -12544,7 +12643,7 @@
         </is>
       </c>
       <c r="Z155" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG155" t="b">
         <v>0</v>
@@ -12659,7 +12758,7 @@
         </is>
       </c>
       <c r="Z156" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG156" t="b">
         <v>0</v>
@@ -12774,7 +12873,7 @@
         </is>
       </c>
       <c r="Z157" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG157" t="b">
         <v>0</v>
@@ -12889,7 +12988,7 @@
         </is>
       </c>
       <c r="Z158" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG158" t="b">
         <v>0</v>
@@ -13004,7 +13103,7 @@
         </is>
       </c>
       <c r="Z159" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG159" t="b">
         <v>0</v>
@@ -13119,7 +13218,7 @@
         </is>
       </c>
       <c r="Z160" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG160" t="b">
         <v>0</v>
@@ -13234,7 +13333,7 @@
         </is>
       </c>
       <c r="Z161" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG161" t="b">
         <v>0</v>
@@ -13349,13 +13448,13 @@
         </is>
       </c>
       <c r="Z162" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG162" t="b">
         <v>0</v>
       </c>
       <c r="AH162" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI162" t="inlineStr">
         <is>
@@ -13464,7 +13563,7 @@
         </is>
       </c>
       <c r="Z163" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG163" t="b">
         <v>0</v>
@@ -13579,7 +13678,7 @@
         </is>
       </c>
       <c r="Z164" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG164" t="b">
         <v>0</v>
@@ -13694,7 +13793,7 @@
         </is>
       </c>
       <c r="Z165" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG165" t="b">
         <v>1</v>
@@ -13809,7 +13908,7 @@
         </is>
       </c>
       <c r="Z166" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG166" t="b">
         <v>0</v>
@@ -13924,7 +14023,7 @@
         </is>
       </c>
       <c r="Z167" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG167" t="b">
         <v>0</v>
@@ -14150,7 +14249,7 @@
         </is>
       </c>
       <c r="Z169" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG169" t="b">
         <v>0</v>
@@ -14265,13 +14364,13 @@
         </is>
       </c>
       <c r="Z170" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG170" t="b">
         <v>0</v>
       </c>
       <c r="AH170" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI170" t="inlineStr">
         <is>
@@ -14380,7 +14479,7 @@
         </is>
       </c>
       <c r="Z171" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG171" t="b">
         <v>0</v>
@@ -14495,7 +14594,7 @@
         </is>
       </c>
       <c r="Z172" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG172" t="b">
         <v>0</v>
@@ -14610,7 +14709,7 @@
         </is>
       </c>
       <c r="Z173" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG173" t="b">
         <v>0</v>
@@ -14725,7 +14824,7 @@
         </is>
       </c>
       <c r="Z174" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG174" t="b">
         <v>0</v>
@@ -14840,13 +14939,13 @@
         </is>
       </c>
       <c r="Z175" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG175" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH175" t="b">
         <v>1</v>
-      </c>
-      <c r="AG175" t="b">
-        <v>0</v>
-      </c>
-      <c r="AH175" t="b">
-        <v>0</v>
       </c>
       <c r="AI175" t="inlineStr">
         <is>
@@ -14955,7 +15054,7 @@
         </is>
       </c>
       <c r="Z176" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG176" t="b">
         <v>0</v>
@@ -15070,7 +15169,7 @@
         </is>
       </c>
       <c r="Z177" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG177" t="b">
         <v>0</v>
@@ -15185,7 +15284,7 @@
         </is>
       </c>
       <c r="Z178" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG178" t="b">
         <v>0</v>
@@ -15411,13 +15510,13 @@
         </is>
       </c>
       <c r="Z180" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG180" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH180" t="b">
         <v>1</v>
-      </c>
-      <c r="AG180" t="b">
-        <v>0</v>
-      </c>
-      <c r="AH180" t="b">
-        <v>0</v>
       </c>
       <c r="AI180" t="inlineStr">
         <is>
@@ -15526,7 +15625,7 @@
         </is>
       </c>
       <c r="Z181" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG181" t="b">
         <v>0</v>
@@ -15641,7 +15740,7 @@
         </is>
       </c>
       <c r="Z182" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG182" t="b">
         <v>0</v>
@@ -15756,7 +15855,7 @@
         </is>
       </c>
       <c r="Z183" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG183" t="b">
         <v>0</v>
@@ -15871,7 +15970,7 @@
         </is>
       </c>
       <c r="Z184" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG184" t="b">
         <v>0</v>
@@ -15986,7 +16085,7 @@
         </is>
       </c>
       <c r="Z185" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG185" t="b">
         <v>0</v>
@@ -16101,7 +16200,7 @@
         </is>
       </c>
       <c r="Z186" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG186" t="b">
         <v>0</v>
@@ -16115,8 +16214,1840 @@
         </is>
       </c>
     </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>1519</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>華城</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E187" t="n">
+        <v>77.54000000000001</v>
+      </c>
+      <c r="F187" t="n">
+        <v>76.72</v>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I187" t="b">
+        <v>0</v>
+      </c>
+      <c r="J187" t="n">
+        <v>10</v>
+      </c>
+      <c r="K187" t="n">
+        <v>788.7</v>
+      </c>
+      <c r="L187" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M187" t="n">
+        <v>3.05</v>
+      </c>
+      <c r="N187" t="n">
+        <v>10</v>
+      </c>
+      <c r="O187" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="P187" t="n">
+        <v>697</v>
+      </c>
+      <c r="Q187" t="n">
+        <v>51.48</v>
+      </c>
+      <c r="R187" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S187" t="n">
+        <v>3.2755</v>
+      </c>
+      <c r="T187" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U187" t="inlineStr">
+        <is>
+          <t>industrial</t>
+        </is>
+      </c>
+      <c r="V187" t="n">
+        <v>717</v>
+      </c>
+      <c r="W187" t="n">
+        <v>860.4</v>
+      </c>
+      <c r="X187" t="n">
+        <v>693.515</v>
+      </c>
+      <c r="Y187" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z187" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG187" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH187" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI187" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>2301</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>光寶科</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E188" t="n">
+        <v>84.66</v>
+      </c>
+      <c r="F188" t="n">
+        <v>46.92</v>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I188" t="b">
+        <v>0</v>
+      </c>
+      <c r="J188" t="n">
+        <v>10</v>
+      </c>
+      <c r="K188" t="n">
+        <v>325.6</v>
+      </c>
+      <c r="L188" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M188" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N188" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="O188" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P188" t="n">
+        <v>273.5</v>
+      </c>
+      <c r="Q188" t="n">
+        <v>69.45999999999999</v>
+      </c>
+      <c r="R188" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="S188" t="n">
+        <v>7</v>
+      </c>
+      <c r="T188" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U188" t="inlineStr">
+        <is>
+          <t>ai_hardware</t>
+        </is>
+      </c>
+      <c r="V188" t="n">
+        <v>296</v>
+      </c>
+      <c r="W188" t="n">
+        <v>355.2</v>
+      </c>
+      <c r="X188" t="n">
+        <v>275.28</v>
+      </c>
+      <c r="Y188" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z188" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG188" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH188" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI188" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>2324</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>仁寶</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E189" t="n">
+        <v>77.16</v>
+      </c>
+      <c r="F189" t="n">
+        <v>55.97</v>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I189" t="b">
+        <v>0</v>
+      </c>
+      <c r="J189" t="n">
+        <v>10</v>
+      </c>
+      <c r="K189" t="n">
+        <v>44.88</v>
+      </c>
+      <c r="L189" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M189" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N189" t="n">
+        <v>7</v>
+      </c>
+      <c r="O189" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="P189" t="n">
+        <v>40.3</v>
+      </c>
+      <c r="Q189" t="n">
+        <v>59.82</v>
+      </c>
+      <c r="R189" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S189" t="n">
+        <v>7</v>
+      </c>
+      <c r="T189" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U189" t="inlineStr">
+        <is>
+          <t>ai_hardware</t>
+        </is>
+      </c>
+      <c r="V189" t="n">
+        <v>40.8</v>
+      </c>
+      <c r="W189" t="n">
+        <v>48.96</v>
+      </c>
+      <c r="X189" t="n">
+        <v>37.944</v>
+      </c>
+      <c r="Y189" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z189" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG189" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH189" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI189" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>2408</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>南亞科</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E190" t="n">
+        <v>77.59</v>
+      </c>
+      <c r="F190" t="n">
+        <v>53.73</v>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I190" t="b">
+        <v>0</v>
+      </c>
+      <c r="J190" t="n">
+        <v>10</v>
+      </c>
+      <c r="K190" t="n">
+        <v>561</v>
+      </c>
+      <c r="L190" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M190" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="N190" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="O190" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="P190" t="n">
+        <v>513</v>
+      </c>
+      <c r="Q190" t="n">
+        <v>54.86</v>
+      </c>
+      <c r="R190" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S190" t="n">
+        <v>6.3529</v>
+      </c>
+      <c r="T190" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U190" t="inlineStr">
+        <is>
+          <t>semiconductor</t>
+        </is>
+      </c>
+      <c r="V190" t="n">
+        <v>510</v>
+      </c>
+      <c r="W190" t="n">
+        <v>612</v>
+      </c>
+      <c r="X190" t="n">
+        <v>477.6</v>
+      </c>
+      <c r="Y190" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z190" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG190" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH190" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI190" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>2603</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>長榮</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E191" t="n">
+        <v>72.04000000000001</v>
+      </c>
+      <c r="F191" t="n">
+        <v>50.93</v>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I191" t="b">
+        <v>0</v>
+      </c>
+      <c r="J191" t="n">
+        <v>10</v>
+      </c>
+      <c r="K191" t="n">
+        <v>270.6</v>
+      </c>
+      <c r="L191" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M191" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N191" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="O191" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="P191" t="n">
+        <v>232.25</v>
+      </c>
+      <c r="Q191" t="n">
+        <v>56.23</v>
+      </c>
+      <c r="R191" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S191" t="n">
+        <v>7</v>
+      </c>
+      <c r="T191" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U191" t="inlineStr">
+        <is>
+          <t>shipping</t>
+        </is>
+      </c>
+      <c r="V191" t="n">
+        <v>246</v>
+      </c>
+      <c r="W191" t="n">
+        <v>295.2</v>
+      </c>
+      <c r="X191" t="n">
+        <v>228.78</v>
+      </c>
+      <c r="Y191" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z191" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG191" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH191" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI191" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>2881</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>富邦金</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E192" t="n">
+        <v>76.98</v>
+      </c>
+      <c r="F192" t="n">
+        <v>32.56</v>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>Reject</t>
+        </is>
+      </c>
+      <c r="I192" t="b">
+        <v>0</v>
+      </c>
+      <c r="J192" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="K192" t="n">
+        <v>144.5</v>
+      </c>
+      <c r="L192" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M192" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="N192" t="n">
+        <v>3</v>
+      </c>
+      <c r="O192" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="P192" t="n">
+        <v>133</v>
+      </c>
+      <c r="Q192" t="n">
+        <v>70.40000000000001</v>
+      </c>
+      <c r="R192" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="S192" t="n">
+        <v>7</v>
+      </c>
+      <c r="T192" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U192" t="inlineStr">
+        <is>
+          <t>finance</t>
+        </is>
+      </c>
+      <c r="V192" t="n">
+        <v>141.5</v>
+      </c>
+      <c r="W192" t="n">
+        <v>169.6014</v>
+      </c>
+      <c r="X192" t="n">
+        <v>131.595</v>
+      </c>
+      <c r="Y192" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z192" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG192" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH192" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI192" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>2882</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>國泰金</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E193" t="n">
+        <v>71.19</v>
+      </c>
+      <c r="F193" t="n">
+        <v>54.21</v>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I193" t="b">
+        <v>0</v>
+      </c>
+      <c r="J193" t="n">
+        <v>9.220000000000001</v>
+      </c>
+      <c r="K193" t="n">
+        <v>112.5</v>
+      </c>
+      <c r="L193" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M193" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="N193" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="O193" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="P193" t="n">
+        <v>100.5</v>
+      </c>
+      <c r="Q193" t="n">
+        <v>58.05</v>
+      </c>
+      <c r="R193" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S193" t="n">
+        <v>6.2961</v>
+      </c>
+      <c r="T193" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U193" t="inlineStr">
+        <is>
+          <t>finance</t>
+        </is>
+      </c>
+      <c r="V193" t="n">
+        <v>103</v>
+      </c>
+      <c r="W193" t="n">
+        <v>116.398</v>
+      </c>
+      <c r="X193" t="n">
+        <v>96.515</v>
+      </c>
+      <c r="Y193" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z193" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG193" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH193" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI193" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>2887</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>台新金</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E194" t="n">
+        <v>70.90000000000001</v>
+      </c>
+      <c r="F194" t="n">
+        <v>62.34</v>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I194" t="b">
+        <v>0</v>
+      </c>
+      <c r="J194" t="n">
+        <v>10.01</v>
+      </c>
+      <c r="K194" t="n">
+        <v>40.87</v>
+      </c>
+      <c r="L194" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M194" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="N194" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="O194" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="P194" t="n">
+        <v>36.23</v>
+      </c>
+      <c r="Q194" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="R194" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S194" t="n">
+        <v>5.9906</v>
+      </c>
+      <c r="T194" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U194" t="inlineStr">
+        <is>
+          <t>finance</t>
+        </is>
+      </c>
+      <c r="V194" t="n">
+        <v>37.15</v>
+      </c>
+      <c r="W194" t="n">
+        <v>42.44</v>
+      </c>
+      <c r="X194" t="n">
+        <v>34.9245</v>
+      </c>
+      <c r="Y194" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z194" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG194" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH194" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI194" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>3006</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>晶豪科</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E195" t="n">
+        <v>71.47</v>
+      </c>
+      <c r="F195" t="n">
+        <v>44.38</v>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I195" t="b">
+        <v>0</v>
+      </c>
+      <c r="J195" t="n">
+        <v>10</v>
+      </c>
+      <c r="K195" t="n">
+        <v>297</v>
+      </c>
+      <c r="L195" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M195" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N195" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="O195" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="P195" t="n">
+        <v>260.75</v>
+      </c>
+      <c r="Q195" t="n">
+        <v>52.51</v>
+      </c>
+      <c r="R195" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S195" t="n">
+        <v>7</v>
+      </c>
+      <c r="T195" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U195" t="inlineStr">
+        <is>
+          <t>unclassified</t>
+        </is>
+      </c>
+      <c r="V195" t="n">
+        <v>270</v>
+      </c>
+      <c r="W195" t="n">
+        <v>324</v>
+      </c>
+      <c r="X195" t="n">
+        <v>251.1</v>
+      </c>
+      <c r="Y195" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z195" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG195" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH195" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI195" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>3008</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>大立光</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E196" t="n">
+        <v>78.18000000000001</v>
+      </c>
+      <c r="F196" t="n">
+        <v>46.15</v>
+      </c>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I196" t="b">
+        <v>0</v>
+      </c>
+      <c r="J196" t="n">
+        <v>10</v>
+      </c>
+      <c r="K196" t="n">
+        <v>6292</v>
+      </c>
+      <c r="L196" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M196" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N196" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="O196" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P196" t="n">
+        <v>4970.86</v>
+      </c>
+      <c r="Q196" t="n">
+        <v>64.31</v>
+      </c>
+      <c r="R196" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="S196" t="n">
+        <v>7</v>
+      </c>
+      <c r="T196" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U196" t="inlineStr">
+        <is>
+          <t>electronic_components</t>
+        </is>
+      </c>
+      <c r="V196" t="n">
+        <v>5720</v>
+      </c>
+      <c r="W196" t="n">
+        <v>6864</v>
+      </c>
+      <c r="X196" t="n">
+        <v>5319.6</v>
+      </c>
+      <c r="Y196" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z196" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG196" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH196" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI196" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>3034</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>聯詠</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E197" t="n">
+        <v>74.81</v>
+      </c>
+      <c r="F197" t="n">
+        <v>54.83</v>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I197" t="b">
+        <v>0</v>
+      </c>
+      <c r="J197" t="n">
+        <v>10</v>
+      </c>
+      <c r="K197" t="n">
+        <v>610.5</v>
+      </c>
+      <c r="L197" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M197" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N197" t="n">
+        <v>7</v>
+      </c>
+      <c r="O197" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="P197" t="n">
+        <v>530.25</v>
+      </c>
+      <c r="Q197" t="n">
+        <v>58.9</v>
+      </c>
+      <c r="R197" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S197" t="n">
+        <v>7</v>
+      </c>
+      <c r="T197" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U197" t="inlineStr">
+        <is>
+          <t>semiconductor</t>
+        </is>
+      </c>
+      <c r="V197" t="n">
+        <v>555</v>
+      </c>
+      <c r="W197" t="n">
+        <v>657.3330999999999</v>
+      </c>
+      <c r="X197" t="n">
+        <v>516.15</v>
+      </c>
+      <c r="Y197" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z197" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG197" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH197" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI197" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>3081</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>聯亞</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E198" t="n">
+        <v>76.13</v>
+      </c>
+      <c r="F198" t="n">
+        <v>44.03</v>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I198" t="b">
+        <v>0</v>
+      </c>
+      <c r="J198" t="n">
+        <v>10</v>
+      </c>
+      <c r="K198" t="n">
+        <v>3256</v>
+      </c>
+      <c r="L198" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M198" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N198" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="O198" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P198" t="n">
+        <v>2740</v>
+      </c>
+      <c r="Q198" t="n">
+        <v>50.23</v>
+      </c>
+      <c r="R198" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S198" t="n">
+        <v>7</v>
+      </c>
+      <c r="T198" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U198" t="inlineStr">
+        <is>
+          <t>unclassified</t>
+        </is>
+      </c>
+      <c r="V198" t="n">
+        <v>2960</v>
+      </c>
+      <c r="W198" t="n">
+        <v>3552</v>
+      </c>
+      <c r="X198" t="n">
+        <v>2752.8</v>
+      </c>
+      <c r="Y198" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="AI198" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="AJ198" t="inlineStr">
+        <is>
+          <t>market_data_temporarily_unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>3324</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>雙鴻</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E199" t="n">
+        <v>72.75</v>
+      </c>
+      <c r="F199" t="n">
+        <v>33.05</v>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>Reject</t>
+        </is>
+      </c>
+      <c r="I199" t="b">
+        <v>0</v>
+      </c>
+      <c r="J199" t="n">
+        <v>3.76</v>
+      </c>
+      <c r="K199" t="n">
+        <v>1105</v>
+      </c>
+      <c r="L199" t="inlineStr">
+        <is>
+          <t>gap_MM_Target_Up</t>
+        </is>
+      </c>
+      <c r="M199" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="N199" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="O199" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="P199" t="n">
+        <v>1017.5</v>
+      </c>
+      <c r="Q199" t="n">
+        <v>57</v>
+      </c>
+      <c r="R199" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S199" t="n">
+        <v>7</v>
+      </c>
+      <c r="T199" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U199" t="inlineStr">
+        <is>
+          <t>unclassified</t>
+        </is>
+      </c>
+      <c r="V199" t="n">
+        <v>1065</v>
+      </c>
+      <c r="W199" t="n">
+        <v>1278</v>
+      </c>
+      <c r="X199" t="n">
+        <v>990.45</v>
+      </c>
+      <c r="Y199" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="AI199" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="AJ199" t="inlineStr">
+        <is>
+          <t>market_data_temporarily_unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>3443</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>創意</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E200" t="n">
+        <v>76.09</v>
+      </c>
+      <c r="F200" t="n">
+        <v>47.11</v>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I200" t="b">
+        <v>0</v>
+      </c>
+      <c r="J200" t="n">
+        <v>10</v>
+      </c>
+      <c r="K200" t="n">
+        <v>6127</v>
+      </c>
+      <c r="L200" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M200" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N200" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="O200" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P200" t="n">
+        <v>5250</v>
+      </c>
+      <c r="Q200" t="n">
+        <v>50.76</v>
+      </c>
+      <c r="R200" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S200" t="n">
+        <v>7</v>
+      </c>
+      <c r="T200" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U200" t="inlineStr">
+        <is>
+          <t>semiconductor</t>
+        </is>
+      </c>
+      <c r="V200" t="n">
+        <v>5570</v>
+      </c>
+      <c r="W200" t="n">
+        <v>6684</v>
+      </c>
+      <c r="X200" t="n">
+        <v>5180.1</v>
+      </c>
+      <c r="Y200" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z200" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG200" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH200" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI200" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>6446</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>藥華藥</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E201" t="n">
+        <v>76.48</v>
+      </c>
+      <c r="F201" t="n">
+        <v>44.78</v>
+      </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I201" t="b">
+        <v>0</v>
+      </c>
+      <c r="J201" t="n">
+        <v>10</v>
+      </c>
+      <c r="K201" t="n">
+        <v>1639</v>
+      </c>
+      <c r="L201" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M201" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N201" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="O201" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P201" t="n">
+        <v>1370</v>
+      </c>
+      <c r="Q201" t="n">
+        <v>55.17</v>
+      </c>
+      <c r="R201" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S201" t="n">
+        <v>7</v>
+      </c>
+      <c r="T201" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U201" t="inlineStr">
+        <is>
+          <t>unclassified</t>
+        </is>
+      </c>
+      <c r="V201" t="n">
+        <v>1490</v>
+      </c>
+      <c r="W201" t="n">
+        <v>1788</v>
+      </c>
+      <c r="X201" t="n">
+        <v>1385.7</v>
+      </c>
+      <c r="Y201" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z201" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG201" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH201" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI201" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>6669</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>緯穎</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>swing_buy_confirmed</t>
+        </is>
+      </c>
+      <c r="E202" t="n">
+        <v>82.8</v>
+      </c>
+      <c r="F202" t="n">
+        <v>58.63</v>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I202" t="b">
+        <v>0</v>
+      </c>
+      <c r="J202" t="n">
+        <v>10</v>
+      </c>
+      <c r="K202" t="n">
+        <v>7084</v>
+      </c>
+      <c r="L202" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M202" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N202" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="O202" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="P202" t="n">
+        <v>6297.5</v>
+      </c>
+      <c r="Q202" t="n">
+        <v>60.84</v>
+      </c>
+      <c r="R202" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="S202" t="n">
+        <v>7</v>
+      </c>
+      <c r="T202" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U202" t="inlineStr">
+        <is>
+          <t>semiconductor</t>
+        </is>
+      </c>
+      <c r="V202" t="n">
+        <v>6440</v>
+      </c>
+      <c r="W202" t="n">
+        <v>7728</v>
+      </c>
+      <c r="X202" t="n">
+        <v>5989.2</v>
+      </c>
+      <c r="Y202" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z202" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG202" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH202" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI202" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AJ186"/>
+  <autoFilter ref="A1:AJ202"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -16366,7 +18297,7 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>2026-08-24 14:50:49</t>
+          <t>2026-08-25 14:23:08</t>
         </is>
       </c>
     </row>
@@ -16413,7 +18344,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>185</v>
+        <v>201</v>
       </c>
     </row>
     <row r="7">
@@ -16433,7 +18364,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>185</v>
+        <v>201</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-08-26 06:24:10
</commit_message>
<xml_diff>
--- a/data/swing_performance_analysis.xlsx
+++ b/data/swing_performance_analysis.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'T20_Tracking'!$A$1:$AJ$202</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'T20_Tracking'!$A$1:$AJ$217</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ202"/>
+  <dimension ref="A1:AJ217"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -731,7 +731,7 @@
         </is>
       </c>
       <c r="Z2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AA2" t="n">
         <v>-1.45</v>
@@ -803,7 +803,7 @@
         </is>
       </c>
       <c r="Z3" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AA3" t="n">
         <v>-5.5</v>
@@ -875,7 +875,7 @@
         </is>
       </c>
       <c r="Z4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AA4" t="n">
         <v>21.91</v>
@@ -947,7 +947,7 @@
         </is>
       </c>
       <c r="Z5" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AA5" t="n">
         <v>3.92</v>
@@ -1019,7 +1019,7 @@
         </is>
       </c>
       <c r="Z6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AA6" t="n">
         <v>7.73</v>
@@ -1091,7 +1091,7 @@
         </is>
       </c>
       <c r="Z7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AA7" t="n">
         <v>5.54</v>
@@ -1163,7 +1163,7 @@
         </is>
       </c>
       <c r="Z8" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AA8" t="n">
         <v>-11.56</v>
@@ -1235,7 +1235,7 @@
         </is>
       </c>
       <c r="Z9" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AA9" t="n">
         <v>-10.14</v>
@@ -1307,7 +1307,7 @@
         </is>
       </c>
       <c r="Z10" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AA10" t="n">
         <v>-12.27</v>
@@ -1379,7 +1379,7 @@
         </is>
       </c>
       <c r="Z11" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AA11" t="n">
         <v>-6.97</v>
@@ -1451,7 +1451,7 @@
         </is>
       </c>
       <c r="Z12" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AA12" t="n">
         <v>5.13</v>
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="Z13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AA13" t="n">
         <v>-5.54</v>
@@ -1657,7 +1657,7 @@
         </is>
       </c>
       <c r="Z15" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AA15" t="n">
         <v>3.09</v>
@@ -1729,7 +1729,7 @@
         </is>
       </c>
       <c r="Z16" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AA16" t="n">
         <v>9.31</v>
@@ -1801,7 +1801,7 @@
         </is>
       </c>
       <c r="Z17" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA17" t="n">
         <v>-1.43</v>
@@ -1873,7 +1873,7 @@
         </is>
       </c>
       <c r="Z18" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA18" t="n">
         <v>-6.69</v>
@@ -1945,7 +1945,7 @@
         </is>
       </c>
       <c r="Z19" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA19" t="n">
         <v>-4.07</v>
@@ -2017,7 +2017,7 @@
         </is>
       </c>
       <c r="Z20" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA20" t="n">
         <v>-1.42</v>
@@ -2089,7 +2089,7 @@
         </is>
       </c>
       <c r="Z21" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA21" t="n">
         <v>-3.59</v>
@@ -2161,7 +2161,7 @@
         </is>
       </c>
       <c r="Z22" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA22" t="n">
         <v>14.67</v>
@@ -2233,7 +2233,7 @@
         </is>
       </c>
       <c r="Z23" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA23" t="n">
         <v>2.43</v>
@@ -2305,7 +2305,7 @@
         </is>
       </c>
       <c r="Z24" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA24" t="n">
         <v>1.05</v>
@@ -2377,7 +2377,7 @@
         </is>
       </c>
       <c r="Z25" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA25" t="n">
         <v>8.18</v>
@@ -2449,7 +2449,7 @@
         </is>
       </c>
       <c r="Z26" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA26" t="n">
         <v>6.01</v>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="Z27" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA27" t="n">
         <v>13.83</v>
@@ -2593,7 +2593,7 @@
         </is>
       </c>
       <c r="Z28" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA28" t="n">
         <v>-10.91</v>
@@ -2665,7 +2665,7 @@
         </is>
       </c>
       <c r="Z29" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA29" t="n">
         <v>-2.87</v>
@@ -2737,7 +2737,7 @@
         </is>
       </c>
       <c r="Z30" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA30" t="n">
         <v>-8.630000000000001</v>
@@ -2809,7 +2809,7 @@
         </is>
       </c>
       <c r="Z31" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA31" t="n">
         <v>-0.91</v>
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Z32" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA32" t="n">
         <v>-6.43</v>
@@ -2953,7 +2953,7 @@
         </is>
       </c>
       <c r="Z33" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA33" t="n">
         <v>-3.11</v>
@@ -3149,7 +3149,7 @@
         </is>
       </c>
       <c r="Z36" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA36" t="n">
         <v>-3.48</v>
@@ -3221,7 +3221,7 @@
         </is>
       </c>
       <c r="Z37" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA37" t="n">
         <v>10.15</v>
@@ -3293,7 +3293,7 @@
         </is>
       </c>
       <c r="Z38" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA38" t="n">
         <v>-5.23</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="Z39" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA39" t="n">
         <v>-5.13</v>
@@ -3437,7 +3437,7 @@
         </is>
       </c>
       <c r="Z40" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA40" t="n">
         <v>-3.13</v>
@@ -3509,7 +3509,7 @@
         </is>
       </c>
       <c r="Z41" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA41" t="n">
         <v>-4.05</v>
@@ -3581,7 +3581,7 @@
         </is>
       </c>
       <c r="Z42" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA42" t="n">
         <v>1.86</v>
@@ -3653,7 +3653,7 @@
         </is>
       </c>
       <c r="Z43" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA43" t="n">
         <v>8.460000000000001</v>
@@ -3725,7 +3725,7 @@
         </is>
       </c>
       <c r="Z44" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA44" t="n">
         <v>10.82</v>
@@ -3797,7 +3797,7 @@
         </is>
       </c>
       <c r="Z45" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA45" t="n">
         <v>-0.71</v>
@@ -3869,7 +3869,7 @@
         </is>
       </c>
       <c r="Z46" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA46" t="n">
         <v>12.1</v>
@@ -3941,7 +3941,7 @@
         </is>
       </c>
       <c r="Z47" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA47" t="n">
         <v>2.72</v>
@@ -4013,7 +4013,7 @@
         </is>
       </c>
       <c r="Z48" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA48" t="n">
         <v>5.32</v>
@@ -4085,7 +4085,7 @@
         </is>
       </c>
       <c r="Z49" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA49" t="n">
         <v>-3.36</v>
@@ -4157,7 +4157,7 @@
         </is>
       </c>
       <c r="Z50" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA50" t="n">
         <v>9.17</v>
@@ -4229,7 +4229,7 @@
         </is>
       </c>
       <c r="Z51" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA51" t="n">
         <v>8.08</v>
@@ -4301,7 +4301,7 @@
         </is>
       </c>
       <c r="Z52" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA52" t="n">
         <v>20.55</v>
@@ -4373,7 +4373,7 @@
         </is>
       </c>
       <c r="Z53" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA53" t="n">
         <v>-0.32</v>
@@ -4445,7 +4445,7 @@
         </is>
       </c>
       <c r="Z54" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA54" t="n">
         <v>-5.24</v>
@@ -4579,7 +4579,7 @@
         </is>
       </c>
       <c r="Z56" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA56" t="n">
         <v>-4.49</v>
@@ -4651,11 +4651,14 @@
         </is>
       </c>
       <c r="Z57" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA57" t="n">
         <v>-0.28</v>
       </c>
+      <c r="AB57" t="n">
+        <v>-0.42</v>
+      </c>
       <c r="AG57" t="b">
         <v>0</v>
       </c>
@@ -4720,11 +4723,14 @@
         </is>
       </c>
       <c r="Z58" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA58" t="n">
         <v>-8.779999999999999</v>
       </c>
+      <c r="AB58" t="n">
+        <v>-7.84</v>
+      </c>
       <c r="AG58" t="b">
         <v>0</v>
       </c>
@@ -4789,11 +4795,14 @@
         </is>
       </c>
       <c r="Z59" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA59" t="n">
         <v>-4.05</v>
       </c>
+      <c r="AB59" t="n">
+        <v>-2.03</v>
+      </c>
       <c r="AG59" t="b">
         <v>0</v>
       </c>
@@ -4858,11 +4867,14 @@
         </is>
       </c>
       <c r="Z60" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA60" t="n">
         <v>-9.26</v>
       </c>
+      <c r="AB60" t="n">
+        <v>-8.699999999999999</v>
+      </c>
       <c r="AG60" t="b">
         <v>0</v>
       </c>
@@ -4927,11 +4939,14 @@
         </is>
       </c>
       <c r="Z61" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA61" t="n">
         <v>8.57</v>
       </c>
+      <c r="AB61" t="n">
+        <v>13.97</v>
+      </c>
       <c r="AG61" t="b">
         <v>1</v>
       </c>
@@ -4996,11 +5011,14 @@
         </is>
       </c>
       <c r="Z62" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA62" t="n">
         <v>-3.42</v>
       </c>
+      <c r="AB62" t="n">
+        <v>-9.789999999999999</v>
+      </c>
       <c r="AG62" t="b">
         <v>0</v>
       </c>
@@ -5065,11 +5083,14 @@
         </is>
       </c>
       <c r="Z63" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA63" t="n">
         <v>2.62</v>
       </c>
+      <c r="AB63" t="n">
+        <v>2.88</v>
+      </c>
       <c r="AG63" t="b">
         <v>0</v>
       </c>
@@ -5134,11 +5155,14 @@
         </is>
       </c>
       <c r="Z64" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA64" t="n">
         <v>1.17</v>
       </c>
+      <c r="AB64" t="n">
+        <v>0.29</v>
+      </c>
       <c r="AG64" t="b">
         <v>0</v>
       </c>
@@ -5203,11 +5227,14 @@
         </is>
       </c>
       <c r="Z65" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA65" t="n">
         <v>12.12</v>
       </c>
+      <c r="AB65" t="n">
+        <v>7.69</v>
+      </c>
       <c r="AG65" t="b">
         <v>1</v>
       </c>
@@ -5272,11 +5299,14 @@
         </is>
       </c>
       <c r="Z66" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA66" t="n">
         <v>-1.13</v>
       </c>
+      <c r="AB66" t="n">
+        <v>-1.76</v>
+      </c>
       <c r="AG66" t="b">
         <v>0</v>
       </c>
@@ -5341,11 +5371,14 @@
         </is>
       </c>
       <c r="Z67" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA67" t="n">
         <v>21.05</v>
       </c>
+      <c r="AB67" t="n">
+        <v>37.19</v>
+      </c>
       <c r="AG67" t="b">
         <v>1</v>
       </c>
@@ -5410,11 +5443,14 @@
         </is>
       </c>
       <c r="Z68" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA68" t="n">
         <v>6.36</v>
       </c>
+      <c r="AB68" t="n">
+        <v>8.42</v>
+      </c>
       <c r="AG68" t="b">
         <v>0</v>
       </c>
@@ -5479,11 +5515,14 @@
         </is>
       </c>
       <c r="Z69" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA69" t="n">
         <v>-5.94</v>
       </c>
+      <c r="AB69" t="n">
+        <v>-5.94</v>
+      </c>
       <c r="AG69" t="b">
         <v>0</v>
       </c>
@@ -5610,11 +5649,14 @@
         </is>
       </c>
       <c r="Z71" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA71" t="n">
         <v>3.22</v>
       </c>
+      <c r="AB71" t="n">
+        <v>19.4</v>
+      </c>
       <c r="AG71" t="b">
         <v>0</v>
       </c>
@@ -5679,11 +5721,14 @@
         </is>
       </c>
       <c r="Z72" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA72" t="n">
         <v>-2.78</v>
       </c>
+      <c r="AB72" t="n">
+        <v>10.07</v>
+      </c>
       <c r="AG72" t="b">
         <v>0</v>
       </c>
@@ -5748,11 +5793,14 @@
         </is>
       </c>
       <c r="Z73" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA73" t="n">
         <v>5.81</v>
       </c>
+      <c r="AB73" t="n">
+        <v>12.61</v>
+      </c>
       <c r="AG73" t="b">
         <v>0</v>
       </c>
@@ -5817,11 +5865,14 @@
         </is>
       </c>
       <c r="Z74" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA74" t="n">
         <v>-5.04</v>
       </c>
+      <c r="AB74" t="n">
+        <v>-9</v>
+      </c>
       <c r="AG74" t="b">
         <v>0</v>
       </c>
@@ -5886,7 +5937,7 @@
         </is>
       </c>
       <c r="Z75" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA75" t="n">
         <v>0.97</v>
@@ -5955,7 +6006,7 @@
         </is>
       </c>
       <c r="Z76" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA76" t="n">
         <v>-3.4</v>
@@ -6024,7 +6075,7 @@
         </is>
       </c>
       <c r="Z77" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA77" t="n">
         <v>-0.93</v>
@@ -6093,7 +6144,7 @@
         </is>
       </c>
       <c r="Z78" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA78" t="n">
         <v>-12.58</v>
@@ -6162,7 +6213,7 @@
         </is>
       </c>
       <c r="Z79" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA79" t="n">
         <v>-3.58</v>
@@ -6231,7 +6282,7 @@
         </is>
       </c>
       <c r="Z80" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA80" t="n">
         <v>0.58</v>
@@ -6300,7 +6351,7 @@
         </is>
       </c>
       <c r="Z81" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA81" t="n">
         <v>14.15</v>
@@ -6369,7 +6420,7 @@
         </is>
       </c>
       <c r="Z82" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA82" t="n">
         <v>29.71</v>
@@ -6438,7 +6489,7 @@
         </is>
       </c>
       <c r="Z83" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA83" t="n">
         <v>-1.5</v>
@@ -6507,7 +6558,7 @@
         </is>
       </c>
       <c r="Z84" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA84" t="n">
         <v>18.35</v>
@@ -6576,7 +6627,7 @@
         </is>
       </c>
       <c r="Z85" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA85" t="n">
         <v>-8.630000000000001</v>
@@ -6645,7 +6696,7 @@
         </is>
       </c>
       <c r="Z86" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA86" t="n">
         <v>1.62</v>
@@ -6714,7 +6765,7 @@
         </is>
       </c>
       <c r="Z87" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA87" t="n">
         <v>-10.5</v>
@@ -6783,7 +6834,7 @@
         </is>
       </c>
       <c r="Z88" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA88" t="n">
         <v>-4.84</v>
@@ -6852,7 +6903,7 @@
         </is>
       </c>
       <c r="Z89" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA89" t="n">
         <v>4.2</v>
@@ -6983,7 +7034,7 @@
         </is>
       </c>
       <c r="Z91" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA91" t="n">
         <v>0.95</v>
@@ -7052,7 +7103,7 @@
         </is>
       </c>
       <c r="Z92" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA92" t="n">
         <v>1.83</v>
@@ -7121,7 +7172,7 @@
         </is>
       </c>
       <c r="Z93" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA93" t="n">
         <v>-1.71</v>
@@ -7190,7 +7241,7 @@
         </is>
       </c>
       <c r="Z94" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA94" t="n">
         <v>-2.25</v>
@@ -7259,7 +7310,7 @@
         </is>
       </c>
       <c r="Z95" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA95" t="n">
         <v>-14.59</v>
@@ -7328,7 +7379,7 @@
         </is>
       </c>
       <c r="Z96" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA96" t="n">
         <v>-11.01</v>
@@ -7397,7 +7448,7 @@
         </is>
       </c>
       <c r="Z97" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA97" t="n">
         <v>-7.87</v>
@@ -7466,7 +7517,7 @@
         </is>
       </c>
       <c r="Z98" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA98" t="n">
         <v>3.12</v>
@@ -7535,7 +7586,7 @@
         </is>
       </c>
       <c r="Z99" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA99" t="n">
         <v>-9.98</v>
@@ -7604,7 +7655,7 @@
         </is>
       </c>
       <c r="Z100" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA100" t="n">
         <v>14.84</v>
@@ -7673,7 +7724,7 @@
         </is>
       </c>
       <c r="Z101" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA101" t="n">
         <v>24.03</v>
@@ -7742,7 +7793,7 @@
         </is>
       </c>
       <c r="Z102" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA102" t="n">
         <v>37.42</v>
@@ -7811,7 +7862,7 @@
         </is>
       </c>
       <c r="Z103" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA103" t="n">
         <v>-0.32</v>
@@ -7880,7 +7931,7 @@
         </is>
       </c>
       <c r="Z104" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA104" t="n">
         <v>-1.32</v>
@@ -7949,7 +8000,7 @@
         </is>
       </c>
       <c r="Z105" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA105" t="n">
         <v>21.69</v>
@@ -8018,7 +8069,7 @@
         </is>
       </c>
       <c r="Z106" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA106" t="n">
         <v>-11.44</v>
@@ -8087,7 +8138,7 @@
         </is>
       </c>
       <c r="Z107" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA107" t="n">
         <v>6.37</v>
@@ -8156,7 +8207,7 @@
         </is>
       </c>
       <c r="Z108" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA108" t="n">
         <v>-5.92</v>
@@ -8225,7 +8276,7 @@
         </is>
       </c>
       <c r="Z109" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA109" t="n">
         <v>-9.300000000000001</v>
@@ -8294,7 +8345,7 @@
         </is>
       </c>
       <c r="Z110" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA110" t="n">
         <v>2.47</v>
@@ -8363,7 +8414,7 @@
         </is>
       </c>
       <c r="Z111" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA111" t="n">
         <v>-6.67</v>
@@ -8432,7 +8483,7 @@
         </is>
       </c>
       <c r="Z112" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA112" t="n">
         <v>-2.8</v>
@@ -8501,7 +8552,7 @@
         </is>
       </c>
       <c r="Z113" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA113" t="n">
         <v>-1.11</v>
@@ -8570,7 +8621,7 @@
         </is>
       </c>
       <c r="Z114" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA114" t="n">
         <v>-2.05</v>
@@ -8639,7 +8690,7 @@
         </is>
       </c>
       <c r="Z115" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA115" t="n">
         <v>-9.960000000000001</v>
@@ -8708,7 +8759,7 @@
         </is>
       </c>
       <c r="Z116" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA116" t="n">
         <v>8.92</v>
@@ -8777,7 +8828,7 @@
         </is>
       </c>
       <c r="Z117" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA117" t="n">
         <v>-1.6</v>
@@ -8846,7 +8897,7 @@
         </is>
       </c>
       <c r="Z118" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA118" t="n">
         <v>-12.29</v>
@@ -8915,7 +8966,7 @@
         </is>
       </c>
       <c r="Z119" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA119" t="n">
         <v>-14.49</v>
@@ -8984,7 +9035,7 @@
         </is>
       </c>
       <c r="Z120" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA120" t="n">
         <v>-4.39</v>
@@ -9053,7 +9104,7 @@
         </is>
       </c>
       <c r="Z121" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA121" t="n">
         <v>8.210000000000001</v>
@@ -9122,7 +9173,7 @@
         </is>
       </c>
       <c r="Z122" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA122" t="n">
         <v>17.92</v>
@@ -9191,7 +9242,7 @@
         </is>
       </c>
       <c r="Z123" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA123" t="n">
         <v>-1.27</v>
@@ -9260,7 +9311,7 @@
         </is>
       </c>
       <c r="Z124" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA124" t="n">
         <v>-8.640000000000001</v>
@@ -9329,7 +9380,7 @@
         </is>
       </c>
       <c r="Z125" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA125" t="n">
         <v>-1.75</v>
@@ -9398,7 +9449,7 @@
         </is>
       </c>
       <c r="Z126" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA126" t="n">
         <v>-9.369999999999999</v>
@@ -9467,7 +9518,7 @@
         </is>
       </c>
       <c r="Z127" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA127" t="n">
         <v>-6.15</v>
@@ -9536,7 +9587,7 @@
         </is>
       </c>
       <c r="Z128" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA128" t="n">
         <v>-8.289999999999999</v>
@@ -9605,7 +9656,7 @@
         </is>
       </c>
       <c r="Z129" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA129" t="n">
         <v>-4.83</v>
@@ -9723,7 +9774,7 @@
         </is>
       </c>
       <c r="Z130" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA130" t="n">
         <v>0.42</v>
@@ -9841,7 +9892,7 @@
         </is>
       </c>
       <c r="Z131" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA131" t="n">
         <v>8.23</v>
@@ -9959,7 +10010,7 @@
         </is>
       </c>
       <c r="Z132" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA132" t="n">
         <v>0.49</v>
@@ -10077,7 +10128,7 @@
         </is>
       </c>
       <c r="Z133" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA133" t="n">
         <v>-9.25</v>
@@ -10195,7 +10246,7 @@
         </is>
       </c>
       <c r="Z134" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA134" t="n">
         <v>-9.83</v>
@@ -10313,7 +10364,7 @@
         </is>
       </c>
       <c r="Z135" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA135" t="n">
         <v>-0.97</v>
@@ -10431,7 +10482,7 @@
         </is>
       </c>
       <c r="Z136" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA136" t="n">
         <v>13.17</v>
@@ -10546,7 +10597,7 @@
         </is>
       </c>
       <c r="Z137" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA137" t="n">
         <v>9.27</v>
@@ -10664,7 +10715,7 @@
         </is>
       </c>
       <c r="Z138" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA138" t="n">
         <v>2.36</v>
@@ -10782,7 +10833,7 @@
         </is>
       </c>
       <c r="Z139" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA139" t="n">
         <v>0.68</v>
@@ -10900,7 +10951,7 @@
         </is>
       </c>
       <c r="Z140" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA140" t="n">
         <v>8.130000000000001</v>
@@ -11018,7 +11069,7 @@
         </is>
       </c>
       <c r="Z141" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA141" t="n">
         <v>-4.37</v>
@@ -11136,7 +11187,7 @@
         </is>
       </c>
       <c r="Z142" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA142" t="n">
         <v>-3.47</v>
@@ -11254,7 +11305,7 @@
         </is>
       </c>
       <c r="Z143" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA143" t="n">
         <v>0.63</v>
@@ -11372,7 +11423,7 @@
         </is>
       </c>
       <c r="Z144" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA144" t="n">
         <v>6.43</v>
@@ -11490,7 +11541,7 @@
         </is>
       </c>
       <c r="Z145" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA145" t="n">
         <v>0.63</v>
@@ -11608,7 +11659,10 @@
         </is>
       </c>
       <c r="Z146" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA146" t="n">
+        <v>4.14</v>
       </c>
       <c r="AG146" t="b">
         <v>0</v>
@@ -11723,7 +11777,10 @@
         </is>
       </c>
       <c r="Z147" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA147" t="n">
+        <v>0.26</v>
       </c>
       <c r="AG147" t="b">
         <v>0</v>
@@ -11838,7 +11895,10 @@
         </is>
       </c>
       <c r="Z148" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA148" t="n">
+        <v>-0.14</v>
       </c>
       <c r="AG148" t="b">
         <v>0</v>
@@ -11953,7 +12013,10 @@
         </is>
       </c>
       <c r="Z149" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA149" t="n">
+        <v>12.25</v>
       </c>
       <c r="AG149" t="b">
         <v>0</v>
@@ -12068,7 +12131,10 @@
         </is>
       </c>
       <c r="Z150" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA150" t="n">
+        <v>-3.95</v>
       </c>
       <c r="AG150" t="b">
         <v>0</v>
@@ -12183,7 +12249,10 @@
         </is>
       </c>
       <c r="Z151" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA151" t="n">
+        <v>13.33</v>
       </c>
       <c r="AG151" t="b">
         <v>0</v>
@@ -12298,7 +12367,10 @@
         </is>
       </c>
       <c r="Z152" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA152" t="n">
+        <v>2.65</v>
       </c>
       <c r="AG152" t="b">
         <v>0</v>
@@ -12413,7 +12485,7 @@
         </is>
       </c>
       <c r="Z153" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG153" t="b">
         <v>0</v>
@@ -12528,7 +12600,7 @@
         </is>
       </c>
       <c r="Z154" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG154" t="b">
         <v>0</v>
@@ -12643,7 +12715,7 @@
         </is>
       </c>
       <c r="Z155" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG155" t="b">
         <v>0</v>
@@ -12758,7 +12830,7 @@
         </is>
       </c>
       <c r="Z156" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG156" t="b">
         <v>0</v>
@@ -12873,7 +12945,7 @@
         </is>
       </c>
       <c r="Z157" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG157" t="b">
         <v>0</v>
@@ -12988,7 +13060,7 @@
         </is>
       </c>
       <c r="Z158" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG158" t="b">
         <v>0</v>
@@ -13103,7 +13175,7 @@
         </is>
       </c>
       <c r="Z159" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG159" t="b">
         <v>0</v>
@@ -13218,7 +13290,7 @@
         </is>
       </c>
       <c r="Z160" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG160" t="b">
         <v>0</v>
@@ -13333,7 +13405,7 @@
         </is>
       </c>
       <c r="Z161" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG161" t="b">
         <v>0</v>
@@ -13448,7 +13520,7 @@
         </is>
       </c>
       <c r="Z162" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG162" t="b">
         <v>0</v>
@@ -13563,7 +13635,7 @@
         </is>
       </c>
       <c r="Z163" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG163" t="b">
         <v>0</v>
@@ -13678,7 +13750,7 @@
         </is>
       </c>
       <c r="Z164" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG164" t="b">
         <v>0</v>
@@ -13793,7 +13865,7 @@
         </is>
       </c>
       <c r="Z165" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG165" t="b">
         <v>1</v>
@@ -13908,7 +13980,7 @@
         </is>
       </c>
       <c r="Z166" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG166" t="b">
         <v>0</v>
@@ -14023,7 +14095,7 @@
         </is>
       </c>
       <c r="Z167" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG167" t="b">
         <v>0</v>
@@ -14249,7 +14321,7 @@
         </is>
       </c>
       <c r="Z169" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG169" t="b">
         <v>0</v>
@@ -14364,7 +14436,7 @@
         </is>
       </c>
       <c r="Z170" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG170" t="b">
         <v>0</v>
@@ -14479,7 +14551,7 @@
         </is>
       </c>
       <c r="Z171" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG171" t="b">
         <v>0</v>
@@ -14594,7 +14666,7 @@
         </is>
       </c>
       <c r="Z172" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG172" t="b">
         <v>0</v>
@@ -14709,7 +14781,7 @@
         </is>
       </c>
       <c r="Z173" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG173" t="b">
         <v>0</v>
@@ -14824,7 +14896,7 @@
         </is>
       </c>
       <c r="Z174" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG174" t="b">
         <v>0</v>
@@ -14939,7 +15011,7 @@
         </is>
       </c>
       <c r="Z175" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG175" t="b">
         <v>0</v>
@@ -15054,7 +15126,7 @@
         </is>
       </c>
       <c r="Z176" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG176" t="b">
         <v>0</v>
@@ -15169,7 +15241,7 @@
         </is>
       </c>
       <c r="Z177" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG177" t="b">
         <v>0</v>
@@ -15284,7 +15356,7 @@
         </is>
       </c>
       <c r="Z178" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG178" t="b">
         <v>0</v>
@@ -15510,7 +15582,7 @@
         </is>
       </c>
       <c r="Z180" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG180" t="b">
         <v>0</v>
@@ -15625,7 +15697,7 @@
         </is>
       </c>
       <c r="Z181" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG181" t="b">
         <v>0</v>
@@ -15740,7 +15812,7 @@
         </is>
       </c>
       <c r="Z182" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG182" t="b">
         <v>0</v>
@@ -15855,13 +15927,13 @@
         </is>
       </c>
       <c r="Z183" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG183" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH183" t="b">
         <v>1</v>
-      </c>
-      <c r="AG183" t="b">
-        <v>0</v>
-      </c>
-      <c r="AH183" t="b">
-        <v>0</v>
       </c>
       <c r="AI183" t="inlineStr">
         <is>
@@ -15970,7 +16042,7 @@
         </is>
       </c>
       <c r="Z184" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG184" t="b">
         <v>0</v>
@@ -16085,7 +16157,7 @@
         </is>
       </c>
       <c r="Z185" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG185" t="b">
         <v>0</v>
@@ -16200,7 +16272,7 @@
         </is>
       </c>
       <c r="Z186" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG186" t="b">
         <v>0</v>
@@ -16315,7 +16387,7 @@
         </is>
       </c>
       <c r="Z187" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG187" t="b">
         <v>0</v>
@@ -16430,7 +16502,7 @@
         </is>
       </c>
       <c r="Z188" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG188" t="b">
         <v>0</v>
@@ -16545,7 +16617,7 @@
         </is>
       </c>
       <c r="Z189" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG189" t="b">
         <v>0</v>
@@ -16660,7 +16732,7 @@
         </is>
       </c>
       <c r="Z190" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG190" t="b">
         <v>0</v>
@@ -16775,13 +16847,13 @@
         </is>
       </c>
       <c r="Z191" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG191" t="b">
         <v>0</v>
       </c>
       <c r="AH191" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI191" t="inlineStr">
         <is>
@@ -16890,7 +16962,7 @@
         </is>
       </c>
       <c r="Z192" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG192" t="b">
         <v>0</v>
@@ -17005,7 +17077,7 @@
         </is>
       </c>
       <c r="Z193" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG193" t="b">
         <v>0</v>
@@ -17120,7 +17192,7 @@
         </is>
       </c>
       <c r="Z194" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG194" t="b">
         <v>0</v>
@@ -17235,7 +17307,7 @@
         </is>
       </c>
       <c r="Z195" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG195" t="b">
         <v>0</v>
@@ -17350,7 +17422,7 @@
         </is>
       </c>
       <c r="Z196" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG196" t="b">
         <v>0</v>
@@ -17465,7 +17537,7 @@
         </is>
       </c>
       <c r="Z197" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG197" t="b">
         <v>0</v>
@@ -17802,7 +17874,7 @@
         </is>
       </c>
       <c r="Z200" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG200" t="b">
         <v>0</v>
@@ -17917,7 +17989,7 @@
         </is>
       </c>
       <c r="Z201" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG201" t="b">
         <v>0</v>
@@ -18032,7 +18104,7 @@
         </is>
       </c>
       <c r="Z202" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG202" t="b">
         <v>0</v>
@@ -18046,8 +18118,1729 @@
         </is>
       </c>
     </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>1605</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>華新</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E203" t="n">
+        <v>70.38</v>
+      </c>
+      <c r="F203" t="n">
+        <v>50.9</v>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I203" t="b">
+        <v>0</v>
+      </c>
+      <c r="J203" t="n">
+        <v>10</v>
+      </c>
+      <c r="K203" t="n">
+        <v>43.34</v>
+      </c>
+      <c r="L203" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M203" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N203" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="O203" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="P203" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="Q203" t="n">
+        <v>55.99</v>
+      </c>
+      <c r="R203" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S203" t="n">
+        <v>7</v>
+      </c>
+      <c r="T203" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U203" t="inlineStr">
+        <is>
+          <t>unclassified</t>
+        </is>
+      </c>
+      <c r="V203" t="n">
+        <v>39.4</v>
+      </c>
+      <c r="W203" t="n">
+        <v>47.28</v>
+      </c>
+      <c r="X203" t="n">
+        <v>36.642</v>
+      </c>
+      <c r="Y203" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z203" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG203" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH203" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI203" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>2301</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>光寶科</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E204" t="n">
+        <v>85.06999999999999</v>
+      </c>
+      <c r="F204" t="n">
+        <v>37.73</v>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I204" t="b">
+        <v>0</v>
+      </c>
+      <c r="J204" t="n">
+        <v>8.449999999999999</v>
+      </c>
+      <c r="K204" t="n">
+        <v>332.93</v>
+      </c>
+      <c r="L204" t="inlineStr">
+        <is>
+          <t>gap_MM_Target_Up</t>
+        </is>
+      </c>
+      <c r="M204" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="N204" t="n">
+        <v>3</v>
+      </c>
+      <c r="O204" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P204" t="n">
+        <v>281.75</v>
+      </c>
+      <c r="Q204" t="n">
+        <v>71.55</v>
+      </c>
+      <c r="R204" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="S204" t="n">
+        <v>7</v>
+      </c>
+      <c r="T204" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U204" t="inlineStr">
+        <is>
+          <t>ai_hardware</t>
+        </is>
+      </c>
+      <c r="V204" t="n">
+        <v>307</v>
+      </c>
+      <c r="W204" t="n">
+        <v>368.4</v>
+      </c>
+      <c r="X204" t="n">
+        <v>285.51</v>
+      </c>
+      <c r="Y204" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z204" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG204" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH204" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI204" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>2313</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>華通</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E205" t="n">
+        <v>72.44</v>
+      </c>
+      <c r="F205" t="n">
+        <v>53.31</v>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I205" t="b">
+        <v>0</v>
+      </c>
+      <c r="J205" t="n">
+        <v>10</v>
+      </c>
+      <c r="K205" t="n">
+        <v>244.2</v>
+      </c>
+      <c r="L205" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M205" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N205" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="O205" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="P205" t="n">
+        <v>214.5</v>
+      </c>
+      <c r="Q205" t="n">
+        <v>58.72</v>
+      </c>
+      <c r="R205" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S205" t="n">
+        <v>7</v>
+      </c>
+      <c r="T205" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U205" t="inlineStr">
+        <is>
+          <t>unclassified</t>
+        </is>
+      </c>
+      <c r="V205" t="n">
+        <v>222</v>
+      </c>
+      <c r="W205" t="n">
+        <v>266.4</v>
+      </c>
+      <c r="X205" t="n">
+        <v>206.46</v>
+      </c>
+      <c r="Y205" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z205" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG205" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH205" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI205" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>2324</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>仁寶</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E206" t="n">
+        <v>76.70999999999999</v>
+      </c>
+      <c r="F206" t="n">
+        <v>58.33</v>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I206" t="b">
+        <v>0</v>
+      </c>
+      <c r="J206" t="n">
+        <v>10.01</v>
+      </c>
+      <c r="K206" t="n">
+        <v>45.05</v>
+      </c>
+      <c r="L206" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M206" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N206" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="O206" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="P206" t="n">
+        <v>40.3</v>
+      </c>
+      <c r="Q206" t="n">
+        <v>58.9</v>
+      </c>
+      <c r="R206" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S206" t="n">
+        <v>7</v>
+      </c>
+      <c r="T206" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U206" t="inlineStr">
+        <is>
+          <t>ai_hardware</t>
+        </is>
+      </c>
+      <c r="V206" t="n">
+        <v>40.95</v>
+      </c>
+      <c r="W206" t="n">
+        <v>49.14</v>
+      </c>
+      <c r="X206" t="n">
+        <v>38.0835</v>
+      </c>
+      <c r="Y206" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z206" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG206" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH206" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI206" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>2357</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>華碩</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E207" t="n">
+        <v>76.02</v>
+      </c>
+      <c r="F207" t="n">
+        <v>51.14</v>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I207" t="b">
+        <v>0</v>
+      </c>
+      <c r="J207" t="n">
+        <v>10</v>
+      </c>
+      <c r="K207" t="n">
+        <v>1068.1</v>
+      </c>
+      <c r="L207" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M207" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N207" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="O207" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="P207" t="n">
+        <v>918.5</v>
+      </c>
+      <c r="Q207" t="n">
+        <v>64.27</v>
+      </c>
+      <c r="R207" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="S207" t="n">
+        <v>7</v>
+      </c>
+      <c r="T207" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U207" t="inlineStr">
+        <is>
+          <t>ai_hardware</t>
+        </is>
+      </c>
+      <c r="V207" t="n">
+        <v>971</v>
+      </c>
+      <c r="W207" t="n">
+        <v>1165.2</v>
+      </c>
+      <c r="X207" t="n">
+        <v>903.03</v>
+      </c>
+      <c r="Y207" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z207" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG207" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH207" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI207" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>2395</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>研華</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E208" t="n">
+        <v>77.69</v>
+      </c>
+      <c r="F208" t="n">
+        <v>53.17</v>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I208" t="b">
+        <v>0</v>
+      </c>
+      <c r="J208" t="n">
+        <v>10</v>
+      </c>
+      <c r="K208" t="n">
+        <v>756.8</v>
+      </c>
+      <c r="L208" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M208" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N208" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="O208" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="P208" t="n">
+        <v>676</v>
+      </c>
+      <c r="Q208" t="n">
+        <v>51.12</v>
+      </c>
+      <c r="R208" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S208" t="n">
+        <v>7</v>
+      </c>
+      <c r="T208" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U208" t="inlineStr">
+        <is>
+          <t>ai_hardware</t>
+        </is>
+      </c>
+      <c r="V208" t="n">
+        <v>688</v>
+      </c>
+      <c r="W208" t="n">
+        <v>825.6</v>
+      </c>
+      <c r="X208" t="n">
+        <v>639.84</v>
+      </c>
+      <c r="Y208" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z208" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG208" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH208" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI208" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>2408</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>南亞科</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E209" t="n">
+        <v>77.19</v>
+      </c>
+      <c r="F209" t="n">
+        <v>53.77</v>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I209" t="b">
+        <v>0</v>
+      </c>
+      <c r="J209" t="n">
+        <v>10</v>
+      </c>
+      <c r="K209" t="n">
+        <v>568.7</v>
+      </c>
+      <c r="L209" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M209" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N209" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="O209" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="P209" t="n">
+        <v>513.5</v>
+      </c>
+      <c r="Q209" t="n">
+        <v>61.82</v>
+      </c>
+      <c r="R209" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="S209" t="n">
+        <v>7</v>
+      </c>
+      <c r="T209" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U209" t="inlineStr">
+        <is>
+          <t>semiconductor</t>
+        </is>
+      </c>
+      <c r="V209" t="n">
+        <v>517</v>
+      </c>
+      <c r="W209" t="n">
+        <v>620.4</v>
+      </c>
+      <c r="X209" t="n">
+        <v>480.81</v>
+      </c>
+      <c r="Y209" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z209" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG209" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH209" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI209" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>2887</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>台新金</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E210" t="n">
+        <v>73.09</v>
+      </c>
+      <c r="F210" t="n">
+        <v>63.62</v>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I210" t="b">
+        <v>0</v>
+      </c>
+      <c r="J210" t="n">
+        <v>10</v>
+      </c>
+      <c r="K210" t="n">
+        <v>41.25</v>
+      </c>
+      <c r="L210" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M210" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="N210" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="O210" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="P210" t="n">
+        <v>36.55</v>
+      </c>
+      <c r="Q210" t="n">
+        <v>54.16</v>
+      </c>
+      <c r="R210" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S210" t="n">
+        <v>6.47</v>
+      </c>
+      <c r="T210" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U210" t="inlineStr">
+        <is>
+          <t>finance</t>
+        </is>
+      </c>
+      <c r="V210" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="W210" t="n">
+        <v>44.0657</v>
+      </c>
+      <c r="X210" t="n">
+        <v>35.0737</v>
+      </c>
+      <c r="Y210" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z210" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG210" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH210" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI210" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>3037</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>欣興</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E211" t="n">
+        <v>76.44</v>
+      </c>
+      <c r="F211" t="n">
+        <v>45.54</v>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I211" t="b">
+        <v>0</v>
+      </c>
+      <c r="J211" t="n">
+        <v>10</v>
+      </c>
+      <c r="K211" t="n">
+        <v>1276</v>
+      </c>
+      <c r="L211" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M211" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N211" t="n">
+        <v>1</v>
+      </c>
+      <c r="O211" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P211" t="n">
+        <v>1086</v>
+      </c>
+      <c r="Q211" t="n">
+        <v>56.92</v>
+      </c>
+      <c r="R211" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S211" t="n">
+        <v>7</v>
+      </c>
+      <c r="T211" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U211" t="inlineStr">
+        <is>
+          <t>electronic_components</t>
+        </is>
+      </c>
+      <c r="V211" t="n">
+        <v>1160</v>
+      </c>
+      <c r="W211" t="n">
+        <v>1392</v>
+      </c>
+      <c r="X211" t="n">
+        <v>1078.8</v>
+      </c>
+      <c r="Y211" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z211" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG211" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH211" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI211" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>3189</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>景碩</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E212" t="n">
+        <v>77.69</v>
+      </c>
+      <c r="F212" t="n">
+        <v>51.1</v>
+      </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I212" t="b">
+        <v>0</v>
+      </c>
+      <c r="J212" t="n">
+        <v>10</v>
+      </c>
+      <c r="K212" t="n">
+        <v>969.1</v>
+      </c>
+      <c r="L212" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M212" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N212" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="O212" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="P212" t="n">
+        <v>851.5</v>
+      </c>
+      <c r="Q212" t="n">
+        <v>57.31</v>
+      </c>
+      <c r="R212" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S212" t="n">
+        <v>7</v>
+      </c>
+      <c r="T212" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U212" t="inlineStr">
+        <is>
+          <t>unclassified</t>
+        </is>
+      </c>
+      <c r="V212" t="n">
+        <v>881</v>
+      </c>
+      <c r="W212" t="n">
+        <v>1057.2</v>
+      </c>
+      <c r="X212" t="n">
+        <v>819.33</v>
+      </c>
+      <c r="Y212" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z212" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG212" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH212" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI212" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>3324</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>雙鴻</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E213" t="n">
+        <v>75.58</v>
+      </c>
+      <c r="F213" t="n">
+        <v>49.8</v>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I213" t="b">
+        <v>0</v>
+      </c>
+      <c r="J213" t="n">
+        <v>10</v>
+      </c>
+      <c r="K213" t="n">
+        <v>1182.5</v>
+      </c>
+      <c r="L213" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M213" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N213" t="n">
+        <v>5</v>
+      </c>
+      <c r="O213" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="P213" t="n">
+        <v>1020</v>
+      </c>
+      <c r="Q213" t="n">
+        <v>58.67</v>
+      </c>
+      <c r="R213" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S213" t="n">
+        <v>7</v>
+      </c>
+      <c r="T213" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U213" t="inlineStr">
+        <is>
+          <t>unclassified</t>
+        </is>
+      </c>
+      <c r="V213" t="n">
+        <v>1075</v>
+      </c>
+      <c r="W213" t="n">
+        <v>1290</v>
+      </c>
+      <c r="X213" t="n">
+        <v>999.75</v>
+      </c>
+      <c r="Y213" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="AI213" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="AJ213" t="inlineStr">
+        <is>
+          <t>market_data_temporarily_unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>3661</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>世芯-KY</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E214" t="n">
+        <v>71.90000000000001</v>
+      </c>
+      <c r="F214" t="n">
+        <v>57.46</v>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I214" t="b">
+        <v>0</v>
+      </c>
+      <c r="J214" t="n">
+        <v>10</v>
+      </c>
+      <c r="K214" t="n">
+        <v>4356</v>
+      </c>
+      <c r="L214" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M214" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N214" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="O214" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="P214" t="n">
+        <v>4057.5</v>
+      </c>
+      <c r="Q214" t="n">
+        <v>59.71</v>
+      </c>
+      <c r="R214" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S214" t="n">
+        <v>7</v>
+      </c>
+      <c r="T214" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U214" t="inlineStr">
+        <is>
+          <t>semiconductor</t>
+        </is>
+      </c>
+      <c r="V214" t="n">
+        <v>3960</v>
+      </c>
+      <c r="W214" t="n">
+        <v>4752</v>
+      </c>
+      <c r="X214" t="n">
+        <v>3682.8</v>
+      </c>
+      <c r="Y214" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z214" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG214" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH214" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI214" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>6446</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>藥華藥</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E215" t="n">
+        <v>73.88</v>
+      </c>
+      <c r="F215" t="n">
+        <v>40.33</v>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I215" t="b">
+        <v>0</v>
+      </c>
+      <c r="J215" t="n">
+        <v>10</v>
+      </c>
+      <c r="K215" t="n">
+        <v>1743.5</v>
+      </c>
+      <c r="L215" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M215" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N215" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="O215" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P215" t="n">
+        <v>1465</v>
+      </c>
+      <c r="Q215" t="n">
+        <v>58.88</v>
+      </c>
+      <c r="R215" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S215" t="n">
+        <v>7</v>
+      </c>
+      <c r="T215" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U215" t="inlineStr">
+        <is>
+          <t>unclassified</t>
+        </is>
+      </c>
+      <c r="V215" t="n">
+        <v>1585</v>
+      </c>
+      <c r="W215" t="n">
+        <v>1902</v>
+      </c>
+      <c r="X215" t="n">
+        <v>1474.05</v>
+      </c>
+      <c r="Y215" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z215" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG215" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH215" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI215" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>6472</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>保瑞</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E216" t="n">
+        <v>73.58</v>
+      </c>
+      <c r="F216" t="n">
+        <v>46.63</v>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I216" t="b">
+        <v>0</v>
+      </c>
+      <c r="J216" t="n">
+        <v>10</v>
+      </c>
+      <c r="K216" t="n">
+        <v>502.7</v>
+      </c>
+      <c r="L216" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M216" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N216" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="O216" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P216" t="n">
+        <v>438</v>
+      </c>
+      <c r="Q216" t="n">
+        <v>60.89</v>
+      </c>
+      <c r="R216" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="S216" t="n">
+        <v>7</v>
+      </c>
+      <c r="T216" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U216" t="inlineStr">
+        <is>
+          <t>unclassified</t>
+        </is>
+      </c>
+      <c r="V216" t="n">
+        <v>457</v>
+      </c>
+      <c r="W216" t="n">
+        <v>548.4</v>
+      </c>
+      <c r="X216" t="n">
+        <v>425.01</v>
+      </c>
+      <c r="Y216" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z216" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG216" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH216" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI216" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>6669</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>緯穎</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E217" t="n">
+        <v>82.37</v>
+      </c>
+      <c r="F217" t="n">
+        <v>50.07</v>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I217" t="b">
+        <v>0</v>
+      </c>
+      <c r="J217" t="n">
+        <v>10</v>
+      </c>
+      <c r="K217" t="n">
+        <v>7463.5</v>
+      </c>
+      <c r="L217" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M217" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N217" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="O217" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="P217" t="n">
+        <v>6390</v>
+      </c>
+      <c r="Q217" t="n">
+        <v>77.11</v>
+      </c>
+      <c r="R217" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="S217" t="n">
+        <v>7</v>
+      </c>
+      <c r="T217" t="inlineStr">
+        <is>
+          <t>RangeRotation</t>
+        </is>
+      </c>
+      <c r="U217" t="inlineStr">
+        <is>
+          <t>semiconductor</t>
+        </is>
+      </c>
+      <c r="V217" t="n">
+        <v>6785</v>
+      </c>
+      <c r="W217" t="n">
+        <v>8142</v>
+      </c>
+      <c r="X217" t="n">
+        <v>6310.05</v>
+      </c>
+      <c r="Y217" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z217" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG217" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH217" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI217" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AJ202"/>
+  <autoFilter ref="A1:AJ217"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -18297,7 +20090,7 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>2026-08-25 14:23:08</t>
+          <t>2026-08-26 14:24:03</t>
         </is>
       </c>
     </row>
@@ -18344,7 +20137,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>201</v>
+        <v>216</v>
       </c>
     </row>
     <row r="7">
@@ -18364,7 +20157,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>201</v>
+        <v>216</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-08-27 06:24:39
</commit_message>
<xml_diff>
--- a/data/swing_performance_analysis.xlsx
+++ b/data/swing_performance_analysis.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'T20_Tracking'!$A$1:$AJ$217</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'T20_Tracking'!$A$1:$AJ$242</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ217"/>
+  <dimension ref="A1:AJ242"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -731,7 +731,7 @@
         </is>
       </c>
       <c r="Z2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="AA2" t="n">
         <v>-1.45</v>
@@ -803,7 +803,7 @@
         </is>
       </c>
       <c r="Z3" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="AA3" t="n">
         <v>-5.5</v>
@@ -875,7 +875,7 @@
         </is>
       </c>
       <c r="Z4" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="AA4" t="n">
         <v>21.91</v>
@@ -947,7 +947,7 @@
         </is>
       </c>
       <c r="Z5" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="AA5" t="n">
         <v>3.92</v>
@@ -1019,7 +1019,7 @@
         </is>
       </c>
       <c r="Z6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="AA6" t="n">
         <v>7.73</v>
@@ -1091,7 +1091,7 @@
         </is>
       </c>
       <c r="Z7" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="AA7" t="n">
         <v>5.54</v>
@@ -1163,7 +1163,7 @@
         </is>
       </c>
       <c r="Z8" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="AA8" t="n">
         <v>-11.56</v>
@@ -1235,7 +1235,7 @@
         </is>
       </c>
       <c r="Z9" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="AA9" t="n">
         <v>-10.14</v>
@@ -1307,7 +1307,7 @@
         </is>
       </c>
       <c r="Z10" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="AA10" t="n">
         <v>-12.27</v>
@@ -1379,7 +1379,7 @@
         </is>
       </c>
       <c r="Z11" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="AA11" t="n">
         <v>-6.97</v>
@@ -1451,7 +1451,7 @@
         </is>
       </c>
       <c r="Z12" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="AA12" t="n">
         <v>5.13</v>
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="Z13" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="AA13" t="n">
         <v>-5.54</v>
@@ -1657,7 +1657,7 @@
         </is>
       </c>
       <c r="Z15" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="AA15" t="n">
         <v>3.09</v>
@@ -1729,7 +1729,7 @@
         </is>
       </c>
       <c r="Z16" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="AA16" t="n">
         <v>9.31</v>
@@ -1801,7 +1801,7 @@
         </is>
       </c>
       <c r="Z17" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AA17" t="n">
         <v>-1.43</v>
@@ -1873,7 +1873,7 @@
         </is>
       </c>
       <c r="Z18" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AA18" t="n">
         <v>-6.69</v>
@@ -1945,7 +1945,7 @@
         </is>
       </c>
       <c r="Z19" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AA19" t="n">
         <v>-4.07</v>
@@ -2017,7 +2017,7 @@
         </is>
       </c>
       <c r="Z20" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AA20" t="n">
         <v>-1.42</v>
@@ -2089,7 +2089,7 @@
         </is>
       </c>
       <c r="Z21" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AA21" t="n">
         <v>-3.59</v>
@@ -2161,7 +2161,7 @@
         </is>
       </c>
       <c r="Z22" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AA22" t="n">
         <v>14.67</v>
@@ -2233,7 +2233,7 @@
         </is>
       </c>
       <c r="Z23" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AA23" t="n">
         <v>2.43</v>
@@ -2305,7 +2305,7 @@
         </is>
       </c>
       <c r="Z24" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AA24" t="n">
         <v>1.05</v>
@@ -2377,7 +2377,7 @@
         </is>
       </c>
       <c r="Z25" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AA25" t="n">
         <v>8.18</v>
@@ -2449,7 +2449,7 @@
         </is>
       </c>
       <c r="Z26" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AA26" t="n">
         <v>6.01</v>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="Z27" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AA27" t="n">
         <v>13.83</v>
@@ -2593,7 +2593,7 @@
         </is>
       </c>
       <c r="Z28" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AA28" t="n">
         <v>-10.91</v>
@@ -2665,7 +2665,7 @@
         </is>
       </c>
       <c r="Z29" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AA29" t="n">
         <v>-2.87</v>
@@ -2737,7 +2737,7 @@
         </is>
       </c>
       <c r="Z30" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AA30" t="n">
         <v>-8.630000000000001</v>
@@ -2809,7 +2809,7 @@
         </is>
       </c>
       <c r="Z31" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AA31" t="n">
         <v>-0.91</v>
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Z32" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AA32" t="n">
         <v>-6.43</v>
@@ -2953,7 +2953,7 @@
         </is>
       </c>
       <c r="Z33" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AA33" t="n">
         <v>-3.11</v>
@@ -3149,7 +3149,7 @@
         </is>
       </c>
       <c r="Z36" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AA36" t="n">
         <v>-3.48</v>
@@ -3221,7 +3221,7 @@
         </is>
       </c>
       <c r="Z37" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AA37" t="n">
         <v>10.15</v>
@@ -3293,7 +3293,7 @@
         </is>
       </c>
       <c r="Z38" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AA38" t="n">
         <v>-5.23</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="Z39" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA39" t="n">
         <v>-5.13</v>
@@ -3437,7 +3437,7 @@
         </is>
       </c>
       <c r="Z40" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA40" t="n">
         <v>-3.13</v>
@@ -3509,7 +3509,7 @@
         </is>
       </c>
       <c r="Z41" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA41" t="n">
         <v>-4.05</v>
@@ -3581,7 +3581,7 @@
         </is>
       </c>
       <c r="Z42" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA42" t="n">
         <v>1.86</v>
@@ -3653,7 +3653,7 @@
         </is>
       </c>
       <c r="Z43" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA43" t="n">
         <v>8.460000000000001</v>
@@ -3725,7 +3725,7 @@
         </is>
       </c>
       <c r="Z44" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA44" t="n">
         <v>10.82</v>
@@ -3797,7 +3797,7 @@
         </is>
       </c>
       <c r="Z45" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA45" t="n">
         <v>-0.71</v>
@@ -3869,7 +3869,7 @@
         </is>
       </c>
       <c r="Z46" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA46" t="n">
         <v>12.1</v>
@@ -3941,7 +3941,7 @@
         </is>
       </c>
       <c r="Z47" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA47" t="n">
         <v>2.72</v>
@@ -4013,7 +4013,7 @@
         </is>
       </c>
       <c r="Z48" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA48" t="n">
         <v>5.32</v>
@@ -4085,7 +4085,7 @@
         </is>
       </c>
       <c r="Z49" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA49" t="n">
         <v>-3.36</v>
@@ -4157,7 +4157,7 @@
         </is>
       </c>
       <c r="Z50" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA50" t="n">
         <v>9.17</v>
@@ -4229,7 +4229,7 @@
         </is>
       </c>
       <c r="Z51" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA51" t="n">
         <v>8.08</v>
@@ -4301,7 +4301,7 @@
         </is>
       </c>
       <c r="Z52" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA52" t="n">
         <v>20.55</v>
@@ -4373,7 +4373,7 @@
         </is>
       </c>
       <c r="Z53" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA53" t="n">
         <v>-0.32</v>
@@ -4445,7 +4445,7 @@
         </is>
       </c>
       <c r="Z54" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA54" t="n">
         <v>-5.24</v>
@@ -4579,7 +4579,7 @@
         </is>
       </c>
       <c r="Z56" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA56" t="n">
         <v>-4.49</v>
@@ -4651,7 +4651,7 @@
         </is>
       </c>
       <c r="Z57" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA57" t="n">
         <v>-0.28</v>
@@ -4723,7 +4723,7 @@
         </is>
       </c>
       <c r="Z58" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA58" t="n">
         <v>-8.779999999999999</v>
@@ -4795,7 +4795,7 @@
         </is>
       </c>
       <c r="Z59" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA59" t="n">
         <v>-4.05</v>
@@ -4867,7 +4867,7 @@
         </is>
       </c>
       <c r="Z60" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA60" t="n">
         <v>-9.26</v>
@@ -4939,7 +4939,7 @@
         </is>
       </c>
       <c r="Z61" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA61" t="n">
         <v>8.57</v>
@@ -5011,7 +5011,7 @@
         </is>
       </c>
       <c r="Z62" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA62" t="n">
         <v>-3.42</v>
@@ -5083,7 +5083,7 @@
         </is>
       </c>
       <c r="Z63" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA63" t="n">
         <v>2.62</v>
@@ -5155,7 +5155,7 @@
         </is>
       </c>
       <c r="Z64" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA64" t="n">
         <v>1.17</v>
@@ -5227,7 +5227,7 @@
         </is>
       </c>
       <c r="Z65" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA65" t="n">
         <v>12.12</v>
@@ -5299,7 +5299,7 @@
         </is>
       </c>
       <c r="Z66" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA66" t="n">
         <v>-1.13</v>
@@ -5371,7 +5371,7 @@
         </is>
       </c>
       <c r="Z67" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA67" t="n">
         <v>21.05</v>
@@ -5443,7 +5443,7 @@
         </is>
       </c>
       <c r="Z68" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA68" t="n">
         <v>6.36</v>
@@ -5515,7 +5515,7 @@
         </is>
       </c>
       <c r="Z69" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA69" t="n">
         <v>-5.94</v>
@@ -5649,7 +5649,7 @@
         </is>
       </c>
       <c r="Z71" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA71" t="n">
         <v>3.22</v>
@@ -5658,7 +5658,7 @@
         <v>19.4</v>
       </c>
       <c r="AG71" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH71" t="b">
         <v>0</v>
@@ -5721,7 +5721,7 @@
         </is>
       </c>
       <c r="Z72" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA72" t="n">
         <v>-2.78</v>
@@ -5793,7 +5793,7 @@
         </is>
       </c>
       <c r="Z73" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA73" t="n">
         <v>5.81</v>
@@ -5865,7 +5865,7 @@
         </is>
       </c>
       <c r="Z74" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AA74" t="n">
         <v>-5.04</v>
@@ -5937,11 +5937,14 @@
         </is>
       </c>
       <c r="Z75" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA75" t="n">
         <v>0.97</v>
       </c>
+      <c r="AB75" t="n">
+        <v>6.94</v>
+      </c>
       <c r="AG75" t="b">
         <v>0</v>
       </c>
@@ -6006,11 +6009,14 @@
         </is>
       </c>
       <c r="Z76" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA76" t="n">
         <v>-3.4</v>
       </c>
+      <c r="AB76" t="n">
+        <v>0.68</v>
+      </c>
       <c r="AG76" t="b">
         <v>0</v>
       </c>
@@ -6075,11 +6081,14 @@
         </is>
       </c>
       <c r="Z77" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA77" t="n">
         <v>-0.93</v>
       </c>
+      <c r="AB77" t="n">
+        <v>11.69</v>
+      </c>
       <c r="AG77" t="b">
         <v>0</v>
       </c>
@@ -6144,11 +6153,14 @@
         </is>
       </c>
       <c r="Z78" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA78" t="n">
         <v>-12.58</v>
       </c>
+      <c r="AB78" t="n">
+        <v>-12.33</v>
+      </c>
       <c r="AG78" t="b">
         <v>0</v>
       </c>
@@ -6213,11 +6225,14 @@
         </is>
       </c>
       <c r="Z79" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA79" t="n">
         <v>-3.58</v>
       </c>
+      <c r="AB79" t="n">
+        <v>-3.3</v>
+      </c>
       <c r="AG79" t="b">
         <v>0</v>
       </c>
@@ -6282,11 +6297,14 @@
         </is>
       </c>
       <c r="Z80" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA80" t="n">
         <v>0.58</v>
       </c>
+      <c r="AB80" t="n">
+        <v>5.25</v>
+      </c>
       <c r="AG80" t="b">
         <v>0</v>
       </c>
@@ -6351,11 +6369,14 @@
         </is>
       </c>
       <c r="Z81" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA81" t="n">
         <v>14.15</v>
       </c>
+      <c r="AB81" t="n">
+        <v>7.89</v>
+      </c>
       <c r="AG81" t="b">
         <v>1</v>
       </c>
@@ -6420,11 +6441,14 @@
         </is>
       </c>
       <c r="Z82" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA82" t="n">
         <v>29.71</v>
       </c>
+      <c r="AB82" t="n">
+        <v>29.71</v>
+      </c>
       <c r="AG82" t="b">
         <v>1</v>
       </c>
@@ -6489,11 +6513,14 @@
         </is>
       </c>
       <c r="Z83" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA83" t="n">
         <v>-1.5</v>
       </c>
+      <c r="AB83" t="n">
+        <v>-1.5</v>
+      </c>
       <c r="AG83" t="b">
         <v>0</v>
       </c>
@@ -6558,11 +6585,14 @@
         </is>
       </c>
       <c r="Z84" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA84" t="n">
         <v>18.35</v>
       </c>
+      <c r="AB84" t="n">
+        <v>48.39</v>
+      </c>
       <c r="AG84" t="b">
         <v>1</v>
       </c>
@@ -6627,11 +6657,14 @@
         </is>
       </c>
       <c r="Z85" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA85" t="n">
         <v>-8.630000000000001</v>
       </c>
+      <c r="AB85" t="n">
+        <v>-8.880000000000001</v>
+      </c>
       <c r="AG85" t="b">
         <v>0</v>
       </c>
@@ -6696,11 +6729,14 @@
         </is>
       </c>
       <c r="Z86" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA86" t="n">
         <v>1.62</v>
       </c>
+      <c r="AB86" t="n">
+        <v>6.86</v>
+      </c>
       <c r="AG86" t="b">
         <v>0</v>
       </c>
@@ -6765,11 +6801,14 @@
         </is>
       </c>
       <c r="Z87" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA87" t="n">
         <v>-10.5</v>
       </c>
+      <c r="AB87" t="n">
+        <v>-7.64</v>
+      </c>
       <c r="AG87" t="b">
         <v>0</v>
       </c>
@@ -6834,11 +6873,14 @@
         </is>
       </c>
       <c r="Z88" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA88" t="n">
         <v>-4.84</v>
       </c>
+      <c r="AB88" t="n">
+        <v>7.96</v>
+      </c>
       <c r="AG88" t="b">
         <v>0</v>
       </c>
@@ -6903,11 +6945,14 @@
         </is>
       </c>
       <c r="Z89" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA89" t="n">
         <v>4.2</v>
       </c>
+      <c r="AB89" t="n">
+        <v>12.27</v>
+      </c>
       <c r="AG89" t="b">
         <v>0</v>
       </c>
@@ -7034,11 +7079,14 @@
         </is>
       </c>
       <c r="Z91" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AA91" t="n">
         <v>0.95</v>
       </c>
+      <c r="AB91" t="n">
+        <v>0</v>
+      </c>
       <c r="AG91" t="b">
         <v>0</v>
       </c>
@@ -7103,7 +7151,7 @@
         </is>
       </c>
       <c r="Z92" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA92" t="n">
         <v>1.83</v>
@@ -7172,7 +7220,7 @@
         </is>
       </c>
       <c r="Z93" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA93" t="n">
         <v>-1.71</v>
@@ -7241,7 +7289,7 @@
         </is>
       </c>
       <c r="Z94" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA94" t="n">
         <v>-2.25</v>
@@ -7310,7 +7358,7 @@
         </is>
       </c>
       <c r="Z95" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA95" t="n">
         <v>-14.59</v>
@@ -7379,7 +7427,7 @@
         </is>
       </c>
       <c r="Z96" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA96" t="n">
         <v>-11.01</v>
@@ -7448,7 +7496,7 @@
         </is>
       </c>
       <c r="Z97" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA97" t="n">
         <v>-7.87</v>
@@ -7517,7 +7565,7 @@
         </is>
       </c>
       <c r="Z98" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA98" t="n">
         <v>3.12</v>
@@ -7586,7 +7634,7 @@
         </is>
       </c>
       <c r="Z99" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA99" t="n">
         <v>-9.98</v>
@@ -7655,7 +7703,7 @@
         </is>
       </c>
       <c r="Z100" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA100" t="n">
         <v>14.84</v>
@@ -7724,7 +7772,7 @@
         </is>
       </c>
       <c r="Z101" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA101" t="n">
         <v>24.03</v>
@@ -7793,7 +7841,7 @@
         </is>
       </c>
       <c r="Z102" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA102" t="n">
         <v>37.42</v>
@@ -7862,7 +7910,7 @@
         </is>
       </c>
       <c r="Z103" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA103" t="n">
         <v>-0.32</v>
@@ -7931,7 +7979,7 @@
         </is>
       </c>
       <c r="Z104" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA104" t="n">
         <v>-1.32</v>
@@ -8000,7 +8048,7 @@
         </is>
       </c>
       <c r="Z105" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA105" t="n">
         <v>21.69</v>
@@ -8069,7 +8117,7 @@
         </is>
       </c>
       <c r="Z106" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA106" t="n">
         <v>-11.44</v>
@@ -8138,7 +8186,7 @@
         </is>
       </c>
       <c r="Z107" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA107" t="n">
         <v>6.37</v>
@@ -8207,7 +8255,7 @@
         </is>
       </c>
       <c r="Z108" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA108" t="n">
         <v>-5.92</v>
@@ -8276,7 +8324,7 @@
         </is>
       </c>
       <c r="Z109" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA109" t="n">
         <v>-9.300000000000001</v>
@@ -8345,7 +8393,7 @@
         </is>
       </c>
       <c r="Z110" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA110" t="n">
         <v>2.47</v>
@@ -8414,7 +8462,7 @@
         </is>
       </c>
       <c r="Z111" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA111" t="n">
         <v>-6.67</v>
@@ -8483,7 +8531,7 @@
         </is>
       </c>
       <c r="Z112" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA112" t="n">
         <v>-2.8</v>
@@ -8552,7 +8600,7 @@
         </is>
       </c>
       <c r="Z113" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA113" t="n">
         <v>-1.11</v>
@@ -8621,7 +8669,7 @@
         </is>
       </c>
       <c r="Z114" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA114" t="n">
         <v>-2.05</v>
@@ -8690,7 +8738,7 @@
         </is>
       </c>
       <c r="Z115" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA115" t="n">
         <v>-9.960000000000001</v>
@@ -8759,7 +8807,7 @@
         </is>
       </c>
       <c r="Z116" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA116" t="n">
         <v>8.92</v>
@@ -8828,7 +8876,7 @@
         </is>
       </c>
       <c r="Z117" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA117" t="n">
         <v>-1.6</v>
@@ -8897,7 +8945,7 @@
         </is>
       </c>
       <c r="Z118" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA118" t="n">
         <v>-12.29</v>
@@ -8966,7 +9014,7 @@
         </is>
       </c>
       <c r="Z119" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA119" t="n">
         <v>-14.49</v>
@@ -9035,7 +9083,7 @@
         </is>
       </c>
       <c r="Z120" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA120" t="n">
         <v>-4.39</v>
@@ -9104,7 +9152,7 @@
         </is>
       </c>
       <c r="Z121" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA121" t="n">
         <v>8.210000000000001</v>
@@ -9173,7 +9221,7 @@
         </is>
       </c>
       <c r="Z122" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA122" t="n">
         <v>17.92</v>
@@ -9242,7 +9290,7 @@
         </is>
       </c>
       <c r="Z123" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA123" t="n">
         <v>-1.27</v>
@@ -9311,7 +9359,7 @@
         </is>
       </c>
       <c r="Z124" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA124" t="n">
         <v>-8.640000000000001</v>
@@ -9380,7 +9428,7 @@
         </is>
       </c>
       <c r="Z125" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA125" t="n">
         <v>-1.75</v>
@@ -9449,7 +9497,7 @@
         </is>
       </c>
       <c r="Z126" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA126" t="n">
         <v>-9.369999999999999</v>
@@ -9518,7 +9566,7 @@
         </is>
       </c>
       <c r="Z127" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA127" t="n">
         <v>-6.15</v>
@@ -9587,7 +9635,7 @@
         </is>
       </c>
       <c r="Z128" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA128" t="n">
         <v>-8.289999999999999</v>
@@ -9656,7 +9704,7 @@
         </is>
       </c>
       <c r="Z129" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA129" t="n">
         <v>-4.83</v>
@@ -9774,7 +9822,7 @@
         </is>
       </c>
       <c r="Z130" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA130" t="n">
         <v>0.42</v>
@@ -9892,7 +9940,7 @@
         </is>
       </c>
       <c r="Z131" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA131" t="n">
         <v>8.23</v>
@@ -10010,7 +10058,7 @@
         </is>
       </c>
       <c r="Z132" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA132" t="n">
         <v>0.49</v>
@@ -10128,7 +10176,7 @@
         </is>
       </c>
       <c r="Z133" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA133" t="n">
         <v>-9.25</v>
@@ -10246,7 +10294,7 @@
         </is>
       </c>
       <c r="Z134" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA134" t="n">
         <v>-9.83</v>
@@ -10364,7 +10412,7 @@
         </is>
       </c>
       <c r="Z135" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA135" t="n">
         <v>-0.97</v>
@@ -10482,7 +10530,7 @@
         </is>
       </c>
       <c r="Z136" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA136" t="n">
         <v>13.17</v>
@@ -10597,7 +10645,7 @@
         </is>
       </c>
       <c r="Z137" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA137" t="n">
         <v>9.27</v>
@@ -10715,7 +10763,7 @@
         </is>
       </c>
       <c r="Z138" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA138" t="n">
         <v>2.36</v>
@@ -10833,7 +10881,7 @@
         </is>
       </c>
       <c r="Z139" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA139" t="n">
         <v>0.68</v>
@@ -10951,13 +10999,13 @@
         </is>
       </c>
       <c r="Z140" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA140" t="n">
         <v>8.130000000000001</v>
       </c>
       <c r="AG140" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH140" t="b">
         <v>0</v>
@@ -11069,7 +11117,7 @@
         </is>
       </c>
       <c r="Z141" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA141" t="n">
         <v>-4.37</v>
@@ -11187,7 +11235,7 @@
         </is>
       </c>
       <c r="Z142" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA142" t="n">
         <v>-3.47</v>
@@ -11305,7 +11353,7 @@
         </is>
       </c>
       <c r="Z143" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA143" t="n">
         <v>0.63</v>
@@ -11423,7 +11471,7 @@
         </is>
       </c>
       <c r="Z144" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA144" t="n">
         <v>6.43</v>
@@ -11541,7 +11589,7 @@
         </is>
       </c>
       <c r="Z145" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA145" t="n">
         <v>0.63</v>
@@ -11659,7 +11707,7 @@
         </is>
       </c>
       <c r="Z146" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA146" t="n">
         <v>4.14</v>
@@ -11777,7 +11825,7 @@
         </is>
       </c>
       <c r="Z147" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA147" t="n">
         <v>0.26</v>
@@ -11895,7 +11943,7 @@
         </is>
       </c>
       <c r="Z148" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA148" t="n">
         <v>-0.14</v>
@@ -12013,7 +12061,7 @@
         </is>
       </c>
       <c r="Z149" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA149" t="n">
         <v>12.25</v>
@@ -12131,7 +12179,7 @@
         </is>
       </c>
       <c r="Z150" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA150" t="n">
         <v>-3.95</v>
@@ -12249,13 +12297,13 @@
         </is>
       </c>
       <c r="Z151" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA151" t="n">
         <v>13.33</v>
       </c>
       <c r="AG151" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH151" t="b">
         <v>0</v>
@@ -12367,7 +12415,7 @@
         </is>
       </c>
       <c r="Z152" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA152" t="n">
         <v>2.65</v>
@@ -12485,7 +12533,10 @@
         </is>
       </c>
       <c r="Z153" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA153" t="n">
+        <v>-2.82</v>
       </c>
       <c r="AG153" t="b">
         <v>0</v>
@@ -12600,7 +12651,10 @@
         </is>
       </c>
       <c r="Z154" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA154" t="n">
+        <v>1.15</v>
       </c>
       <c r="AG154" t="b">
         <v>0</v>
@@ -12715,7 +12769,10 @@
         </is>
       </c>
       <c r="Z155" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA155" t="n">
+        <v>-1.41</v>
       </c>
       <c r="AG155" t="b">
         <v>0</v>
@@ -12830,7 +12887,10 @@
         </is>
       </c>
       <c r="Z156" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA156" t="n">
+        <v>-2.74</v>
       </c>
       <c r="AG156" t="b">
         <v>0</v>
@@ -12945,7 +13005,10 @@
         </is>
       </c>
       <c r="Z157" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA157" t="n">
+        <v>5.91</v>
       </c>
       <c r="AG157" t="b">
         <v>0</v>
@@ -13060,7 +13123,10 @@
         </is>
       </c>
       <c r="Z158" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA158" t="n">
+        <v>-1.91</v>
       </c>
       <c r="AG158" t="b">
         <v>0</v>
@@ -13175,7 +13241,10 @@
         </is>
       </c>
       <c r="Z159" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA159" t="n">
+        <v>11.07</v>
       </c>
       <c r="AG159" t="b">
         <v>0</v>
@@ -13290,7 +13359,10 @@
         </is>
       </c>
       <c r="Z160" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA160" t="n">
+        <v>-8.1</v>
       </c>
       <c r="AG160" t="b">
         <v>0</v>
@@ -13405,7 +13477,10 @@
         </is>
       </c>
       <c r="Z161" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA161" t="n">
+        <v>-1.03</v>
       </c>
       <c r="AG161" t="b">
         <v>0</v>
@@ -13520,7 +13595,10 @@
         </is>
       </c>
       <c r="Z162" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA162" t="n">
+        <v>4.64</v>
       </c>
       <c r="AG162" t="b">
         <v>0</v>
@@ -13635,13 +13713,16 @@
         </is>
       </c>
       <c r="Z163" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA163" t="n">
+        <v>-4.52</v>
       </c>
       <c r="AG163" t="b">
         <v>0</v>
       </c>
       <c r="AH163" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI163" t="inlineStr">
         <is>
@@ -13750,7 +13831,10 @@
         </is>
       </c>
       <c r="Z164" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA164" t="n">
+        <v>-3.02</v>
       </c>
       <c r="AG164" t="b">
         <v>0</v>
@@ -13865,7 +13949,10 @@
         </is>
       </c>
       <c r="Z165" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA165" t="n">
+        <v>5.09</v>
       </c>
       <c r="AG165" t="b">
         <v>1</v>
@@ -13980,10 +14067,13 @@
         </is>
       </c>
       <c r="Z166" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA166" t="n">
+        <v>25.39</v>
       </c>
       <c r="AG166" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH166" t="b">
         <v>0</v>
@@ -14095,7 +14185,10 @@
         </is>
       </c>
       <c r="Z167" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA167" t="n">
+        <v>3.51</v>
       </c>
       <c r="AG167" t="b">
         <v>0</v>
@@ -14321,7 +14414,10 @@
         </is>
       </c>
       <c r="Z169" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA169" t="n">
+        <v>7.4</v>
       </c>
       <c r="AG169" t="b">
         <v>0</v>
@@ -14436,7 +14532,10 @@
         </is>
       </c>
       <c r="Z170" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA170" t="n">
+        <v>5.15</v>
       </c>
       <c r="AG170" t="b">
         <v>0</v>
@@ -14551,7 +14650,10 @@
         </is>
       </c>
       <c r="Z171" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="AA171" t="n">
+        <v>7.75</v>
       </c>
       <c r="AG171" t="b">
         <v>0</v>
@@ -14666,7 +14768,7 @@
         </is>
       </c>
       <c r="Z172" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG172" t="b">
         <v>0</v>
@@ -14781,7 +14883,7 @@
         </is>
       </c>
       <c r="Z173" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG173" t="b">
         <v>0</v>
@@ -14896,13 +14998,13 @@
         </is>
       </c>
       <c r="Z174" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG174" t="b">
         <v>0</v>
       </c>
       <c r="AH174" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI174" t="inlineStr">
         <is>
@@ -15011,7 +15113,7 @@
         </is>
       </c>
       <c r="Z175" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG175" t="b">
         <v>0</v>
@@ -15126,7 +15228,7 @@
         </is>
       </c>
       <c r="Z176" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG176" t="b">
         <v>0</v>
@@ -15241,7 +15343,7 @@
         </is>
       </c>
       <c r="Z177" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG177" t="b">
         <v>0</v>
@@ -15356,10 +15458,10 @@
         </is>
       </c>
       <c r="Z178" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG178" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH178" t="b">
         <v>0</v>
@@ -15582,7 +15684,7 @@
         </is>
       </c>
       <c r="Z180" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG180" t="b">
         <v>0</v>
@@ -15697,7 +15799,7 @@
         </is>
       </c>
       <c r="Z181" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG181" t="b">
         <v>0</v>
@@ -15812,7 +15914,7 @@
         </is>
       </c>
       <c r="Z182" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG182" t="b">
         <v>0</v>
@@ -15927,7 +16029,7 @@
         </is>
       </c>
       <c r="Z183" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG183" t="b">
         <v>0</v>
@@ -16042,10 +16144,10 @@
         </is>
       </c>
       <c r="Z184" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG184" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH184" t="b">
         <v>0</v>
@@ -16157,7 +16259,7 @@
         </is>
       </c>
       <c r="Z185" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG185" t="b">
         <v>0</v>
@@ -16272,7 +16374,7 @@
         </is>
       </c>
       <c r="Z186" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG186" t="b">
         <v>0</v>
@@ -16387,7 +16489,7 @@
         </is>
       </c>
       <c r="Z187" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG187" t="b">
         <v>0</v>
@@ -16502,7 +16604,7 @@
         </is>
       </c>
       <c r="Z188" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG188" t="b">
         <v>0</v>
@@ -16617,7 +16719,7 @@
         </is>
       </c>
       <c r="Z189" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG189" t="b">
         <v>0</v>
@@ -16732,7 +16834,7 @@
         </is>
       </c>
       <c r="Z190" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG190" t="b">
         <v>0</v>
@@ -16847,7 +16949,7 @@
         </is>
       </c>
       <c r="Z191" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG191" t="b">
         <v>0</v>
@@ -16962,7 +17064,7 @@
         </is>
       </c>
       <c r="Z192" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG192" t="b">
         <v>0</v>
@@ -17077,7 +17179,7 @@
         </is>
       </c>
       <c r="Z193" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG193" t="b">
         <v>0</v>
@@ -17192,7 +17294,7 @@
         </is>
       </c>
       <c r="Z194" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG194" t="b">
         <v>0</v>
@@ -17307,7 +17409,7 @@
         </is>
       </c>
       <c r="Z195" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG195" t="b">
         <v>0</v>
@@ -17422,10 +17524,10 @@
         </is>
       </c>
       <c r="Z196" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG196" t="b">
         <v>1</v>
-      </c>
-      <c r="AG196" t="b">
-        <v>0</v>
       </c>
       <c r="AH196" t="b">
         <v>0</v>
@@ -17537,7 +17639,7 @@
         </is>
       </c>
       <c r="Z197" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG197" t="b">
         <v>0</v>
@@ -17874,7 +17976,7 @@
         </is>
       </c>
       <c r="Z200" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG200" t="b">
         <v>0</v>
@@ -17989,7 +18091,7 @@
         </is>
       </c>
       <c r="Z201" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG201" t="b">
         <v>0</v>
@@ -18104,7 +18206,7 @@
         </is>
       </c>
       <c r="Z202" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG202" t="b">
         <v>0</v>
@@ -18219,7 +18321,7 @@
         </is>
       </c>
       <c r="Z203" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG203" t="b">
         <v>0</v>
@@ -18334,7 +18436,7 @@
         </is>
       </c>
       <c r="Z204" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG204" t="b">
         <v>0</v>
@@ -18449,7 +18551,7 @@
         </is>
       </c>
       <c r="Z205" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG205" t="b">
         <v>0</v>
@@ -18564,7 +18666,7 @@
         </is>
       </c>
       <c r="Z206" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG206" t="b">
         <v>0</v>
@@ -18679,7 +18781,7 @@
         </is>
       </c>
       <c r="Z207" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG207" t="b">
         <v>0</v>
@@ -18794,7 +18896,7 @@
         </is>
       </c>
       <c r="Z208" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG208" t="b">
         <v>0</v>
@@ -18909,7 +19011,7 @@
         </is>
       </c>
       <c r="Z209" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG209" t="b">
         <v>0</v>
@@ -19024,7 +19126,7 @@
         </is>
       </c>
       <c r="Z210" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG210" t="b">
         <v>0</v>
@@ -19139,7 +19241,7 @@
         </is>
       </c>
       <c r="Z211" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG211" t="b">
         <v>0</v>
@@ -19254,7 +19356,7 @@
         </is>
       </c>
       <c r="Z212" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG212" t="b">
         <v>0</v>
@@ -19480,7 +19582,7 @@
         </is>
       </c>
       <c r="Z214" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG214" t="b">
         <v>0</v>
@@ -19595,7 +19697,7 @@
         </is>
       </c>
       <c r="Z215" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG215" t="b">
         <v>0</v>
@@ -19710,7 +19812,7 @@
         </is>
       </c>
       <c r="Z216" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG216" t="b">
         <v>0</v>
@@ -19825,7 +19927,7 @@
         </is>
       </c>
       <c r="Z217" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG217" t="b">
         <v>0</v>
@@ -19839,8 +19941,2871 @@
         </is>
       </c>
     </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>1301</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>台塑</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E218" t="n">
+        <v>77.64</v>
+      </c>
+      <c r="F218" t="n">
+        <v>53.07</v>
+      </c>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I218" t="b">
+        <v>0</v>
+      </c>
+      <c r="J218" t="n">
+        <v>10</v>
+      </c>
+      <c r="K218" t="n">
+        <v>69.41</v>
+      </c>
+      <c r="L218" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M218" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N218" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="O218" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="P218" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q218" t="n">
+        <v>70.47</v>
+      </c>
+      <c r="R218" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="S218" t="n">
+        <v>7</v>
+      </c>
+      <c r="T218" t="inlineStr">
+        <is>
+          <t>BullTrend</t>
+        </is>
+      </c>
+      <c r="U218" t="inlineStr">
+        <is>
+          <t>materials</t>
+        </is>
+      </c>
+      <c r="V218" t="n">
+        <v>63.1</v>
+      </c>
+      <c r="W218" t="n">
+        <v>75.72</v>
+      </c>
+      <c r="X218" t="n">
+        <v>58.683</v>
+      </c>
+      <c r="Y218" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z218" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG218" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH218" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI218" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>1504</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>東元</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>swing_buy_confirmed</t>
+        </is>
+      </c>
+      <c r="E219" t="n">
+        <v>82.47</v>
+      </c>
+      <c r="F219" t="n">
+        <v>68.93000000000001</v>
+      </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="H219" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I219" t="b">
+        <v>0</v>
+      </c>
+      <c r="J219" t="n">
+        <v>10</v>
+      </c>
+      <c r="K219" t="n">
+        <v>80.73999999999999</v>
+      </c>
+      <c r="L219" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M219" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="N219" t="n">
+        <v>10</v>
+      </c>
+      <c r="O219" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="P219" t="n">
+        <v>71.34999999999999</v>
+      </c>
+      <c r="Q219" t="n">
+        <v>52.88</v>
+      </c>
+      <c r="R219" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S219" t="n">
+        <v>5.3801</v>
+      </c>
+      <c r="T219" t="inlineStr">
+        <is>
+          <t>BullTrend</t>
+        </is>
+      </c>
+      <c r="U219" t="inlineStr">
+        <is>
+          <t>unclassified</t>
+        </is>
+      </c>
+      <c r="V219" t="n">
+        <v>73.40000000000001</v>
+      </c>
+      <c r="W219" t="n">
+        <v>88.08</v>
+      </c>
+      <c r="X219" t="n">
+        <v>69.45099999999999</v>
+      </c>
+      <c r="Y219" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z219" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG219" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH219" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI219" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>1519</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>華城</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E220" t="n">
+        <v>78.06</v>
+      </c>
+      <c r="F220" t="n">
+        <v>52.28</v>
+      </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I220" t="b">
+        <v>0</v>
+      </c>
+      <c r="J220" t="n">
+        <v>10</v>
+      </c>
+      <c r="K220" t="n">
+        <v>847</v>
+      </c>
+      <c r="L220" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M220" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N220" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="O220" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="P220" t="n">
+        <v>737</v>
+      </c>
+      <c r="Q220" t="n">
+        <v>65.17</v>
+      </c>
+      <c r="R220" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="S220" t="n">
+        <v>7</v>
+      </c>
+      <c r="T220" t="inlineStr">
+        <is>
+          <t>BullTrend</t>
+        </is>
+      </c>
+      <c r="U220" t="inlineStr">
+        <is>
+          <t>industrial</t>
+        </is>
+      </c>
+      <c r="V220" t="n">
+        <v>770</v>
+      </c>
+      <c r="W220" t="n">
+        <v>924</v>
+      </c>
+      <c r="X220" t="n">
+        <v>716.1</v>
+      </c>
+      <c r="Y220" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z220" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG220" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH220" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI220" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>1605</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>華新</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E221" t="n">
+        <v>71.95</v>
+      </c>
+      <c r="F221" t="n">
+        <v>57.88</v>
+      </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H221" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I221" t="b">
+        <v>0</v>
+      </c>
+      <c r="J221" t="n">
+        <v>10</v>
+      </c>
+      <c r="K221" t="n">
+        <v>42.79</v>
+      </c>
+      <c r="L221" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M221" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N221" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="O221" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="P221" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="Q221" t="n">
+        <v>49.18</v>
+      </c>
+      <c r="R221" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S221" t="n">
+        <v>7</v>
+      </c>
+      <c r="T221" t="inlineStr">
+        <is>
+          <t>BullTrend</t>
+        </is>
+      </c>
+      <c r="U221" t="inlineStr">
+        <is>
+          <t>unclassified</t>
+        </is>
+      </c>
+      <c r="V221" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="W221" t="n">
+        <v>46.68</v>
+      </c>
+      <c r="X221" t="n">
+        <v>36.177</v>
+      </c>
+      <c r="Y221" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z221" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG221" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH221" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI221" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>2301</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>光寶科</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E222" t="n">
+        <v>79.09999999999999</v>
+      </c>
+      <c r="F222" t="n">
+        <v>47.95</v>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I222" t="b">
+        <v>0</v>
+      </c>
+      <c r="J222" t="n">
+        <v>10</v>
+      </c>
+      <c r="K222" t="n">
+        <v>331.1</v>
+      </c>
+      <c r="L222" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M222" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N222" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="O222" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P222" t="n">
+        <v>281.75</v>
+      </c>
+      <c r="Q222" t="n">
+        <v>69.66</v>
+      </c>
+      <c r="R222" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="S222" t="n">
+        <v>7</v>
+      </c>
+      <c r="T222" t="inlineStr">
+        <is>
+          <t>BullTrend</t>
+        </is>
+      </c>
+      <c r="U222" t="inlineStr">
+        <is>
+          <t>ai_hardware</t>
+        </is>
+      </c>
+      <c r="V222" t="n">
+        <v>301</v>
+      </c>
+      <c r="W222" t="n">
+        <v>361.2</v>
+      </c>
+      <c r="X222" t="n">
+        <v>279.93</v>
+      </c>
+      <c r="Y222" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z222" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG222" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH222" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI222" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>2324</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>仁寶</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E223" t="n">
+        <v>70.34</v>
+      </c>
+      <c r="F223" t="n">
+        <v>69.55</v>
+      </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I223" t="b">
+        <v>0</v>
+      </c>
+      <c r="J223" t="n">
+        <v>10.01</v>
+      </c>
+      <c r="K223" t="n">
+        <v>43.73</v>
+      </c>
+      <c r="L223" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M223" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="N223" t="n">
+        <v>8</v>
+      </c>
+      <c r="O223" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="P223" t="n">
+        <v>40.77</v>
+      </c>
+      <c r="Q223" t="n">
+        <v>43.66</v>
+      </c>
+      <c r="R223" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S223" t="n">
+        <v>5.1308</v>
+      </c>
+      <c r="T223" t="inlineStr">
+        <is>
+          <t>BullTrend</t>
+        </is>
+      </c>
+      <c r="U223" t="inlineStr">
+        <is>
+          <t>ai_hardware</t>
+        </is>
+      </c>
+      <c r="V223" t="n">
+        <v>39.75</v>
+      </c>
+      <c r="W223" t="n">
+        <v>47.7</v>
+      </c>
+      <c r="X223" t="n">
+        <v>37.7105</v>
+      </c>
+      <c r="Y223" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z223" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG223" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH223" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI223" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>2357</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>華碩</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E224" t="n">
+        <v>74.48999999999999</v>
+      </c>
+      <c r="F224" t="n">
+        <v>55.92</v>
+      </c>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H224" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I224" t="b">
+        <v>0</v>
+      </c>
+      <c r="J224" t="n">
+        <v>10</v>
+      </c>
+      <c r="K224" t="n">
+        <v>1064.8</v>
+      </c>
+      <c r="L224" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M224" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N224" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="O224" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="P224" t="n">
+        <v>928</v>
+      </c>
+      <c r="Q224" t="n">
+        <v>62.78</v>
+      </c>
+      <c r="R224" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="S224" t="n">
+        <v>7</v>
+      </c>
+      <c r="T224" t="inlineStr">
+        <is>
+          <t>BullTrend</t>
+        </is>
+      </c>
+      <c r="U224" t="inlineStr">
+        <is>
+          <t>ai_hardware</t>
+        </is>
+      </c>
+      <c r="V224" t="n">
+        <v>968</v>
+      </c>
+      <c r="W224" t="n">
+        <v>1161.6</v>
+      </c>
+      <c r="X224" t="n">
+        <v>900.24</v>
+      </c>
+      <c r="Y224" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z224" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG224" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH224" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI224" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>2368</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>金像電</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E225" t="n">
+        <v>70.28</v>
+      </c>
+      <c r="F225" t="n">
+        <v>56.91</v>
+      </c>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H225" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I225" t="b">
+        <v>0</v>
+      </c>
+      <c r="J225" t="n">
+        <v>10</v>
+      </c>
+      <c r="K225" t="n">
+        <v>1133</v>
+      </c>
+      <c r="L225" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M225" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N225" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="O225" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="P225" t="n">
+        <v>1012.5</v>
+      </c>
+      <c r="Q225" t="n">
+        <v>42.7</v>
+      </c>
+      <c r="R225" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S225" t="n">
+        <v>7</v>
+      </c>
+      <c r="T225" t="inlineStr">
+        <is>
+          <t>BullTrend</t>
+        </is>
+      </c>
+      <c r="U225" t="inlineStr">
+        <is>
+          <t>unclassified</t>
+        </is>
+      </c>
+      <c r="V225" t="n">
+        <v>1030</v>
+      </c>
+      <c r="W225" t="n">
+        <v>1236</v>
+      </c>
+      <c r="X225" t="n">
+        <v>957.9</v>
+      </c>
+      <c r="Y225" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z225" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG225" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH225" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI225" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>2395</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>研華</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E226" t="n">
+        <v>74.45</v>
+      </c>
+      <c r="F226" t="n">
+        <v>72.36</v>
+      </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="H226" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I226" t="b">
+        <v>0</v>
+      </c>
+      <c r="J226" t="n">
+        <v>10</v>
+      </c>
+      <c r="K226" t="n">
+        <v>742.5</v>
+      </c>
+      <c r="L226" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M226" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="N226" t="n">
+        <v>10</v>
+      </c>
+      <c r="O226" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="P226" t="n">
+        <v>676</v>
+      </c>
+      <c r="Q226" t="n">
+        <v>49.08</v>
+      </c>
+      <c r="R226" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S226" t="n">
+        <v>5.217</v>
+      </c>
+      <c r="T226" t="inlineStr">
+        <is>
+          <t>BullTrend</t>
+        </is>
+      </c>
+      <c r="U226" t="inlineStr">
+        <is>
+          <t>ai_hardware</t>
+        </is>
+      </c>
+      <c r="V226" t="n">
+        <v>675</v>
+      </c>
+      <c r="W226" t="n">
+        <v>810</v>
+      </c>
+      <c r="X226" t="n">
+        <v>639.785</v>
+      </c>
+      <c r="Y226" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z226" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG226" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH226" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI226" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>2408</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>南亞科</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E227" t="n">
+        <v>76.81999999999999</v>
+      </c>
+      <c r="F227" t="n">
+        <v>53.62</v>
+      </c>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H227" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I227" t="b">
+        <v>0</v>
+      </c>
+      <c r="J227" t="n">
+        <v>10</v>
+      </c>
+      <c r="K227" t="n">
+        <v>595.1</v>
+      </c>
+      <c r="L227" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M227" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N227" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="O227" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="P227" t="n">
+        <v>517.5</v>
+      </c>
+      <c r="Q227" t="n">
+        <v>60.82</v>
+      </c>
+      <c r="R227" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="S227" t="n">
+        <v>7</v>
+      </c>
+      <c r="T227" t="inlineStr">
+        <is>
+          <t>BullTrend</t>
+        </is>
+      </c>
+      <c r="U227" t="inlineStr">
+        <is>
+          <t>semiconductor</t>
+        </is>
+      </c>
+      <c r="V227" t="n">
+        <v>541</v>
+      </c>
+      <c r="W227" t="n">
+        <v>649.2</v>
+      </c>
+      <c r="X227" t="n">
+        <v>503.13</v>
+      </c>
+      <c r="Y227" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z227" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG227" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH227" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI227" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>2881</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>富邦金</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E228" t="n">
+        <v>74.90000000000001</v>
+      </c>
+      <c r="F228" t="n">
+        <v>37.36</v>
+      </c>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H228" t="inlineStr">
+        <is>
+          <t>Reject</t>
+        </is>
+      </c>
+      <c r="I228" t="b">
+        <v>0</v>
+      </c>
+      <c r="J228" t="n">
+        <v>6.36</v>
+      </c>
+      <c r="K228" t="n">
+        <v>150.5</v>
+      </c>
+      <c r="L228" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M228" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="N228" t="n">
+        <v>5</v>
+      </c>
+      <c r="O228" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="P228" t="n">
+        <v>133.5</v>
+      </c>
+      <c r="Q228" t="n">
+        <v>75.72</v>
+      </c>
+      <c r="R228" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="S228" t="n">
+        <v>7</v>
+      </c>
+      <c r="T228" t="inlineStr">
+        <is>
+          <t>BullTrend</t>
+        </is>
+      </c>
+      <c r="U228" t="inlineStr">
+        <is>
+          <t>finance</t>
+        </is>
+      </c>
+      <c r="V228" t="n">
+        <v>141.5</v>
+      </c>
+      <c r="W228" t="n">
+        <v>169.8</v>
+      </c>
+      <c r="X228" t="n">
+        <v>131.595</v>
+      </c>
+      <c r="Y228" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z228" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG228" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH228" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI228" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>3006</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>晶豪科</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E229" t="n">
+        <v>70.48999999999999</v>
+      </c>
+      <c r="F229" t="n">
+        <v>53.81</v>
+      </c>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H229" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I229" t="b">
+        <v>0</v>
+      </c>
+      <c r="J229" t="n">
+        <v>10</v>
+      </c>
+      <c r="K229" t="n">
+        <v>301.4</v>
+      </c>
+      <c r="L229" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M229" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N229" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="O229" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="P229" t="n">
+        <v>260.75</v>
+      </c>
+      <c r="Q229" t="n">
+        <v>48.7</v>
+      </c>
+      <c r="R229" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S229" t="n">
+        <v>7</v>
+      </c>
+      <c r="T229" t="inlineStr">
+        <is>
+          <t>BullTrend</t>
+        </is>
+      </c>
+      <c r="U229" t="inlineStr">
+        <is>
+          <t>unclassified</t>
+        </is>
+      </c>
+      <c r="V229" t="n">
+        <v>274</v>
+      </c>
+      <c r="W229" t="n">
+        <v>328.8</v>
+      </c>
+      <c r="X229" t="n">
+        <v>254.82</v>
+      </c>
+      <c r="Y229" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z229" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG229" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH229" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI229" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>3017</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>奇鋐</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E230" t="n">
+        <v>76.76000000000001</v>
+      </c>
+      <c r="F230" t="n">
+        <v>43.67</v>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H230" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I230" t="b">
+        <v>0</v>
+      </c>
+      <c r="J230" t="n">
+        <v>10</v>
+      </c>
+      <c r="K230" t="n">
+        <v>3674</v>
+      </c>
+      <c r="L230" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M230" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N230" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="O230" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P230" t="n">
+        <v>3089.38</v>
+      </c>
+      <c r="Q230" t="n">
+        <v>54.48</v>
+      </c>
+      <c r="R230" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S230" t="n">
+        <v>7</v>
+      </c>
+      <c r="T230" t="inlineStr">
+        <is>
+          <t>BullTrend</t>
+        </is>
+      </c>
+      <c r="U230" t="inlineStr">
+        <is>
+          <t>electronic_components</t>
+        </is>
+      </c>
+      <c r="V230" t="n">
+        <v>3340</v>
+      </c>
+      <c r="W230" t="n">
+        <v>4008</v>
+      </c>
+      <c r="X230" t="n">
+        <v>3106.2</v>
+      </c>
+      <c r="Y230" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z230" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG230" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH230" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI230" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>3037</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>欣興</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E231" t="n">
+        <v>79.27</v>
+      </c>
+      <c r="F231" t="n">
+        <v>51.66</v>
+      </c>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H231" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I231" t="b">
+        <v>0</v>
+      </c>
+      <c r="J231" t="n">
+        <v>10</v>
+      </c>
+      <c r="K231" t="n">
+        <v>1298</v>
+      </c>
+      <c r="L231" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M231" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N231" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="O231" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P231" t="n">
+        <v>1090.5</v>
+      </c>
+      <c r="Q231" t="n">
+        <v>61.09</v>
+      </c>
+      <c r="R231" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="S231" t="n">
+        <v>7</v>
+      </c>
+      <c r="T231" t="inlineStr">
+        <is>
+          <t>BullTrend</t>
+        </is>
+      </c>
+      <c r="U231" t="inlineStr">
+        <is>
+          <t>electronic_components</t>
+        </is>
+      </c>
+      <c r="V231" t="n">
+        <v>1180</v>
+      </c>
+      <c r="W231" t="n">
+        <v>1416</v>
+      </c>
+      <c r="X231" t="n">
+        <v>1097.4</v>
+      </c>
+      <c r="Y231" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z231" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG231" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH231" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI231" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>3081</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>聯亞</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E232" t="n">
+        <v>79.44</v>
+      </c>
+      <c r="F232" t="n">
+        <v>41.61</v>
+      </c>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H232" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I232" t="b">
+        <v>0</v>
+      </c>
+      <c r="J232" t="n">
+        <v>10</v>
+      </c>
+      <c r="K232" t="n">
+        <v>3707</v>
+      </c>
+      <c r="L232" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M232" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N232" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="O232" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P232" t="n">
+        <v>2990</v>
+      </c>
+      <c r="Q232" t="n">
+        <v>54.05</v>
+      </c>
+      <c r="R232" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S232" t="n">
+        <v>7</v>
+      </c>
+      <c r="T232" t="inlineStr">
+        <is>
+          <t>BullTrend</t>
+        </is>
+      </c>
+      <c r="U232" t="inlineStr">
+        <is>
+          <t>unclassified</t>
+        </is>
+      </c>
+      <c r="V232" t="n">
+        <v>3370</v>
+      </c>
+      <c r="W232" t="n">
+        <v>4044</v>
+      </c>
+      <c r="X232" t="n">
+        <v>3134.1</v>
+      </c>
+      <c r="Y232" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="AI232" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="AJ232" t="inlineStr">
+        <is>
+          <t>market_data_temporarily_unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>3189</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>景碩</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E233" t="n">
+        <v>74.14</v>
+      </c>
+      <c r="F233" t="n">
+        <v>47.95</v>
+      </c>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H233" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I233" t="b">
+        <v>0</v>
+      </c>
+      <c r="J233" t="n">
+        <v>10</v>
+      </c>
+      <c r="K233" t="n">
+        <v>1005.4</v>
+      </c>
+      <c r="L233" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M233" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N233" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="O233" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="P233" t="n">
+        <v>863</v>
+      </c>
+      <c r="Q233" t="n">
+        <v>49.68</v>
+      </c>
+      <c r="R233" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S233" t="n">
+        <v>7</v>
+      </c>
+      <c r="T233" t="inlineStr">
+        <is>
+          <t>BullTrend</t>
+        </is>
+      </c>
+      <c r="U233" t="inlineStr">
+        <is>
+          <t>unclassified</t>
+        </is>
+      </c>
+      <c r="V233" t="n">
+        <v>914</v>
+      </c>
+      <c r="W233" t="n">
+        <v>1096.8</v>
+      </c>
+      <c r="X233" t="n">
+        <v>850.02</v>
+      </c>
+      <c r="Y233" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z233" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG233" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH233" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI233" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>3324</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>雙鴻</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E234" t="n">
+        <v>76.39</v>
+      </c>
+      <c r="F234" t="n">
+        <v>38.1</v>
+      </c>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H234" t="inlineStr">
+        <is>
+          <t>Reject</t>
+        </is>
+      </c>
+      <c r="I234" t="b">
+        <v>0</v>
+      </c>
+      <c r="J234" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="K234" t="n">
+        <v>1105</v>
+      </c>
+      <c r="L234" t="inlineStr">
+        <is>
+          <t>gap_MM_Target_Up</t>
+        </is>
+      </c>
+      <c r="M234" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="N234" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="O234" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="P234" t="n">
+        <v>1037.5</v>
+      </c>
+      <c r="Q234" t="n">
+        <v>50.68</v>
+      </c>
+      <c r="R234" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S234" t="n">
+        <v>7</v>
+      </c>
+      <c r="T234" t="inlineStr">
+        <is>
+          <t>BullTrend</t>
+        </is>
+      </c>
+      <c r="U234" t="inlineStr">
+        <is>
+          <t>unclassified</t>
+        </is>
+      </c>
+      <c r="V234" t="n">
+        <v>1060</v>
+      </c>
+      <c r="W234" t="n">
+        <v>1272</v>
+      </c>
+      <c r="X234" t="n">
+        <v>985.8</v>
+      </c>
+      <c r="Y234" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="AI234" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="AJ234" t="inlineStr">
+        <is>
+          <t>market_data_temporarily_unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>3374</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>精材</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E235" t="n">
+        <v>75.38</v>
+      </c>
+      <c r="F235" t="n">
+        <v>42.65</v>
+      </c>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H235" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I235" t="b">
+        <v>0</v>
+      </c>
+      <c r="J235" t="n">
+        <v>10</v>
+      </c>
+      <c r="K235" t="n">
+        <v>386.1</v>
+      </c>
+      <c r="L235" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M235" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N235" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="O235" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P235" t="n">
+        <v>325.25</v>
+      </c>
+      <c r="Q235" t="n">
+        <v>60.99</v>
+      </c>
+      <c r="R235" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="S235" t="n">
+        <v>7</v>
+      </c>
+      <c r="T235" t="inlineStr">
+        <is>
+          <t>BullTrend</t>
+        </is>
+      </c>
+      <c r="U235" t="inlineStr">
+        <is>
+          <t>unclassified</t>
+        </is>
+      </c>
+      <c r="V235" t="n">
+        <v>351</v>
+      </c>
+      <c r="W235" t="n">
+        <v>421.2</v>
+      </c>
+      <c r="X235" t="n">
+        <v>326.43</v>
+      </c>
+      <c r="Y235" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="AI235" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="AJ235" t="inlineStr">
+        <is>
+          <t>market_data_temporarily_unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>3443</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>創意</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E236" t="n">
+        <v>78.63</v>
+      </c>
+      <c r="F236" t="n">
+        <v>49.57</v>
+      </c>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H236" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I236" t="b">
+        <v>0</v>
+      </c>
+      <c r="J236" t="n">
+        <v>10</v>
+      </c>
+      <c r="K236" t="n">
+        <v>6512</v>
+      </c>
+      <c r="L236" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M236" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N236" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="O236" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P236" t="n">
+        <v>5657.5</v>
+      </c>
+      <c r="Q236" t="n">
+        <v>60.47</v>
+      </c>
+      <c r="R236" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="S236" t="n">
+        <v>7</v>
+      </c>
+      <c r="T236" t="inlineStr">
+        <is>
+          <t>BullTrend</t>
+        </is>
+      </c>
+      <c r="U236" t="inlineStr">
+        <is>
+          <t>semiconductor</t>
+        </is>
+      </c>
+      <c r="V236" t="n">
+        <v>5920</v>
+      </c>
+      <c r="W236" t="n">
+        <v>7104</v>
+      </c>
+      <c r="X236" t="n">
+        <v>5505.6</v>
+      </c>
+      <c r="Y236" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z236" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG236" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH236" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI236" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>3532</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>台勝科</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E237" t="n">
+        <v>74.05</v>
+      </c>
+      <c r="F237" t="n">
+        <v>41.97</v>
+      </c>
+      <c r="G237" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H237" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I237" t="b">
+        <v>0</v>
+      </c>
+      <c r="J237" t="n">
+        <v>10</v>
+      </c>
+      <c r="K237" t="n">
+        <v>433.4</v>
+      </c>
+      <c r="L237" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M237" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N237" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="O237" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P237" t="n">
+        <v>344.5</v>
+      </c>
+      <c r="Q237" t="n">
+        <v>56.45</v>
+      </c>
+      <c r="R237" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S237" t="n">
+        <v>7</v>
+      </c>
+      <c r="T237" t="inlineStr">
+        <is>
+          <t>BullTrend</t>
+        </is>
+      </c>
+      <c r="U237" t="inlineStr">
+        <is>
+          <t>unclassified</t>
+        </is>
+      </c>
+      <c r="V237" t="n">
+        <v>394</v>
+      </c>
+      <c r="W237" t="n">
+        <v>472.8</v>
+      </c>
+      <c r="X237" t="n">
+        <v>366.42</v>
+      </c>
+      <c r="Y237" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z237" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG237" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH237" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI237" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>3583</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>辛耘</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E238" t="n">
+        <v>76.3</v>
+      </c>
+      <c r="F238" t="n">
+        <v>55.72</v>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H238" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I238" t="b">
+        <v>0</v>
+      </c>
+      <c r="J238" t="n">
+        <v>10</v>
+      </c>
+      <c r="K238" t="n">
+        <v>836</v>
+      </c>
+      <c r="L238" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M238" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N238" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="O238" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="P238" t="n">
+        <v>714.5</v>
+      </c>
+      <c r="Q238" t="n">
+        <v>61.44</v>
+      </c>
+      <c r="R238" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="S238" t="n">
+        <v>7</v>
+      </c>
+      <c r="T238" t="inlineStr">
+        <is>
+          <t>BullTrend</t>
+        </is>
+      </c>
+      <c r="U238" t="inlineStr">
+        <is>
+          <t>unclassified</t>
+        </is>
+      </c>
+      <c r="V238" t="n">
+        <v>760</v>
+      </c>
+      <c r="W238" t="n">
+        <v>912</v>
+      </c>
+      <c r="X238" t="n">
+        <v>706.8</v>
+      </c>
+      <c r="Y238" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z238" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG238" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH238" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI238" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>6446</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>藥華藥</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E239" t="n">
+        <v>73.2</v>
+      </c>
+      <c r="F239" t="n">
+        <v>44.17</v>
+      </c>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H239" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I239" t="b">
+        <v>0</v>
+      </c>
+      <c r="J239" t="n">
+        <v>10</v>
+      </c>
+      <c r="K239" t="n">
+        <v>1716</v>
+      </c>
+      <c r="L239" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M239" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N239" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="O239" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P239" t="n">
+        <v>1492.5</v>
+      </c>
+      <c r="Q239" t="n">
+        <v>57.77</v>
+      </c>
+      <c r="R239" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S239" t="n">
+        <v>7</v>
+      </c>
+      <c r="T239" t="inlineStr">
+        <is>
+          <t>BullTrend</t>
+        </is>
+      </c>
+      <c r="U239" t="inlineStr">
+        <is>
+          <t>unclassified</t>
+        </is>
+      </c>
+      <c r="V239" t="n">
+        <v>1560</v>
+      </c>
+      <c r="W239" t="n">
+        <v>1872</v>
+      </c>
+      <c r="X239" t="n">
+        <v>1450.8</v>
+      </c>
+      <c r="Y239" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z239" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG239" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH239" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI239" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>6472</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>保瑞</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E240" t="n">
+        <v>70.09999999999999</v>
+      </c>
+      <c r="F240" t="n">
+        <v>53.41</v>
+      </c>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H240" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I240" t="b">
+        <v>0</v>
+      </c>
+      <c r="J240" t="n">
+        <v>10</v>
+      </c>
+      <c r="K240" t="n">
+        <v>483.45</v>
+      </c>
+      <c r="L240" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M240" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N240" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="O240" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="P240" t="n">
+        <v>438</v>
+      </c>
+      <c r="Q240" t="n">
+        <v>46.05</v>
+      </c>
+      <c r="R240" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S240" t="n">
+        <v>7</v>
+      </c>
+      <c r="T240" t="inlineStr">
+        <is>
+          <t>BullTrend</t>
+        </is>
+      </c>
+      <c r="U240" t="inlineStr">
+        <is>
+          <t>unclassified</t>
+        </is>
+      </c>
+      <c r="V240" t="n">
+        <v>439.5</v>
+      </c>
+      <c r="W240" t="n">
+        <v>527.4</v>
+      </c>
+      <c r="X240" t="n">
+        <v>408.735</v>
+      </c>
+      <c r="Y240" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z240" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG240" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH240" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI240" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>6669</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>緯穎</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E241" t="n">
+        <v>81.37</v>
+      </c>
+      <c r="F241" t="n">
+        <v>57.47</v>
+      </c>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H241" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I241" t="b">
+        <v>0</v>
+      </c>
+      <c r="J241" t="n">
+        <v>10</v>
+      </c>
+      <c r="K241" t="n">
+        <v>7496.5</v>
+      </c>
+      <c r="L241" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M241" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N241" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="O241" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="P241" t="n">
+        <v>6430</v>
+      </c>
+      <c r="Q241" t="n">
+        <v>73.11</v>
+      </c>
+      <c r="R241" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="S241" t="n">
+        <v>7</v>
+      </c>
+      <c r="T241" t="inlineStr">
+        <is>
+          <t>BullTrend</t>
+        </is>
+      </c>
+      <c r="U241" t="inlineStr">
+        <is>
+          <t>semiconductor</t>
+        </is>
+      </c>
+      <c r="V241" t="n">
+        <v>6815</v>
+      </c>
+      <c r="W241" t="n">
+        <v>8178</v>
+      </c>
+      <c r="X241" t="n">
+        <v>6337.95</v>
+      </c>
+      <c r="Y241" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z241" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG241" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH241" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI241" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>9921</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>巨大</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>swing_accumulation_ready</t>
+        </is>
+      </c>
+      <c r="E242" t="n">
+        <v>75.66</v>
+      </c>
+      <c r="F242" t="n">
+        <v>55.75</v>
+      </c>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H242" t="inlineStr">
+        <is>
+          <t>WaitPullback</t>
+        </is>
+      </c>
+      <c r="I242" t="b">
+        <v>0</v>
+      </c>
+      <c r="J242" t="n">
+        <v>10</v>
+      </c>
+      <c r="K242" t="n">
+        <v>115.5</v>
+      </c>
+      <c r="L242" t="inlineStr">
+        <is>
+          <t>measured_move_target_up</t>
+        </is>
+      </c>
+      <c r="M242" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="N242" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="O242" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="P242" t="n">
+        <v>102.53</v>
+      </c>
+      <c r="Q242" t="n">
+        <v>48.32</v>
+      </c>
+      <c r="R242" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="S242" t="n">
+        <v>7</v>
+      </c>
+      <c r="T242" t="inlineStr">
+        <is>
+          <t>BullTrend</t>
+        </is>
+      </c>
+      <c r="U242" t="inlineStr">
+        <is>
+          <t>unclassified</t>
+        </is>
+      </c>
+      <c r="V242" t="n">
+        <v>105</v>
+      </c>
+      <c r="W242" t="n">
+        <v>126</v>
+      </c>
+      <c r="X242" t="n">
+        <v>97.65000000000001</v>
+      </c>
+      <c r="Y242" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="Z242" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG242" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH242" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI242" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AJ217"/>
+  <autoFilter ref="A1:AJ242"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -20090,7 +23055,7 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>2026-08-26 14:24:03</t>
+          <t>2026-08-27 14:24:27</t>
         </is>
       </c>
     </row>
@@ -20137,7 +23102,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>216</v>
+        <v>241</v>
       </c>
     </row>
     <row r="7">
@@ -20157,7 +23122,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>216</v>
+        <v>241</v>
       </c>
     </row>
     <row r="9">

</xml_diff>